<commit_message>
Ajoute une vraie présentation aux courriels froids
Gabriel: « Aucune présentation, mise en contexte. » Le courriel demandait à un
inconnu de s'intéresser à une entreprise dont il n'a jamais entendu parler et à
une matière qu'il ne connaît pas.

Chaque courriel froid commence maintenant par qui est Gabriel, ce qu'est
Lasclay, et ce qu'est l'asclépiade sous le nom de « petits cochons », que tout
le monde reconnaît au Québec. Puis une phrase qui dit explicitement pourquoi je
lui écris à lui: sa région quand l'asclépiade y a une histoire réelle, son sujet
sinon.

Retire aussi une accroche régionale qui n'en était pas une: « notre atelier est
dans Limoilou » ne dit rien à un journal de Charlevoix. Les quatre contacts de
la liste chaude sans historique documenté reçoivent la même présentation.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015pjLsGPzf1MX1JC7QiKGGk
</commit_message>
<xml_diff>
--- a/communique-dragons/Lasclay_v2.xlsx
+++ b/communique-dragons/Lasclay_v2.xlsx
@@ -3080,7 +3080,7 @@
       <c r="N29" s="46" t="inlineStr">
         <is>
           <t>Bonjour Mme Roberge,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou. On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -3144,7 +3144,7 @@
       <c r="N30" s="46" t="inlineStr">
         <is>
           <t>Bonjour Mme Laforest,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile. L'asclépiade est la seule plante que les chenilles du monarque peuvent manger, et la soie attachée à ses graines est un isolant creux, très léger et naturellement hydrophobe.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou. On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -3412,7 +3412,7 @@
       <c r="N34" s="46" t="inlineStr">
         <is>
           <t>Bonjour Mme Goubau,
-Vous couvrez le textile et la mode, alors voici une matière que peu de gens ont vue de près. La soie d'asclépiade est une fibre creuse et hydrophobe attachée aux graines d'une plante que les agriculteurs arrachent depuis 50 ans. On en fait de l'isolant pour des manteaux, des mitaines et des tuques.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou. Vous couvrez le textile et la mode, alors voici une matière que peu de gens ont vue de près : la soie d'asclépiade, une fibre creuse et naturellement hydrophobe attachée aux graines d'une plante que les agriculteurs arrachent de leurs champs depuis 50 ans. On la transforme en isolant, et on en fait des manteaux, des mitaines et des tuques.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -3476,7 +3476,7 @@
       <c r="N35" s="46" t="inlineStr">
         <is>
           <t>Bonjour Mme Dostie,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile. La fibre est attachée aux graines de la plante : elle est creuse, très légère et naturellement hydrophobe.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou. On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -3995,12 +3995,13 @@
       <c r="S3" s="46" t="inlineStr">
         <is>
           <t>Bonjour Zoé Allemand,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade est une vivace indigène qui pousse avec peu d'intrants, ce qui en fait une culture intéressante pour des régions où les grandes cultures rendent mal.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -4080,12 +4081,13 @@
       <c r="S4" s="46" t="inlineStr">
         <is>
           <t>Bonjour Victoria Bakos,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade est la plante que les agriculteurs arrachent depuis 50 ans. La soie attachée à ses graines est ce qui isole nos manteaux, nos mitaines et nos tuques.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. J'ai du matériel photo qui montre bien le contraste : la gousse dans le champ, la soie dans la main, le produit porté. L'atelier de Limoilou est ouvert si vous voulez voir la matière.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière, et j'ai du matériel photo.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -4164,9 +4166,10 @@
       <c r="S5" s="46" t="inlineStr">
         <is>
           <t>Bonjour Marie-Émélie Bernier,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-Notre atelier est dans Limoilou, et c'est là que la soie d'asclépiade devient de l'isolant.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
@@ -4253,12 +4256,13 @@
       <c r="S6" s="46" t="inlineStr">
         <is>
           <t>Bonjour Normand Blouin,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-Huit ans après l'effondrement de la première filière québécoise de l'asclépiade, on achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes à Québec.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -4338,9 +4342,10 @@
       <c r="S7" s="46" t="inlineStr">
         <is>
           <t>Bonjour Louise Bourbonnais,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-Notre atelier est dans Limoilou, et c'est là que la soie d'asclépiade devient de l'isolant.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
@@ -4423,12 +4428,13 @@
       <c r="S8" s="46" t="inlineStr">
         <is>
           <t>Bonjour Francois Bourque,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-Notre atelier est dans Limoilou, et c'est là que la soie d'asclépiade devient de l'isolant.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a pas de chaîne d'approvisionnement.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -4512,12 +4518,13 @@
       <c r="S9" s="46" t="inlineStr">
         <is>
           <t>Bonjour Ariane Boyer,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade est une vivace indigène qui pousse avec peu d'intrants, ce qui en fait une culture intéressante pour des régions où les grandes cultures rendent mal.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de la campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -4596,9 +4603,10 @@
       <c r="S10" s="46" t="inlineStr">
         <is>
           <t>Bonjour Gilbert Bégin,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-Notre atelier est dans Limoilou, et c'est là que la soie d'asclépiade devient de l'isolant.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
@@ -4685,9 +4693,10 @@
       <c r="S11" s="46" t="inlineStr">
         <is>
           <t>Bonjour Papa Moussa Camara,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-Notre atelier est dans Limoilou, et c'est là que la soie d'asclépiade devient de l'isolant.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
@@ -4769,9 +4778,10 @@
       <c r="S12" s="46" t="inlineStr">
         <is>
           <t>Bonjour Victor Carré,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-Notre atelier est dans Limoilou, et c'est là que la soie d'asclépiade devient de l'isolant.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
@@ -4854,12 +4864,13 @@
       <c r="S13" s="46" t="inlineStr">
         <is>
           <t>Bonjour Eric Chabot,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-La soie d'asclépiade est une fibre creuse et naturellement hydrophobe attachée aux graines de la plante. On en fait l'isolant de nos manteaux, de nos mitaines et de nos sacs isothermes.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez le plein air. À poids égal, la littérature donne la soie d'asclépiade pour environ 10 % plus isolante que le duvet. C'est un repère de laboratoire, pas une promesse de manteau, et c'est exactement pour ça que je préfère qu'on la teste.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester la fibre plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -4939,9 +4950,10 @@
       <c r="S14" s="46" t="inlineStr">
         <is>
           <t>Bonjour Tristan Champagne-Lessard,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-La Montérégie est une des régions où l'asclépiade se cultive encore, et c'est de champs comme ceux-là que vient la fibre qu'on transforme.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
@@ -5028,12 +5040,13 @@
       <c r="S15" s="46" t="inlineStr">
         <is>
           <t>Bonjour Jean-Marc Chevalier,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-La Montérégie est une des régions où l'asclépiade se cultive encore, et c'est de champs comme ceux-là que vient la fibre qu'on transforme.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -5117,12 +5130,13 @@
       <c r="S16" s="46" t="inlineStr">
         <is>
           <t>Bonjour Simon Chrétien,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-Notre atelier est dans Limoilou, et c'est là que la soie d'asclépiade devient de l'isolant.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -5197,9 +5211,10 @@
       <c r="S17" s="46" t="inlineStr">
         <is>
           <t>Bonjour Maxime Corneau,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-Un de nos fournisseurs d'asclépiade cultive au Lac-Saint-Jean depuis nos tout débuts, et il l'est encore aujourd'hui. La fibre de chez vous se retrouve dans nos produits.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris entre autres parce qu'un de nos fournisseurs d'asclépiade cultive au Lac-Saint-Jean depuis nos tout débuts, et qu'il l'est encore aujourd'hui. La fibre de chez vous se retrouve dans nos produits.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
@@ -5282,12 +5297,13 @@
       <c r="S18" s="46" t="inlineStr">
         <is>
           <t>Bonjour Aurélia Crémoux,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-La soie d'asclépiade est une fibre creuse et naturellement hydrophobe attachée aux graines de la plante. On en fait l'isolant de nos manteaux, de nos mitaines et de nos sacs isothermes.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez le plein air. À poids égal, la littérature donne la soie d'asclépiade pour environ 10 % plus isolante que le duvet. C'est un repère de laboratoire, pas une promesse de manteau, et c'est exactement pour ça que je préfère qu'on la teste.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester la fibre plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -5367,12 +5383,13 @@
       <c r="S19" s="46" t="inlineStr">
         <is>
           <t>Bonjour Catherine Dallaire,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'Estrie compte encore des producteurs d'asclépiade, et une des premières usines de transformation de la fibre était à Granby.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris entre autres parce qu'une des premières usines de transformation de la fibre était à Granby, et que l'Estrie compte encore des producteurs d'asclépiade.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -5535,12 +5552,13 @@
       <c r="S21" s="46" t="inlineStr">
         <is>
           <t>Bonjour Anaïs Desjardins,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade est la seule plante que les chenilles du monarque peuvent manger, et le déclin du papillon suit celui de la plante dans les zones agricoles. Notre pari est simple : si l'asclépiade devient payante, les agriculteurs la gardent.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de la campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -5624,12 +5642,13 @@
       <c r="S22" s="46" t="inlineStr">
         <is>
           <t>Bonjour Simon Dominé,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-Huit ans après l'effondrement de la première filière québécoise de l'asclépiade, on achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes à Québec.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -5708,8 +5727,10 @@
       <c r="S23" s="46" t="inlineStr">
         <is>
           <t>Bonjour Karl-Ivann Dubé,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
@@ -5791,8 +5812,10 @@
       <c r="S24" s="46" t="inlineStr">
         <is>
           <t>Bonjour André Fauteux,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
@@ -5874,12 +5897,13 @@
       <c r="S25" s="46" t="inlineStr">
         <is>
           <t>Bonjour Myriam Fimbry,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-Huit ans après l'effondrement de la première filière québécoise de l'asclépiade, on achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes à Québec.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -5954,8 +5978,10 @@
       <c r="S26" s="46" t="inlineStr">
         <is>
           <t>Bonjour Étienne Fortin-Gauthier,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
@@ -6037,9 +6063,10 @@
       <c r="S27" s="46" t="inlineStr">
         <is>
           <t>Bonjour Johanne Fournier,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade est une vivace indigène qui pousse avec peu d'intrants, ce qui en fait une culture intéressante pour des régions où les grandes cultures rendent mal.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
@@ -6126,12 +6153,13 @@
       <c r="S28" s="46" t="inlineStr">
         <is>
           <t>Bonjour Jean Garon,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade est la seule plante que les chenilles du monarque peuvent manger, et le déclin du papillon suit celui de la plante dans les zones agricoles. Notre pari est simple : si l'asclépiade devient payante, les agriculteurs la gardent.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de la campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -6211,8 +6239,10 @@
       <c r="S29" s="46" t="inlineStr">
         <is>
           <t>Bonjour Cécile Gladel,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
@@ -6299,12 +6329,13 @@
       <c r="S30" s="46" t="inlineStr">
         <is>
           <t>Bonjour Marieke Glorieux-Stryckman,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-La soie d'asclépiade est une fibre creuse et naturellement hydrophobe attachée aux graines de la plante. On en fait l'isolant de nos manteaux, de nos mitaines et de nos sacs isothermes.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez le plein air. À poids égal, la littérature donne la soie d'asclépiade pour environ 10 % plus isolante que le duvet. C'est un repère de laboratoire, pas une promesse de manteau, et c'est exactement pour ça que je préfère qu'on la teste.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester la fibre plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -6388,12 +6419,13 @@
       <c r="S31" s="46" t="inlineStr">
         <is>
           <t>Bonjour Maude Goyer,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-La soie d'asclépiade est une fibre creuse et naturellement hydrophobe attachée aux graines de la plante. On en fait l'isolant de nos manteaux, de nos mitaines et de nos sacs isothermes.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez le plein air. À poids égal, la littérature donne la soie d'asclépiade pour environ 10 % plus isolante que le duvet. C'est un repère de laboratoire, pas une promesse de manteau, et c'est exactement pour ça que je préfère qu'on la teste.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester la fibre plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -6472,12 +6504,13 @@
       <c r="S32" s="46" t="inlineStr">
         <is>
           <t>Bonjour Pauline Gravel,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-Huit ans après l'effondrement de la première filière québécoise de l'asclépiade, on achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes à Québec.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -6556,9 +6589,10 @@
       <c r="S33" s="46" t="inlineStr">
         <is>
           <t>Bonjour Bernard Hervieux,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-Notre atelier est dans Limoilou, et c'est là que la soie d'asclépiade devient de l'isolant.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
@@ -6645,12 +6679,13 @@
       <c r="S34" s="46" t="inlineStr">
         <is>
           <t>Bonjour Leïla Jolin-Dahel,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-Huit ans après l'effondrement de la première filière québécoise de l'asclépiade, on achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes à Québec.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -6734,12 +6769,13 @@
       <c r="S35" s="46" t="inlineStr">
         <is>
           <t>Bonjour Kodjo Edjinam Nulagnon LOGO,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade est une vivace indigène qui pousse avec peu d'intrants, ce qui en fait une culture intéressante pour des régions où les grandes cultures rendent mal.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de la campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -6814,12 +6850,13 @@
       <c r="S36" s="46" t="inlineStr">
         <is>
           <t>Bonjour Annie Labrecque,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-Huit ans après l'effondrement de la première filière québécoise de l'asclépiade, on achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes à Québec.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -6894,9 +6931,10 @@
       <c r="S37" s="46" t="inlineStr">
         <is>
           <t>Bonjour Marianne Lachapelle,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'Estrie compte encore des producteurs d'asclépiade, et une des premières usines de transformation de la fibre était à Granby.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris entre autres parce qu'une des premières usines de transformation de la fibre était à Granby, et que l'Estrie compte encore des producteurs d'asclépiade.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
@@ -6983,12 +7021,13 @@
       <c r="S38" s="46" t="inlineStr">
         <is>
           <t>Bonjour Sophie Lachapelle,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-Huit ans après l'effondrement de la première filière québécoise de l'asclépiade, on achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes à Québec.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -7063,9 +7102,10 @@
       <c r="S39" s="46" t="inlineStr">
         <is>
           <t>Bonjour Alain Laforest,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-Notre atelier est dans Limoilou, et c'est là que la soie d'asclépiade devient de l'isolant.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
@@ -7143,9 +7183,10 @@
       <c r="S40" s="46" t="inlineStr">
         <is>
           <t>Bonjour Mikaël Lalancette,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-Notre atelier est dans Limoilou, et c'est là que la soie d'asclépiade devient de l'isolant.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
@@ -7227,12 +7268,13 @@
       <c r="S41" s="46" t="inlineStr">
         <is>
           <t>Bonjour Jean-Luc Lavallée,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-Notre atelier est dans Limoilou, et c'est là que la soie d'asclépiade devient de l'isolant.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a pas de chaîne d'approvisionnement.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -7316,12 +7358,13 @@
       <c r="S42" s="46" t="inlineStr">
         <is>
           <t>Bonjour Jean-Francois Leblanc,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-La soie d'asclépiade est une fibre creuse et naturellement hydrophobe attachée aux graines de la plante. On en fait l'isolant de nos manteaux, de nos mitaines et de nos sacs isothermes.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez le plein air. À poids égal, la littérature donne la soie d'asclépiade pour environ 10 % plus isolante que le duvet. C'est un repère de laboratoire, pas une promesse de manteau, et c'est exactement pour ça que je préfère qu'on la teste.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester la fibre plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -7396,12 +7439,13 @@
       <c r="S43" s="46" t="inlineStr">
         <is>
           <t>Bonjour Julie Leduc,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-La soie d'asclépiade est une fibre creuse et naturellement hydrophobe attachée aux graines de la plante. On en fait l'isolant de nos manteaux, de nos mitaines et de nos sacs isothermes.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez le plein air. À poids égal, la littérature donne la soie d'asclépiade pour environ 10 % plus isolante que le duvet. C'est un repère de laboratoire, pas une promesse de manteau, et c'est exactement pour ça que je préfère qu'on la teste.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester la fibre plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -7485,12 +7529,13 @@
       <c r="S44" s="46" t="inlineStr">
         <is>
           <t>Bonjour Annie Martin,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-Huit ans après l'effondrement de la première filière québécoise de l'asclépiade, on achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes à Québec.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -7659,12 +7704,13 @@
       <c r="S46" s="46" t="inlineStr">
         <is>
           <t>Bonjour Charles Mathieu,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade est la seule plante que les chenilles du monarque peuvent manger, et le déclin du papillon suit celui de la plante dans les zones agricoles. Notre pari est simple : si l'asclépiade devient payante, les agriculteurs la gardent.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de la campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -7744,12 +7790,13 @@
       <c r="S47" s="46" t="inlineStr">
         <is>
           <t>Bonjour Clara Matthey-Jonais,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-Huit ans après l'effondrement de la première filière québécoise de l'asclépiade, on achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes à Québec.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -7828,12 +7875,13 @@
       <c r="S48" s="46" t="inlineStr">
         <is>
           <t>Bonjour Valérian Mazataud,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-Huit ans après l'effondrement de la première filière québécoise de l'asclépiade, on achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes à Québec.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -7912,8 +7960,10 @@
       <c r="S49" s="46" t="inlineStr">
         <is>
           <t>Bonjour Lili Mercure,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
@@ -8000,12 +8050,13 @@
       <c r="S50" s="46" t="inlineStr">
         <is>
           <t>Bonjour Nicolas Mesly,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-Huit ans après l'effondrement de la première filière québécoise de l'asclépiade, on achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes à Québec.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -8089,12 +8140,13 @@
       <c r="S51" s="46" t="inlineStr">
         <is>
           <t>Bonjour Nicolas Michaud,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-Huit ans après l'effondrement de la première filière québécoise de l'asclépiade, on achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes à Québec.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -8173,12 +8225,13 @@
       <c r="S52" s="46" t="inlineStr">
         <is>
           <t>Bonjour Véronique Morin,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-Notre atelier est dans Limoilou, et c'est là que la soie d'asclépiade devient de l'isolant.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -8257,8 +8310,10 @@
       <c r="S53" s="46" t="inlineStr">
         <is>
           <t>Bonjour Lila Mouch,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
@@ -8336,9 +8391,10 @@
       <c r="S54" s="46" t="inlineStr">
         <is>
           <t>Bonjour Olivier Mougeot,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-Notre atelier est dans Limoilou, et c'est là que la soie d'asclépiade devient de l'isolant.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
@@ -8425,12 +8481,13 @@
       <c r="S55" s="46" t="inlineStr">
         <is>
           <t>Bonjour Emmanuelle Mozayan-Verschaeve,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-La soie d'asclépiade est une fibre creuse et naturellement hydrophobe attachée aux graines de la plante. On en fait l'isolant de nos manteaux, de nos mitaines et de nos sacs isothermes.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez le plein air. À poids égal, la littérature donne la soie d'asclépiade pour environ 10 % plus isolante que le duvet. C'est un repère de laboratoire, pas une promesse de manteau, et c'est exactement pour ça que je préfère qu'on la teste.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester la fibre plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -8509,12 +8566,13 @@
       <c r="S56" s="46" t="inlineStr">
         <is>
           <t>Bonjour Jean-Benoît Nadeau,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-La soie d'asclépiade est une fibre creuse et naturellement hydrophobe attachée aux graines de la plante. On en fait l'isolant de nos manteaux, de nos mitaines et de nos sacs isothermes.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez le plein air. À poids égal, la littérature donne la soie d'asclépiade pour environ 10 % plus isolante que le duvet. C'est un repère de laboratoire, pas une promesse de manteau, et c'est exactement pour ça que je préfère qu'on la teste.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester la fibre plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -8598,12 +8656,13 @@
       <c r="S57" s="46" t="inlineStr">
         <is>
           <t>Bonjour Yves Ouellet,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-Notre atelier est dans Limoilou, et c'est là que la soie d'asclépiade devient de l'isolant.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez le plein air. À poids égal, la littérature donne la soie d'asclépiade pour environ 10 % plus isolante que le duvet. C'est un repère de laboratoire, pas une promesse de manteau, et c'est exactement pour ça que je préfère qu'on la teste.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester la fibre plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -8687,12 +8746,13 @@
       <c r="S58" s="46" t="inlineStr">
         <is>
           <t>Bonjour Josée Panet-Raymond,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-Huit ans après l'effondrement de la première filière québécoise de l'asclépiade, on achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes à Québec.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -8772,12 +8832,13 @@
       <c r="S59" s="46" t="inlineStr">
         <is>
           <t>Bonjour Yannick Patelli,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-Notre atelier est dans Limoilou, et c'est là que la soie d'asclépiade devient de l'isolant.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -8861,12 +8922,13 @@
       <c r="S60" s="46" t="inlineStr">
         <is>
           <t>Bonjour Félix Pedneault,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade est la seule plante que les chenilles du monarque peuvent manger, et le déclin du papillon suit celui de la plante dans les zones agricoles. Notre pari est simple : si l'asclépiade devient payante, les agriculteurs la gardent.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de la campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -8950,12 +9012,13 @@
       <c r="S61" s="46" t="inlineStr">
         <is>
           <t>Bonjour Marie-Eve Poulin,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade est une vivace indigène qui pousse avec peu d'intrants, ce qui en fait une culture intéressante pour des régions où les grandes cultures rendent mal.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez le plein air. À poids égal, la littérature donne la soie d'asclépiade pour environ 10 % plus isolante que le duvet. C'est un repère de laboratoire, pas une promesse de manteau, et c'est exactement pour ça que je préfère qu'on la teste.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester la fibre plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -9034,12 +9097,13 @@
       <c r="S62" s="46" t="inlineStr">
         <is>
           <t>Bonjour Marie-Hélène Proulx,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-Huit ans après l'effondrement de la première filière québécoise de l'asclépiade, on achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes à Québec.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -9118,8 +9182,10 @@
       <c r="S63" s="46" t="inlineStr">
         <is>
           <t>Bonjour Jean-Hugues Roy,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
@@ -9201,9 +9267,10 @@
       <c r="S64" s="46" t="inlineStr">
         <is>
           <t>Bonjour Martin Roy,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-Notre atelier est dans Limoilou, et c'est là que la soie d'asclépiade devient de l'isolant.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
@@ -9285,12 +9352,13 @@
       <c r="S65" s="46" t="inlineStr">
         <is>
           <t>Bonjour Sylvain Sarrazin,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-La soie d'asclépiade est une fibre creuse et naturellement hydrophobe attachée aux graines de la plante. On en fait l'isolant de nos manteaux, de nos mitaines et de nos sacs isothermes.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez le plein air. À poids égal, la littérature donne la soie d'asclépiade pour environ 10 % plus isolante que le duvet. C'est un repère de laboratoire, pas une promesse de manteau, et c'est exactement pour ça que je préfère qu'on la teste.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester la fibre plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -9374,12 +9442,13 @@
       <c r="S66" s="46" t="inlineStr">
         <is>
           <t>Bonjour Pierre Sormany,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-La soie d'asclépiade est une fibre creuse et naturellement hydrophobe attachée aux graines de la plante. On en fait l'isolant de nos manteaux, de nos mitaines et de nos sacs isothermes.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez le plein air. À poids égal, la littérature donne la soie d'asclépiade pour environ 10 % plus isolante que le duvet. C'est un repère de laboratoire, pas une promesse de manteau, et c'est exactement pour ça que je préfère qu'on la teste.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester la fibre plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -9463,12 +9532,13 @@
       <c r="S67" s="46" t="inlineStr">
         <is>
           <t>Bonjour Scott Stevenson,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'Estrie compte encore des producteurs d'asclépiade, et une des premières usines de transformation de la fibre était à Granby.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris entre autres parce qu'une des premières usines de transformation de la fibre était à Granby, et que l'Estrie compte encore des producteurs d'asclépiade.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -9552,12 +9622,13 @@
       <c r="S68" s="46" t="inlineStr">
         <is>
           <t>Bonjour Michèle Tanganika,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-Huit ans après l'effondrement de la première filière québécoise de l'asclépiade, on achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes à Québec.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -9641,8 +9712,10 @@
       <c r="S69" s="46" t="inlineStr">
         <is>
           <t>Bonjour Stephane Tellier,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
@@ -9724,9 +9797,10 @@
       <c r="S70" s="46" t="inlineStr">
         <is>
           <t>Bonjour Karine Tremblay,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'Estrie compte encore des producteurs d'asclépiade, et une des premières usines de transformation de la fibre était à Granby.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris entre autres parce qu'une des premières usines de transformation de la fibre était à Granby, et que l'Estrie compte encore des producteurs d'asclépiade.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
@@ -9809,12 +9883,13 @@
       <c r="S71" s="46" t="inlineStr">
         <is>
           <t>Bonjour Jean-Francois Venne,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade est la seule plante que les chenilles du monarque peuvent manger, et le déclin du papillon suit celui de la plante dans les zones agricoles. Notre pari est simple : si l'asclépiade devient payante, les agriculteurs la gardent.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de la campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -9898,12 +9973,13 @@
       <c r="S72" s="46" t="inlineStr">
         <is>
           <t>Bonjour Shahram Yazdanpanah,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-La soie d'asclépiade est une fibre creuse et naturellement hydrophobe attachée aux graines de la plante. On en fait l'isolant de nos manteaux, de nos mitaines et de nos sacs isothermes.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez le plein air. À poids égal, la littérature donne la soie d'asclépiade pour environ 10 % plus isolante que le duvet. C'est un repère de laboratoire, pas une promesse de manteau, et c'est exactement pour ça que je préfère qu'on la teste.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester la fibre plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -9983,12 +10059,13 @@
       <c r="S73" s="46" t="inlineStr">
         <is>
           <t>Bonjour Malika Alaoui,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade est la plante que les agriculteurs arrachent depuis 50 ans. La soie attachée à ses graines est ce qui isole nos manteaux, nos mitaines et nos tuques.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. J'ai du matériel photo qui montre bien le contraste : la gousse dans le champ, la soie dans la main, le produit porté. L'atelier de Limoilou est ouvert si vous voulez voir la matière.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière, et j'ai du matériel photo.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -10067,12 +10144,13 @@
       <c r="S74" s="46" t="inlineStr">
         <is>
           <t>Bonjour Yahia Arkat,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade est la seule plante que les chenilles du monarque peuvent manger, et le déclin du papillon suit celui de la plante dans les zones agricoles. Notre pari est simple : si l'asclépiade devient payante, les agriculteurs la gardent.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de la campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -10156,12 +10234,13 @@
       <c r="S75" s="46" t="inlineStr">
         <is>
           <t>Bonjour MARC-OLIVIER BISSON,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-Huit ans après l'effondrement de la première filière québécoise de l'asclépiade, on achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes à Québec.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -10241,12 +10320,13 @@
       <c r="S76" s="46" t="inlineStr">
         <is>
           <t>Bonjour Maïté Belmir,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade est la seule plante que les chenilles du monarque peuvent manger, et le déclin du papillon suit celui de la plante dans les zones agricoles. Notre pari est simple : si l'asclépiade devient payante, les agriculteurs la gardent.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de la campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -10321,12 +10401,13 @@
       <c r="S77" s="46" t="inlineStr">
         <is>
           <t>Bonjour André Bernard,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade est la seule plante que les chenilles du monarque peuvent manger, et le déclin du papillon suit celui de la plante dans les zones agricoles. Notre pari est simple : si l'asclépiade devient payante, les agriculteurs la gardent.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de la campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -10410,12 +10491,13 @@
       <c r="S78" s="46" t="inlineStr">
         <is>
           <t>Bonjour Didier Bert,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade est la seule plante que les chenilles du monarque peuvent manger, et le déclin du papillon suit celui de la plante dans les zones agricoles. Notre pari est simple : si l'asclépiade devient payante, les agriculteurs la gardent.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de la campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -10490,8 +10572,10 @@
       <c r="S79" s="46" t="inlineStr">
         <is>
           <t>Bonjour Sophie-Andrée Blondin,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
@@ -10573,9 +10657,10 @@
       <c r="S80" s="46" t="inlineStr">
         <is>
           <t>Bonjour Pierre Brochu,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'Estrie compte encore des producteurs d'asclépiade, et une des premières usines de transformation de la fibre était à Granby.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris entre autres parce qu'une des premières usines de transformation de la fibre était à Granby, et que l'Estrie compte encore des producteurs d'asclépiade.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
@@ -10662,12 +10747,13 @@
       <c r="S81" s="46" t="inlineStr">
         <is>
           <t>Bonjour Gilles Bérubé,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-La Montérégie est une des régions où l'asclépiade se cultive encore, et c'est de champs comme ceux-là que vient la fibre qu'on transforme.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -10746,12 +10832,13 @@
       <c r="S82" s="46" t="inlineStr">
         <is>
           <t>Bonjour Daphné Cameron,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-Huit ans après l'effondrement de la première filière québécoise de l'asclépiade, on achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes à Québec.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -10830,8 +10917,10 @@
       <c r="S83" s="46" t="inlineStr">
         <is>
           <t>Bonjour Godefroy Macaire Chabi,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
@@ -10913,12 +11002,13 @@
       <c r="S84" s="46" t="inlineStr">
         <is>
           <t>Bonjour Sara Champagne,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade est la seule plante que les chenilles du monarque peuvent manger, et le déclin du papillon suit celui de la plante dans les zones agricoles. Notre pari est simple : si l'asclépiade devient payante, les agriculteurs la gardent.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de la campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -10997,12 +11087,13 @@
       <c r="S85" s="46" t="inlineStr">
         <is>
           <t>Bonjour Sarah Champagne,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-Huit ans après l'effondrement de la première filière québécoise de l'asclépiade, on achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes à Québec.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -11081,12 +11172,13 @@
       <c r="S86" s="46" t="inlineStr">
         <is>
           <t>Bonjour Éric-Pierre Champagne,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade est la seule plante que les chenilles du monarque peuvent manger, et le déclin du papillon suit celui de la plante dans les zones agricoles. Notre pari est simple : si l'asclépiade devient payante, les agriculteurs la gardent.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de la campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -11165,12 +11257,13 @@
       <c r="S87" s="46" t="inlineStr">
         <is>
           <t>Bonjour Marine Corniou,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade est la seule plante que les chenilles du monarque peuvent manger, et le déclin du papillon suit celui de la plante dans les zones agricoles. Notre pari est simple : si l'asclépiade devient payante, les agriculteurs la gardent.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de la campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -11245,12 +11338,13 @@
       <c r="S88" s="46" t="inlineStr">
         <is>
           <t>Bonjour Catherine Crépeau,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade est la seule plante que les chenilles du monarque peuvent manger, et le déclin du papillon suit celui de la plante dans les zones agricoles. Notre pari est simple : si l'asclépiade devient payante, les agriculteurs la gardent.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de la campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -11329,9 +11423,10 @@
       <c r="S89" s="46" t="inlineStr">
         <is>
           <t>Bonjour Laurence Dami-Houle,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade est une vivace indigène qui pousse avec peu d'intrants, ce qui en fait une culture intéressante pour des régions où les grandes cultures rendent mal.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
@@ -11414,12 +11509,13 @@
       <c r="S90" s="46" t="inlineStr">
         <is>
           <t>Bonjour Amélie Daoust-Boisvert,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-La Montérégie est une des régions où l'asclépiade se cultive encore, et c'est de champs comme ceux-là que vient la fibre qu'on transforme.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de la campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -11494,9 +11590,10 @@
       <c r="S91" s="46" t="inlineStr">
         <is>
           <t>Bonjour Dominique Degré,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-La Montérégie est une des régions où l'asclépiade se cultive encore, et c'est de champs comme ceux-là que vient la fibre qu'on transforme.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
@@ -11583,12 +11680,13 @@
       <c r="S92" s="46" t="inlineStr">
         <is>
           <t>Bonjour Quentin Dufranne,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade est la seule plante que les chenilles du monarque peuvent manger, et le déclin du papillon suit celui de la plante dans les zones agricoles. Notre pari est simple : si l'asclépiade devient payante, les agriculteurs la gardent.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de la campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -11667,12 +11765,13 @@
       <c r="S93" s="46" t="inlineStr">
         <is>
           <t>Bonjour Ève Dumas,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-Huit ans après l'effondrement de la première filière québécoise de l'asclépiade, on achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes à Québec.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -11751,8 +11850,10 @@
       <c r="S94" s="46" t="inlineStr">
         <is>
           <t>Bonjour Michel Fortier,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
@@ -11834,12 +11935,13 @@
       <c r="S95" s="46" t="inlineStr">
         <is>
           <t>Bonjour Marie-Eve Fournier,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a pas de chaîne d'approvisionnement.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -11923,9 +12025,10 @@
       <c r="S96" s="46" t="inlineStr">
         <is>
           <t>Bonjour Raymond Fournier,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-La Montérégie est une des régions où l'asclépiade se cultive encore, et c'est de champs comme ceux-là que vient la fibre qu'on transforme.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
@@ -12007,12 +12110,13 @@
       <c r="S97" s="46" t="inlineStr">
         <is>
           <t>Bonjour Marie-Pier Frappier,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a pas de chaîne d'approvisionnement.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -12096,9 +12200,10 @@
       <c r="S98" s="46" t="inlineStr">
         <is>
           <t>Bonjour Marie-Julie Gagnon,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-La Montérégie est une des régions où l'asclépiade se cultive encore, et c'est de champs comme ceux-là que vient la fibre qu'on transforme.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
@@ -12180,12 +12285,13 @@
       <c r="S99" s="46" t="inlineStr">
         <is>
           <t>Bonjour Chloé Germain-Thérien,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade a eu son grand moment industriel chez vous : l'usine de Saint-Tite achetait 90 % des récoltes du Québec. La filière s'est cassée en 2018, mais des producteurs de la Mauricie cultivent encore, et on continue d'acheter leur récolte.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris entre autres parce que l'asclépiade a eu son grand moment industriel chez vous : l'usine de Saint-Tite achetait 90 % des récoltes du Québec avant que la filière se casse en 2018. Des producteurs de la Mauricie cultivent encore, et on continue d'acheter leur récolte.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -12269,12 +12375,13 @@
       <c r="S100" s="46" t="inlineStr">
         <is>
           <t>Bonjour Charlotte Glorieux,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-La soie d'asclépiade est une fibre creuse et naturellement hydrophobe attachée aux graines de la plante. On en fait l'isolant de nos manteaux, de nos mitaines et de nos sacs isothermes.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez le plein air. À poids égal, la littérature donne la soie d'asclépiade pour environ 10 % plus isolante que le duvet. C'est un repère de laboratoire, pas une promesse de manteau, et c'est exactement pour ça que je préfère qu'on la teste.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester la fibre plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -12353,12 +12460,13 @@
       <c r="S101" s="46" t="inlineStr">
         <is>
           <t>Bonjour Annie Hudon,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a pas de chaîne d'approvisionnement.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -12437,12 +12545,13 @@
       <c r="S102" s="46" t="inlineStr">
         <is>
           <t>Bonjour Ahmed Kouaou,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade est la seule plante que les chenilles du monarque peuvent manger, et le déclin du papillon suit celui de la plante dans les zones agricoles. Notre pari est simple : si l'asclépiade devient payante, les agriculteurs la gardent.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de la campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -12517,12 +12626,13 @@
       <c r="S103" s="46" t="inlineStr">
         <is>
           <t>Bonjour Tania Krywiak,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade est la seule plante que les chenilles du monarque peuvent manger, et le déclin du papillon suit celui de la plante dans les zones agricoles. Notre pari est simple : si l'asclépiade devient payante, les agriculteurs la gardent.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de la campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -12601,9 +12711,10 @@
       <c r="S104" s="46" t="inlineStr">
         <is>
           <t>Bonjour Jacinthe Lafrance,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade a eu son grand moment industriel chez vous : l'usine de Saint-Tite achetait 90 % des récoltes du Québec. La filière s'est cassée en 2018, mais des producteurs de la Mauricie cultivent encore, et on continue d'acheter leur récolte.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris entre autres parce que l'asclépiade a eu son grand moment industriel chez vous : l'usine de Saint-Tite achetait 90 % des récoltes du Québec avant que la filière se casse en 2018. Des producteurs de la Mauricie cultivent encore, et on continue d'acheter leur récolte.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
@@ -12685,12 +12796,13 @@
       <c r="S105" s="46" t="inlineStr">
         <is>
           <t>Bonjour Bruno Lamolet,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-La Montérégie est une des régions où l'asclépiade se cultive encore, et c'est de champs comme ceux-là que vient la fibre qu'on transforme.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester la fibre plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -12769,12 +12881,13 @@
       <c r="S106" s="46" t="inlineStr">
         <is>
           <t>Bonjour Yvan Lamontagne,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'Estrie compte encore des producteurs d'asclépiade, et une des premières usines de transformation de la fibre était à Granby.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris entre autres parce qu'une des premières usines de transformation de la fibre était à Granby, et que l'Estrie compte encore des producteurs d'asclépiade.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a pas de chaîne d'approvisionnement.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -12858,12 +12971,13 @@
       <c r="S107" s="46" t="inlineStr">
         <is>
           <t>Bonjour Yves Langlois,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'Estrie compte encore des producteurs d'asclépiade, et une des premières usines de transformation de la fibre était à Granby.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris entre autres parce qu'une des premières usines de transformation de la fibre était à Granby, et que l'Estrie compte encore des producteurs d'asclépiade.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester la fibre plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -12942,12 +13056,13 @@
       <c r="S108" s="46" t="inlineStr">
         <is>
           <t>Bonjour Anne Marie Lecomte,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a pas de chaîne d'approvisionnement.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -13026,9 +13141,10 @@
       <c r="S109" s="46" t="inlineStr">
         <is>
           <t>Bonjour Stéphanie Mac Farlane,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-La Montérégie est une des régions où l'asclépiade se cultive encore, et c'est de champs comme ceux-là que vient la fibre qu'on transforme.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
@@ -13115,9 +13231,10 @@
       <c r="S110" s="46" t="inlineStr">
         <is>
           <t>Bonjour Philippe Marois,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-La Montérégie est une des régions où l'asclépiade se cultive encore, et c'est de champs comme ceux-là que vient la fibre qu'on transforme.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
@@ -13199,12 +13316,13 @@
       <c r="S111" s="46" t="inlineStr">
         <is>
           <t>Bonjour Gildas Meneu,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-Huit ans après l'effondrement de la première filière québécoise de l'asclépiade, on achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes à Québec.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -13283,8 +13401,10 @@
       <c r="S112" s="46" t="inlineStr">
         <is>
           <t>Bonjour Louis-Xavier Michaud,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
@@ -13367,12 +13487,13 @@
       <c r="S113" s="46" t="inlineStr">
         <is>
           <t>Bonjour Anne Montplaisir,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-La soie d'asclépiade est une fibre creuse et naturellement hydrophobe attachée aux graines de la plante. On en fait l'isolant de nos manteaux, de nos mitaines et de nos sacs isothermes.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez le plein air. À poids égal, la littérature donne la soie d'asclépiade pour environ 10 % plus isolante que le duvet. C'est un repère de laboratoire, pas une promesse de manteau, et c'est exactement pour ça que je préfère qu'on la teste.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester la fibre plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -13451,9 +13572,10 @@
       <c r="S114" s="46" t="inlineStr">
         <is>
           <t>Bonjour Karianne Nepton-Philippe,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade est une vivace indigène qui pousse avec peu d'intrants, ce qui en fait une culture intéressante pour des régions où les grandes cultures rendent mal.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
@@ -13535,9 +13657,10 @@
       <c r="S115" s="46" t="inlineStr">
         <is>
           <t>Bonjour Geneviève Normand,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-La Montérégie est une des régions où l'asclépiade se cultive encore, et c'est de champs comme ceux-là que vient la fibre qu'on transforme.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
@@ -13624,9 +13747,10 @@
       <c r="S116" s="46" t="inlineStr">
         <is>
           <t>Bonjour Carole Payer,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade se cultive dans votre région depuis la première vague de 2013, et plusieurs des producteurs qui ont tenu bon nous vendent encore leur récolte.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris entre autres parce que l'asclépiade se cultive dans votre région depuis la première vague de 2013, et que plusieurs des producteurs qui ont tenu bon nous vendent encore leur récolte.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
@@ -13708,12 +13832,13 @@
       <c r="S117" s="46" t="inlineStr">
         <is>
           <t>Bonjour Boris Proulx,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade est la seule plante que les chenilles du monarque peuvent manger, et le déclin du papillon suit celui de la plante dans les zones agricoles. Notre pari est simple : si l'asclépiade devient payante, les agriculteurs la gardent.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de la campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -13788,12 +13913,13 @@
       <c r="S118" s="46" t="inlineStr">
         <is>
           <t>Bonjour Philippe Robitaille-Grou,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade est la seule plante que les chenilles du monarque peuvent manger, et le déclin du papillon suit celui de la plante dans les zones agricoles. Notre pari est simple : si l'asclépiade devient payante, les agriculteurs la gardent.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de la campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -13868,12 +13994,13 @@
       <c r="S119" s="46" t="inlineStr">
         <is>
           <t>Bonjour Gwen Roley,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade est la seule plante que les chenilles du monarque peuvent manger, et le déclin du papillon suit celui de la plante dans les zones agricoles. Notre pari est simple : si l'asclépiade devient payante, les agriculteurs la gardent.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de la campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -13948,12 +14075,13 @@
       <c r="S120" s="46" t="inlineStr">
         <is>
           <t>Bonjour Mathieu-Robert Sauvé,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade est la seule plante que les chenilles du monarque peuvent manger, et le déclin du papillon suit celui de la plante dans les zones agricoles. Notre pari est simple : si l'asclépiade devient payante, les agriculteurs la gardent.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de la campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -14028,12 +14156,13 @@
       <c r="S121" s="46" t="inlineStr">
         <is>
           <t>Bonjour Pierre St-Arnaud,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-Huit ans après l'effondrement de la première filière québécoise de l'asclépiade, on achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes à Québec.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -14108,12 +14237,13 @@
       <c r="S122" s="46" t="inlineStr">
         <is>
           <t>Bonjour Katherine Tremblay,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-La Montérégie est une des régions où l'asclépiade se cultive encore, et c'est de champs comme ceux-là que vient la fibre qu'on transforme.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a pas de chaîne d'approvisionnement.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -14197,12 +14327,13 @@
       <c r="S123" s="46" t="inlineStr">
         <is>
           <t>Bonjour Michel Tremblay,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade se cultive dans votre région depuis la première vague de 2013, et plusieurs des producteurs qui ont tenu bon nous vendent encore leur récolte.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris entre autres parce que l'asclépiade se cultive dans votre région depuis la première vague de 2013, et que plusieurs des producteurs qui ont tenu bon nous vendent encore leur récolte.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester la fibre plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -14281,12 +14412,13 @@
       <c r="S124" s="46" t="inlineStr">
         <is>
           <t>Bonjour Martin Vallières,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a pas de chaîne d'approvisionnement.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -14366,12 +14498,13 @@
       <c r="S125" s="46" t="inlineStr">
         <is>
           <t>Bonjour Yanick Villedieu,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade est la seule plante que les chenilles du monarque peuvent manger, et le déclin du papillon suit celui de la plante dans les zones agricoles. Notre pari est simple : si l'asclépiade devient payante, les agriculteurs la gardent.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de la campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -14450,12 +14583,13 @@
       <c r="S126" s="46" t="inlineStr">
         <is>
           <t>Bonjour Jonathan Allard,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade est la seule plante que les chenilles du monarque peuvent manger, et le déclin du papillon suit celui de la plante dans les zones agricoles. Notre pari est simple : si l'asclépiade devient payante, les agriculteurs la gardent.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de la campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -14539,12 +14673,13 @@
       <c r="S127" s="46" t="inlineStr">
         <is>
           <t>Bonjour Anick Baribeau,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade a eu son grand moment industriel chez vous : l'usine de Saint-Tite achetait 90 % des récoltes du Québec. La filière s'est cassée en 2018, mais des producteurs de la Mauricie cultivent encore, et on continue d'acheter leur récolte.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris entre autres parce que l'asclépiade a eu son grand moment industriel chez vous : l'usine de Saint-Tite achetait 90 % des récoltes du Québec avant que la filière se casse en 2018. Des producteurs de la Mauricie cultivent encore, et on continue d'acheter leur récolte.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de la campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -14624,12 +14759,13 @@
       <c r="S128" s="46" t="inlineStr">
         <is>
           <t>Bonjour Félix-Antoine Beauchemin,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-La Montérégie est une des régions où l'asclépiade se cultive encore, et c'est de champs comme ceux-là que vient la fibre qu'on transforme.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a pas de chaîne d'approvisionnement.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -14708,12 +14844,13 @@
       <c r="S129" s="46" t="inlineStr">
         <is>
           <t>Bonjour Karim Benessaieh,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade est la seule plante que les chenilles du monarque peuvent manger, et le déclin du papillon suit celui de la plante dans les zones agricoles. Notre pari est simple : si l'asclépiade devient payante, les agriculteurs la gardent.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de la campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -14793,12 +14930,13 @@
       <c r="S130" s="46" t="inlineStr">
         <is>
           <t>Bonjour Julia Bernier,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade se cultive dans votre région depuis la première vague de 2013, et plusieurs des producteurs qui ont tenu bon nous vendent encore leur récolte.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris entre autres parce que l'asclépiade se cultive dans votre région depuis la première vague de 2013, et que plusieurs des producteurs qui ont tenu bon nous vendent encore leur récolte.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. J'ai du matériel photo qui montre bien le contraste : la gousse dans le champ, la soie dans la main, le produit porté. L'atelier de Limoilou est ouvert si vous voulez voir la matière.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière, et j'ai du matériel photo.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -14882,12 +15020,13 @@
       <c r="S131" s="46" t="inlineStr">
         <is>
           <t>Bonjour Karine Boivin Forcier,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-Un de nos fournisseurs d'asclépiade cultive au Lac-Saint-Jean depuis nos tout débuts, et il l'est encore aujourd'hui. La fibre de chez vous se retrouve dans nos produits.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris entre autres parce qu'un de nos fournisseurs d'asclépiade cultive au Lac-Saint-Jean depuis nos tout débuts, et qu'il l'est encore aujourd'hui. La fibre de chez vous se retrouve dans nos produits.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a pas de chaîne d'approvisionnement.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -14967,8 +15106,10 @@
       <c r="S132" s="46" t="inlineStr">
         <is>
           <t>Bonjour Audrey Bonaque,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
@@ -15050,12 +15191,13 @@
       <c r="S133" s="46" t="inlineStr">
         <is>
           <t>Bonjour Luc Boulanger,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade est la plante que les agriculteurs arrachent depuis 50 ans. La soie attachée à ses graines est ce qui isole nos manteaux, nos mitaines et nos tuques.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. J'ai du matériel photo qui montre bien le contraste : la gousse dans le champ, la soie dans la main, le produit porté. L'atelier de Limoilou est ouvert si vous voulez voir la matière.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière, et j'ai du matériel photo.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -15134,8 +15276,10 @@
       <c r="S134" s="46" t="inlineStr">
         <is>
           <t>Bonjour Mario Boulianne,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
@@ -15222,12 +15366,13 @@
       <c r="S135" s="46" t="inlineStr">
         <is>
           <t>Bonjour Bernard Brault,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-La Montérégie est une des régions où l'asclépiade se cultive encore, et c'est de champs comme ceux-là que vient la fibre qu'on transforme.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester la fibre plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -15311,12 +15456,13 @@
       <c r="S136" s="46" t="inlineStr">
         <is>
           <t>Bonjour Pierre Brisson,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a pas de chaîne d'approvisionnement.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -15395,8 +15541,10 @@
       <c r="S137" s="46" t="inlineStr">
         <is>
           <t>Bonjour Laurence Brisson Dubreuil,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
@@ -15479,8 +15627,10 @@
       <c r="S138" s="46" t="inlineStr">
         <is>
           <t>Bonjour Nathaniel Bronner,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
@@ -15562,12 +15712,13 @@
       <c r="S139" s="46" t="inlineStr">
         <is>
           <t>Bonjour Marie-France Bélanger,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade est la plante que les agriculteurs arrachent depuis 50 ans. La soie attachée à ses graines est ce qui isole nos manteaux, nos mitaines et nos tuques.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. J'ai du matériel photo qui montre bien le contraste : la gousse dans le champ, la soie dans la main, le produit porté. L'atelier de Limoilou est ouvert si vous voulez voir la matière.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière, et j'ai du matériel photo.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -15647,12 +15798,13 @@
       <c r="S140" s="46" t="inlineStr">
         <is>
           <t>Bonjour Diane Bérard,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a pas de chaîne d'approvisionnement.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -15736,12 +15888,13 @@
       <c r="S141" s="46" t="inlineStr">
         <is>
           <t>Bonjour Julien Cayouette,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade est la seule plante que les chenilles du monarque peuvent manger, et le déclin du papillon suit celui de la plante dans les zones agricoles. Notre pari est simple : si l'asclépiade devient payante, les agriculteurs la gardent.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de la campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -15820,8 +15973,10 @@
       <c r="S142" s="46" t="inlineStr">
         <is>
           <t>Bonjour Rudy Chabannes,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
@@ -15908,8 +16063,10 @@
       <c r="S143" s="46" t="inlineStr">
         <is>
           <t>Bonjour Denis-Martin Chabot,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
@@ -15992,8 +16149,10 @@
       <c r="S144" s="46" t="inlineStr">
         <is>
           <t>Bonjour Loubna Majda Chourouk,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
@@ -16080,12 +16239,13 @@
       <c r="S145" s="46" t="inlineStr">
         <is>
           <t>Bonjour Sarah Collardey,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade est la seule plante que les chenilles du monarque peuvent manger, et le déclin du papillon suit celui de la plante dans les zones agricoles. Notre pari est simple : si l'asclépiade devient payante, les agriculteurs la gardent.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de la campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -16165,9 +16325,10 @@
       <c r="S146" s="46" t="inlineStr">
         <is>
           <t>Bonjour Kathleen Couillard,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-La Montérégie est une des régions où l'asclépiade se cultive encore, et c'est de champs comme ceux-là que vient la fibre qu'on transforme.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
@@ -16254,12 +16415,13 @@
       <c r="S147" s="46" t="inlineStr">
         <is>
           <t>Bonjour Oumou DIAKITÉ,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade est la plante que les agriculteurs arrachent depuis 50 ans. La soie attachée à ses graines est ce qui isole nos manteaux, nos mitaines et nos tuques.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. J'ai du matériel photo qui montre bien le contraste : la gousse dans le champ, la soie dans la main, le produit porté. L'atelier de Limoilou est ouvert si vous voulez voir la matière.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière, et j'ai du matériel photo.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -16338,12 +16500,13 @@
       <c r="S148" s="46" t="inlineStr">
         <is>
           <t>Bonjour Agnès Delavault,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade est la plante que les agriculteurs arrachent depuis 50 ans. La soie attachée à ses graines est ce qui isole nos manteaux, nos mitaines et nos tuques.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. J'ai du matériel photo qui montre bien le contraste : la gousse dans le champ, la soie dans la main, le produit porté. L'atelier de Limoilou est ouvert si vous voulez voir la matière.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière, et j'ai du matériel photo.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -16423,12 +16586,13 @@
       <c r="S149" s="46" t="inlineStr">
         <is>
           <t>Bonjour Marcelin Delice,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade est la seule plante que les chenilles du monarque peuvent manger, et le déclin du papillon suit celui de la plante dans les zones agricoles. Notre pari est simple : si l'asclépiade devient payante, les agriculteurs la gardent.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de la campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -16508,12 +16672,13 @@
       <c r="S150" s="46" t="inlineStr">
         <is>
           <t>Bonjour Alain Demers,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-La soie d'asclépiade est une fibre creuse et naturellement hydrophobe attachée aux graines de la plante. On en fait l'isolant de nos manteaux, de nos mitaines et de nos sacs isothermes.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez le plein air. À poids égal, la littérature donne la soie d'asclépiade pour environ 10 % plus isolante que le duvet. C'est un repère de laboratoire, pas une promesse de manteau, et c'est exactement pour ça que je préfère qu'on la teste.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester la fibre plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -16592,12 +16757,13 @@
       <c r="S151" s="46" t="inlineStr">
         <is>
           <t>Bonjour Ivanoh Demers,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a pas de chaîne d'approvisionnement.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -16677,12 +16843,13 @@
       <c r="S152" s="46" t="inlineStr">
         <is>
           <t>Bonjour Claude Deschênes,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade est la plante que les agriculteurs arrachent depuis 50 ans. La soie attachée à ses graines est ce qui isole nos manteaux, nos mitaines et nos tuques.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. J'ai du matériel photo qui montre bien le contraste : la gousse dans le champ, la soie dans la main, le produit porté. L'atelier de Limoilou est ouvert si vous voulez voir la matière.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière, et j'ai du matériel photo.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -16761,9 +16928,10 @@
       <c r="S153" s="46" t="inlineStr">
         <is>
           <t>Bonjour Thomas Deshaies,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'Estrie compte encore des producteurs d'asclépiade, et une des premières usines de transformation de la fibre était à Granby.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris entre autres parce qu'une des premières usines de transformation de la fibre était à Granby, et que l'Estrie compte encore des producteurs d'asclépiade.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
@@ -16850,12 +17018,13 @@
       <c r="S154" s="46" t="inlineStr">
         <is>
           <t>Bonjour Claude Desjardins,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a pas de chaîne d'approvisionnement.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -16935,12 +17104,13 @@
       <c r="S155" s="46" t="inlineStr">
         <is>
           <t>Bonjour Martine Deslauriers,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade est la seule plante que les chenilles du monarque peuvent manger, et le déclin du papillon suit celui de la plante dans les zones agricoles. Notre pari est simple : si l'asclépiade devient payante, les agriculteurs la gardent.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de la campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -17024,8 +17194,10 @@
       <c r="S156" s="46" t="inlineStr">
         <is>
           <t>Bonjour Marie-Claude Di Lillo,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
@@ -17107,8 +17279,10 @@
       <c r="S157" s="46" t="inlineStr">
         <is>
           <t>Bonjour Jean-René Dufort,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
@@ -17191,12 +17365,13 @@
       <c r="S158" s="46" t="inlineStr">
         <is>
           <t>Bonjour Richard Dupaul,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a pas de chaîne d'approvisionnement.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -17280,12 +17455,13 @@
       <c r="S159" s="46" t="inlineStr">
         <is>
           <t>Bonjour Stéphanie Dupuis,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade est la plante que les agriculteurs arrachent depuis 50 ans. La soie attachée à ses graines est ce qui isole nos manteaux, nos mitaines et nos tuques.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. J'ai du matériel photo qui montre bien le contraste : la gousse dans le champ, la soie dans la main, le produit porté. L'atelier de Limoilou est ouvert si vous voulez voir la matière.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière, et j'ai du matériel photo.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -17365,12 +17541,13 @@
       <c r="S160" s="46" t="inlineStr">
         <is>
           <t>Bonjour Maxim Fauteux,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-Un de nos fournisseurs d'asclépiade cultive au Lac-Saint-Jean depuis nos tout débuts, et il l'est encore aujourd'hui. La fibre de chez vous se retrouve dans nos produits.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris entre autres parce qu'un de nos fournisseurs d'asclépiade cultive au Lac-Saint-Jean depuis nos tout débuts, et qu'il l'est encore aujourd'hui. La fibre de chez vous se retrouve dans nos produits.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de la campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -17449,8 +17626,10 @@
       <c r="S161" s="46" t="inlineStr">
         <is>
           <t>Bonjour Ronald Georges,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
@@ -17528,12 +17707,13 @@
       <c r="S162" s="46" t="inlineStr">
         <is>
           <t>Bonjour Stéphane Giroux,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a pas de chaîne d'approvisionnement.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -17612,12 +17792,13 @@
       <c r="S163" s="46" t="inlineStr">
         <is>
           <t>Bonjour Zacharie Goudreault,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade est la seule plante que les chenilles du monarque peuvent manger, et le déclin du papillon suit celui de la plante dans les zones agricoles. Notre pari est simple : si l'asclépiade devient payante, les agriculteurs la gardent.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de la campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -17697,12 +17878,13 @@
       <c r="S164" s="46" t="inlineStr">
         <is>
           <t>Bonjour Isabelle Grégoire,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade est la plante que les agriculteurs arrachent depuis 50 ans. La soie attachée à ses graines est ce qui isole nos manteaux, nos mitaines et nos tuques.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. J'ai du matériel photo qui montre bien le contraste : la gousse dans le champ, la soie dans la main, le produit porté. L'atelier de Limoilou est ouvert si vous voulez voir la matière.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière, et j'ai du matériel photo.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -17781,12 +17963,13 @@
       <c r="S165" s="46" t="inlineStr">
         <is>
           <t>Bonjour Chantal Guy,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade est la plante que les agriculteurs arrachent depuis 50 ans. La soie attachée à ses graines est ce qui isole nos manteaux, nos mitaines et nos tuques.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. J'ai du matériel photo qui montre bien le contraste : la gousse dans le champ, la soie dans la main, le produit porté. L'atelier de Limoilou est ouvert si vous voulez voir la matière.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière, et j'ai du matériel photo.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -17865,12 +18048,13 @@
       <c r="S166" s="46" t="inlineStr">
         <is>
           <t>Bonjour Matthieu Hains,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a pas de chaîne d'approvisionnement.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -18035,12 +18219,13 @@
       <c r="S168" s="46" t="inlineStr">
         <is>
           <t>Bonjour ANGELO JEAN-BAPTISTE,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade est la seule plante que les chenilles du monarque peuvent manger, et le déclin du papillon suit celui de la plante dans les zones agricoles. Notre pari est simple : si l'asclépiade devient payante, les agriculteurs la gardent.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de la campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -18124,12 +18309,13 @@
       <c r="S169" s="46" t="inlineStr">
         <is>
           <t>Bonjour Andréanne Joly,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade est la plante que les agriculteurs arrachent depuis 50 ans. La soie attachée à ses graines est ce qui isole nos manteaux, nos mitaines et nos tuques.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. J'ai du matériel photo qui montre bien le contraste : la gousse dans le champ, la soie dans la main, le produit porté. L'atelier de Limoilou est ouvert si vous voulez voir la matière.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière, et j'ai du matériel photo.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -18208,12 +18394,13 @@
       <c r="S170" s="46" t="inlineStr">
         <is>
           <t>Bonjour Hugo Joncas,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a pas de chaîne d'approvisionnement.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -18297,8 +18484,10 @@
       <c r="S171" s="46" t="inlineStr">
         <is>
           <t>Bonjour Philémon La Frenière-Prémont,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
@@ -18385,8 +18574,10 @@
       <c r="S172" s="46" t="inlineStr">
         <is>
           <t>Bonjour Henri Laban,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
@@ -18554,12 +18745,13 @@
       <c r="S174" s="46" t="inlineStr">
         <is>
           <t>Bonjour Joannie Lafrenière,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade est la plante que les agriculteurs arrachent depuis 50 ans. La soie attachée à ses graines est ce qui isole nos manteaux, nos mitaines et nos tuques.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. J'ai du matériel photo qui montre bien le contraste : la gousse dans le champ, la soie dans la main, le produit porté. L'atelier de Limoilou est ouvert si vous voulez voir la matière.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière, et j'ai du matériel photo.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -18634,12 +18826,13 @@
       <c r="S175" s="46" t="inlineStr">
         <is>
           <t>Bonjour Angie Landry,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade est la seule plante que les chenilles du monarque peuvent manger, et le déclin du papillon suit celui de la plante dans les zones agricoles. Notre pari est simple : si l'asclépiade devient payante, les agriculteurs la gardent.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de la campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -18719,12 +18912,13 @@
       <c r="S176" s="46" t="inlineStr">
         <is>
           <t>Bonjour Camille Langlade,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade est la seule plante que les chenilles du monarque peuvent manger, et le déclin du papillon suit celui de la plante dans les zones agricoles. Notre pari est simple : si l'asclépiade devient payante, les agriculteurs la gardent.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de la campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -18808,8 +19002,10 @@
       <c r="S177" s="46" t="inlineStr">
         <is>
           <t>Bonjour Claudia Larochelle,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
@@ -18891,12 +19087,13 @@
       <c r="S178" s="46" t="inlineStr">
         <is>
           <t>Bonjour Étienne Leblanc,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade est la seule plante que les chenilles du monarque peuvent manger, et le déclin du papillon suit celui de la plante dans les zones agricoles. Notre pari est simple : si l'asclépiade devient payante, les agriculteurs la gardent.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de la campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -18975,12 +19172,13 @@
       <c r="S179" s="46" t="inlineStr">
         <is>
           <t>Bonjour Louise Leduc,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade est la plante que les agriculteurs arrachent depuis 50 ans. La soie attachée à ses graines est ce qui isole nos manteaux, nos mitaines et nos tuques.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. J'ai du matériel photo qui montre bien le contraste : la gousse dans le champ, la soie dans la main, le produit porté. L'atelier de Limoilou est ouvert si vous voulez voir la matière.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière, et j'ai du matériel photo.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -19060,12 +19258,13 @@
       <c r="S180" s="46" t="inlineStr">
         <is>
           <t>Bonjour Guillaume Longuépée,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a pas de chaîne d'approvisionnement.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -19144,12 +19343,13 @@
       <c r="S181" s="46" t="inlineStr">
         <is>
           <t>Bonjour Roxane Léouzon,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a pas de chaîne d'approvisionnement.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -19229,8 +19429,10 @@
       <c r="S182" s="46" t="inlineStr">
         <is>
           <t>Bonjour Ève Lévesque,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
@@ -19313,8 +19515,10 @@
       <c r="S183" s="46" t="inlineStr">
         <is>
           <t>Bonjour Sophie Mangado,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
@@ -19401,12 +19605,13 @@
       <c r="S184" s="46" t="inlineStr">
         <is>
           <t>Bonjour Colin McGregor,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade est la seule plante que les chenilles du monarque peuvent manger, et le déclin du papillon suit celui de la plante dans les zones agricoles. Notre pari est simple : si l'asclépiade devient payante, les agriculteurs la gardent.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de la campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -19485,12 +19690,13 @@
       <c r="S185" s="46" t="inlineStr">
         <is>
           <t>Bonjour Isabelle Morin,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade est la plante que les agriculteurs arrachent depuis 50 ans. La soie attachée à ses graines est ce qui isole nos manteaux, nos mitaines et nos tuques.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. J'ai du matériel photo qui montre bien le contraste : la gousse dans le champ, la soie dans la main, le produit porté. L'atelier de Limoilou est ouvert si vous voulez voir la matière.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière, et j'ai du matériel photo.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -19574,12 +19780,13 @@
       <c r="S186" s="46" t="inlineStr">
         <is>
           <t>Bonjour Timothy Morson,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade se cultive dans votre région depuis la première vague de 2013, et plusieurs des producteurs qui ont tenu bon nous vendent encore leur récolte.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris entre autres parce que l'asclépiade se cultive dans votre région depuis la première vague de 2013, et que plusieurs des producteurs qui ont tenu bon nous vendent encore leur récolte.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a pas de chaîne d'approvisionnement.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -19663,12 +19870,13 @@
       <c r="S187" s="46" t="inlineStr">
         <is>
           <t>Bonjour Rachid Najahi,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade est la plante que les agriculteurs arrachent depuis 50 ans. La soie attachée à ses graines est ce qui isole nos manteaux, nos mitaines et nos tuques.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. J'ai du matériel photo qui montre bien le contraste : la gousse dans le champ, la soie dans la main, le produit porté. L'atelier de Limoilou est ouvert si vous voulez voir la matière.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière, et j'ai du matériel photo.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -19748,8 +19956,10 @@
       <c r="S188" s="46" t="inlineStr">
         <is>
           <t>Bonjour Richard Olivier,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
@@ -19836,9 +20046,10 @@
       <c r="S189" s="46" t="inlineStr">
         <is>
           <t>Bonjour MELISSA PELLETIER,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-La Montérégie est une des régions où l'asclépiade se cultive encore, et c'est de champs comme ceux-là que vient la fibre qu'on transforme.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
@@ -19920,9 +20131,10 @@
       <c r="S190" s="46" t="inlineStr">
         <is>
           <t>Bonjour Isaac Peltz,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade se cultive dans votre région depuis la première vague de 2013, et plusieurs des producteurs qui ont tenu bon nous vendent encore leur récolte.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris entre autres parce que l'asclépiade se cultive dans votre région depuis la première vague de 2013, et que plusieurs des producteurs qui ont tenu bon nous vendent encore leur récolte.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
@@ -20004,12 +20216,13 @@
       <c r="S191" s="46" t="inlineStr">
         <is>
           <t>Bonjour Frédéric Perron,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade est la plante que les agriculteurs arrachent depuis 50 ans. La soie attachée à ses graines est ce qui isole nos manteaux, nos mitaines et nos tuques.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. J'ai du matériel photo qui montre bien le contraste : la gousse dans le champ, la soie dans la main, le produit porté. L'atelier de Limoilou est ouvert si vous voulez voir la matière.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière, et j'ai du matériel photo.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -20093,8 +20306,10 @@
       <c r="S192" s="46" t="inlineStr">
         <is>
           <t>Bonjour Nathalie Petrowski,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
@@ -20176,8 +20391,10 @@
       <c r="S193" s="46" t="inlineStr">
         <is>
           <t>Bonjour Francis Plourde,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
@@ -20264,8 +20481,10 @@
       <c r="S194" s="46" t="inlineStr">
         <is>
           <t>Bonjour Raymonde Provencher,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
@@ -20352,12 +20571,13 @@
       <c r="S195" s="46" t="inlineStr">
         <is>
           <t>Bonjour Richard Prudhomme,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade est la plante que les agriculteurs arrachent depuis 50 ans. La soie attachée à ses graines est ce qui isole nos manteaux, nos mitaines et nos tuques.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. J'ai du matériel photo qui montre bien le contraste : la gousse dans le champ, la soie dans la main, le produit porté. L'atelier de Limoilou est ouvert si vous voulez voir la matière.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière, et j'ai du matériel photo.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -20441,12 +20661,13 @@
       <c r="S196" s="46" t="inlineStr">
         <is>
           <t>Bonjour Pascale Renaud,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade est la plante que les agriculteurs arrachent depuis 50 ans. La soie attachée à ses graines est ce qui isole nos manteaux, nos mitaines et nos tuques.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. J'ai du matériel photo qui montre bien le contraste : la gousse dans le champ, la soie dans la main, le produit porté. L'atelier de Limoilou est ouvert si vous voulez voir la matière.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière, et j'ai du matériel photo.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -20525,12 +20746,13 @@
       <c r="S197" s="46" t="inlineStr">
         <is>
           <t>Bonjour Marc Sony Ricot,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade est la plante que les agriculteurs arrachent depuis 50 ans. La soie attachée à ses graines est ce qui isole nos manteaux, nos mitaines et nos tuques.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. J'ai du matériel photo qui montre bien le contraste : la gousse dans le champ, la soie dans la main, le produit porté. L'atelier de Limoilou est ouvert si vous voulez voir la matière.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière, et j'ai du matériel photo.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -20614,12 +20836,13 @@
       <c r="S198" s="46" t="inlineStr">
         <is>
           <t>Bonjour Marie-Paul Rouleau,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade est la seule plante que les chenilles du monarque peuvent manger, et le déclin du papillon suit celui de la plante dans les zones agricoles. Notre pari est simple : si l'asclépiade devient payante, les agriculteurs la gardent.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de la campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -20694,8 +20917,10 @@
       <c r="S199" s="46" t="inlineStr">
         <is>
           <t>Bonjour Emmalie Ruest,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
@@ -20777,9 +21002,10 @@
       <c r="S200" s="46" t="inlineStr">
         <is>
           <t>Bonjour Louis-Philippe Samson,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade se cultive dans votre région depuis la première vague de 2013, et plusieurs des producteurs qui ont tenu bon nous vendent encore leur récolte.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris entre autres parce que l'asclépiade se cultive dans votre région depuis la première vague de 2013, et que plusieurs des producteurs qui ont tenu bon nous vendent encore leur récolte.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
@@ -20861,12 +21087,13 @@
       <c r="S201" s="46" t="inlineStr">
         <is>
           <t>Bonjour Catherine Schlager,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade est la plante que les agriculteurs arrachent depuis 50 ans. La soie attachée à ses graines est ce qui isole nos manteaux, nos mitaines et nos tuques.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. J'ai du matériel photo qui montre bien le contraste : la gousse dans le champ, la soie dans la main, le produit porté. L'atelier de Limoilou est ouvert si vous voulez voir la matière.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière, et j'ai du matériel photo.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -20941,12 +21168,13 @@
       <c r="S202" s="46" t="inlineStr">
         <is>
           <t>Bonjour Olivier Schmouker,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a pas de chaîne d'approvisionnement.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -21021,8 +21249,10 @@
       <c r="S203" s="46" t="inlineStr">
         <is>
           <t>Bonjour Jacques Sennechael,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
@@ -21104,12 +21334,13 @@
       <c r="S204" s="46" t="inlineStr">
         <is>
           <t>Bonjour Alexandre Shields,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade est la seule plante que les chenilles du monarque peuvent manger, et le déclin du papillon suit celui de la plante dans les zones agricoles. Notre pari est simple : si l'asclépiade devient payante, les agriculteurs la gardent.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de la campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -21184,12 +21415,13 @@
       <c r="S205" s="46" t="inlineStr">
         <is>
           <t>Bonjour Chloé Sondervorst,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade est la seule plante que les chenilles du monarque peuvent manger, et le déclin du papillon suit celui de la plante dans les zones agricoles. Notre pari est simple : si l'asclépiade devient payante, les agriculteurs la gardent.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de la campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -21273,9 +21505,10 @@
       <c r="S206" s="46" t="inlineStr">
         <is>
           <t>Bonjour Kimberley Sullivan,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-La Montérégie est une des régions où l'asclépiade se cultive encore, et c'est de champs comme ceux-là que vient la fibre qu'on transforme.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
@@ -21358,12 +21591,13 @@
       <c r="S207" s="46" t="inlineStr">
         <is>
           <t>Bonjour William Thériault,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-La Montérégie est une des régions où l'asclépiade se cultive encore, et c'est de champs comme ceux-là que vient la fibre qu'on transforme.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a pas de chaîne d'approvisionnement.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -21442,12 +21676,13 @@
       <c r="S208" s="46" t="inlineStr">
         <is>
           <t>Bonjour Katia Tobar,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a pas de chaîne d'approvisionnement.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -21522,12 +21757,13 @@
       <c r="S209" s="46" t="inlineStr">
         <is>
           <t>Bonjour Martin Tremblay,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade est la seule plante que les chenilles du monarque peuvent manger, et le déclin du papillon suit celui de la plante dans les zones agricoles. Notre pari est simple : si l'asclépiade devient payante, les agriculteurs la gardent.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de la campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -21606,8 +21842,10 @@
       <c r="S210" s="46" t="inlineStr">
         <is>
           <t>Bonjour Marie-Christine Trottier,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
@@ -21689,12 +21927,13 @@
       <c r="S211" s="46" t="inlineStr">
         <is>
           <t>Bonjour Pierre-Luc Trudel,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a pas de chaîne d'approvisionnement.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -21774,8 +22013,10 @@
       <c r="S212" s="46" t="inlineStr">
         <is>
           <t>Bonjour David Turbis,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
@@ -21857,9 +22098,10 @@
       <c r="S213" s="46" t="inlineStr">
         <is>
           <t>Bonjour Paule Vermot-Desroches,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade a eu son grand moment industriel chez vous : l'usine de Saint-Tite achetait 90 % des récoltes du Québec. La filière s'est cassée en 2018, mais des producteurs de la Mauricie cultivent encore, et on continue d'acheter leur récolte.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris entre autres parce que l'asclépiade a eu son grand moment industriel chez vous : l'usine de Saint-Tite achetait 90 % des récoltes du Québec avant que la filière se casse en 2018. Des producteurs de la Mauricie cultivent encore, et on continue d'acheter leur récolte.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
@@ -21941,8 +22183,10 @@
       <c r="S214" s="46" t="inlineStr">
         <is>
           <t>Bonjour Alexandra Viau,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
@@ -22029,12 +22273,13 @@
       <c r="S215" s="46" t="inlineStr">
         <is>
           <t>Bonjour Raymond Viger,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade est la seule plante que les chenilles du monarque peuvent manger, et le déclin du papillon suit celui de la plante dans les zones agricoles. Notre pari est simple : si l'asclépiade devient payante, les agriculteurs la gardent.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de la campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -22113,8 +22358,10 @@
       <c r="S216" s="46" t="inlineStr">
         <is>
           <t>Bonjour Paul Émile d'Entremont,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
@@ -22196,12 +22443,13 @@
       <c r="S217" s="46" t="inlineStr">
         <is>
           <t>Bonjour Augustin de Baudinière,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade est la seule plante que les chenilles du monarque peuvent manger, et le déclin du papillon suit celui de la plante dans les zones agricoles. Notre pari est simple : si l'asclépiade devient payante, les agriculteurs la gardent.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de la campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -22276,12 +22524,13 @@
       <c r="S218" s="46" t="inlineStr">
         <is>
           <t>Bonjour Ivan de Jacquelin-Dulphe,
-Je dirige Lasclay, une entreprise de Québec qui transforme la soie d'asclépiade en isolant textile : manteaux, mitaines, tuques, sacs isothermes.
-L'asclépiade est la seule plante que les chenilles du monarque peuvent manger, et le déclin du papillon suit celui de la plante dans les zones agricoles. Notre pari est simple : si l'asclépiade devient payante, les agriculteurs la gardent.
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de Québec dont l'atelier est dans Limoilou.
+On travaille l'asclépiade, cette plante que tout le monde connaît ici sous le nom de « petits cochons » et que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe : on la transforme en isolant, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes, vendus en ligne au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de la campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>

</xml_diff>

<commit_message>
Propage le registre corrigé partout et met la page à jour
Les cinq brouillons froids écrits à la main n'avaient pas de présentation: ils
en ont une maintenant, comme les 212 autres. Le document des gabarits est
réécrit sur le squelette de Gabriel plutôt que sur celui du premier jet, et la
matrice ne prescrit plus de nommer ce que le virage a coûté ni d'ajouter la
mise en garde sur les monarques, qui appartient aux textes publics de la marque
et pas à un courriel de presse.

Vérifié sur les 253 brouillons: zéro occurrence des formules pénitentes du
premier jet, et 217 présentations sur 217 dans la liste froide.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015pjLsGPzf1MX1JC7QiKGGk
</commit_message>
<xml_diff>
--- a/communique-dragons/Lasclay_v2.xlsx
+++ b/communique-dragons/Lasclay_v2.xlsx
@@ -3905,6 +3905,8 @@
       <c r="S2" s="46" t="inlineStr">
         <is>
           <t>Bonjour Marie Allard,
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de
+Québec dont l'atelier est dans Limoilou.
 Il y a une belle histoire de sciences dans l'asclépiade. La soie attachée à ses graines n'est
 pas un poil : c'est un tube creux enduit d'une cire hydrophobe, et les fibres portent une
 charge qui les fait se repousser. C'est ce qui forme le parachute autour de la graine, et
@@ -5468,9 +5470,11 @@
       <c r="S20" s="46" t="inlineStr">
         <is>
           <t>Bonjour Gabriel Delisle,
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de
+Québec dont l'atelier est dans Limoilou.
 L'asclépiade a été une histoire mauricienne avant d'être la nôtre : l'usine de Saint-Tite
-achetait 90 % des récoltes du Québec. On est l'entreprise qui a démarré après la chute de
-cette filière, et six ans plus tard on achète encore de l'asclépiade québécoise et on la
+achetait 90 % des récoltes du Québec. On a démarré après la chute de cette filière, et six ans
+plus tard on achète encore de l'asclépiade québécoise et on la
 transforme nous-mêmes à Québec.
 Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la
 culture de l'asclépiade.
@@ -7619,11 +7623,13 @@
       <c r="S45" s="46" t="inlineStr">
         <is>
           <t>Bonjour Réjean Martin,
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de
+Québec dont l'atelier est dans Limoilou.
 Vous couvrez Mékinac, donc Saint-Tite, donc l'endroit où l'asclépiade a eu son grand moment
 industriel au Québec. L'usine achetait 90 % des récoltes de la province avant que la filière
 se casse en 2018.
-On est l'entreprise qui a démarré après. Six ans plus tard, on achète encore de l'asclépiade
-québécoise et on la transforme nous-mêmes à Québec. Mes 2 grandes missions : faire connaître
+On a démarré après. Six ans plus tard, on achète encore de l'asclépiade québécoise et on la
+transforme nous-mêmes à Québec. Mes 2 grandes missions : faire connaître
 l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -22600,12 +22606,13 @@
       <c r="S219" s="46" t="inlineStr">
         <is>
           <t>Bonjour Jean-Michel Leprince,
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de
+Québec dont l'atelier est dans Limoilou.
 Vous couvrez l'asclépiade depuis au moins 2014 : le Téléjournal, la soie d'Amérique partie
 sur l'Everest, le pouvoir absorbant de la fibre sur les hydrocarbures, le lien avec le
 monarque. Vous avez suivi cette histoire plus longtemps que la plupart des entreprises qui
 s'y sont essayées.
-On est l'entreprise qui a démarré après la chute de la première filière. Six ans plus tard,
-on achète encore de l'asclépiade québécoise et on transforme l'isolant nous-mêmes à
+On a démarré après la chute de la première filière. Six ans plus tard, on achète encore de l'asclépiade québécoise et on transforme l'isolant nous-mêmes à
 Limoilou. Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques
 par la culture de l'asclépiade.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
@@ -22683,10 +22690,11 @@
       <c r="S220" s="46" t="inlineStr">
         <is>
           <t>Bonjour Antoine Stab,
+Je m'appelle Gabriel Gouveia et je suis le fondateur de Lasclay, une entreprise de
+Québec dont l'atelier est dans Limoilou.
 Vous aviez écrit sur le soyer du Québec dans Espaces en février 2015, à l'époque où la fibre
 devait remplacer le duvet.
-On est l'entreprise qui a démarré après la chute de cette première filière. Six ans plus
-tard, on achète encore de l'asclépiade québécoise, on transforme l'isolant nous-mêmes, et il
+On a démarré après la chute de cette première filière. Six ans plus tard, on achète encore de l'asclépiade québécoise, on transforme l'isolant nous-mêmes, et il
 existe maintenant un manteau à inserts d'asclépiade amovibles autour de 300 $.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.

</xml_diff>

<commit_message>
Refait les objets de courriel sur le modèle donné par Gabriel
Les objets décrivaient un thème: « Le monarque, l'asclépiade, et l'idée qu'il
faut la rendre payante » est un titre d'essai, pas un objet de courriel, et ils
étaient sans accents. Ils annoncent maintenant la nouvelle avec sa date, sur le
modèle « Nous serons diffusés à Dragons' Den le 17 septembre! »

Quatre variantes selon l'angle plutôt qu'une seule: 253 courriels portant
exactement la même ligne d'objet se comportent comme du publipostage aux yeux
des filtres, et « l'asclépiade s'en va à Dragons' Den » parle plus à un
journaliste agricole qu'à un chroniqueur d'affaires.

Ajoute la colonne Objet au chiffrier d'édition et documente la règle dans
04-gabarits-courriels.md.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015pjLsGPzf1MX1JC7QiKGGk
</commit_message>
<xml_diff>
--- a/communique-dragons/Lasclay_v2.xlsx
+++ b/communique-dragons/Lasclay_v2.xlsx
@@ -1130,7 +1130,7 @@
       </c>
       <c r="L2" s="25" t="inlineStr">
         <is>
-          <t>Suite a votre article de 2026 sur l'asclepiade</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="M2" s="25" t="inlineStr">
@@ -1209,7 +1209,7 @@
       </c>
       <c r="L3" s="25" t="inlineStr">
         <is>
-          <t>Suite a votre article de 2026 sur l'asclepiade</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="M3" s="25" t="inlineStr">
@@ -1281,7 +1281,7 @@
       </c>
       <c r="L4" s="25" t="inlineStr">
         <is>
-          <t>Suite a votre article de 2025 sur l'asclepiade</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="M4" s="25" t="inlineStr">
@@ -1366,7 +1366,7 @@
       </c>
       <c r="L5" s="25" t="inlineStr">
         <is>
-          <t>Invite disponible : Lasclay a Dragons' Den le 17 septembre</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
         </is>
       </c>
       <c r="M5" s="25" t="inlineStr">
@@ -1437,7 +1437,7 @@
       </c>
       <c r="L6" s="25" t="inlineStr">
         <is>
-          <t>Suite a votre article de 2025 sur l'asclepiade</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="M6" s="25" t="inlineStr">
@@ -1509,7 +1509,7 @@
       </c>
       <c r="L7" s="25" t="inlineStr">
         <is>
-          <t>Suite a votre article de 2024 sur l'asclepiade</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="M7" s="25" t="inlineStr">
@@ -1581,7 +1581,7 @@
       </c>
       <c r="L8" s="25" t="inlineStr">
         <is>
-          <t>Suite a votre article de 2023 sur l'asclepiade</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="M8" s="25" t="inlineStr">
@@ -1653,7 +1653,7 @@
       </c>
       <c r="L9" s="25" t="inlineStr">
         <is>
-          <t>Invite disponible : Lasclay a Dragons' Den le 17 septembre</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
         </is>
       </c>
       <c r="M9" s="25" t="inlineStr">
@@ -1725,7 +1725,7 @@
       </c>
       <c r="L10" s="25" t="inlineStr">
         <is>
-          <t>Suite a votre article de 2023 sur l'asclepiade</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="M10" s="25" t="inlineStr">
@@ -1797,7 +1797,7 @@
       </c>
       <c r="L11" s="25" t="inlineStr">
         <is>
-          <t>Suite a votre article de 2023 sur l'asclepiade</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="M11" s="25" t="inlineStr">
@@ -1869,7 +1869,7 @@
       </c>
       <c r="L12" s="25" t="inlineStr">
         <is>
-          <t>Suite a votre article de 2023 sur l'asclepiade</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="M12" s="25" t="inlineStr">
@@ -1941,7 +1941,7 @@
       </c>
       <c r="L13" s="25" t="inlineStr">
         <is>
-          <t>Suite a votre article de 2022 sur l'asclepiade</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="M13" s="25" t="inlineStr">
@@ -2013,7 +2013,7 @@
       </c>
       <c r="L14" s="25" t="inlineStr">
         <is>
-          <t>Suite a votre article de 2022 sur l'asclepiade</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="M14" s="25" t="inlineStr">
@@ -2085,7 +2085,7 @@
       </c>
       <c r="L15" s="25" t="inlineStr">
         <is>
-          <t>Suite a votre article de 2022 sur l'asclepiade</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="M15" s="25" t="inlineStr">
@@ -2157,7 +2157,7 @@
       </c>
       <c r="L16" s="25" t="inlineStr">
         <is>
-          <t>Invite disponible : Lasclay a Dragons' Den le 17 septembre</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
         </is>
       </c>
       <c r="M16" s="25" t="inlineStr">
@@ -2228,7 +2228,7 @@
       </c>
       <c r="L17" s="25" t="inlineStr">
         <is>
-          <t>Suite a votre article de 2022 sur l'asclepiade</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="M17" s="25" t="inlineStr">
@@ -2300,7 +2300,7 @@
       </c>
       <c r="L18" s="25" t="inlineStr">
         <is>
-          <t>Suite a votre article de 2021 sur l'asclepiade</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="M18" s="25" t="inlineStr">
@@ -2372,7 +2372,7 @@
       </c>
       <c r="L19" s="25" t="inlineStr">
         <is>
-          <t>Suite a votre article de 2021 sur l'asclepiade</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="M19" s="25" t="inlineStr">
@@ -2444,7 +2444,7 @@
       </c>
       <c r="L20" s="25" t="inlineStr">
         <is>
-          <t>Suite a votre article de 2021 sur l'asclepiade</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="M20" s="25" t="inlineStr">
@@ -2516,7 +2516,7 @@
       </c>
       <c r="L21" s="25" t="inlineStr">
         <is>
-          <t>Suite a votre article de 2021 sur l'asclepiade</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="M21" s="25" t="inlineStr">
@@ -2588,7 +2588,7 @@
       </c>
       <c r="L22" s="25" t="inlineStr">
         <is>
-          <t>Suite a votre article de 2021 sur l'asclepiade</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="M22" s="25" t="inlineStr">
@@ -2660,7 +2660,7 @@
       </c>
       <c r="L23" s="25" t="inlineStr">
         <is>
-          <t>Suite a votre article de 2021 sur l'asclepiade</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="M23" s="25" t="inlineStr">
@@ -2732,7 +2732,7 @@
       </c>
       <c r="L24" s="25" t="inlineStr">
         <is>
-          <t>Suite a votre article de 2021 sur l'asclepiade</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="M24" s="25" t="inlineStr">
@@ -2804,7 +2804,7 @@
       </c>
       <c r="L25" s="25" t="inlineStr">
         <is>
-          <t>Suite a votre article de 2021 sur l'asclepiade</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="M25" s="25" t="inlineStr">
@@ -2876,7 +2876,7 @@
       </c>
       <c r="L26" s="25" t="inlineStr">
         <is>
-          <t>Suite a votre article de 2020 sur l'asclepiade</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M26" s="25" t="inlineStr">
@@ -2941,7 +2941,7 @@
       </c>
       <c r="L27" s="25" t="inlineStr">
         <is>
-          <t>Suite a votre article de 2020 sur l'asclepiade</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="M27" s="25" t="inlineStr">
@@ -3005,7 +3005,7 @@
       </c>
       <c r="L28" s="25" t="inlineStr">
         <is>
-          <t>Suite a votre article de [année] sur l'asclepiade</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="M28" s="25" t="inlineStr">
@@ -3069,7 +3069,7 @@
       </c>
       <c r="L29" s="25" t="inlineStr">
         <is>
-          <t>Suite a votre article de [année] sur l'asclepiade</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="M29" s="25" t="inlineStr">
@@ -3133,7 +3133,7 @@
       </c>
       <c r="L30" s="25" t="inlineStr">
         <is>
-          <t>Suite a votre article de [année] sur l'asclepiade</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="M30" s="25" t="inlineStr">
@@ -3209,7 +3209,7 @@
       </c>
       <c r="L31" s="25" t="inlineStr">
         <is>
-          <t>Suite a votre article de 2021 sur les ecouteurs de Quebec</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="M31" s="25" t="inlineStr">
@@ -3273,7 +3273,7 @@
       </c>
       <c r="L32" s="25" t="inlineStr">
         <is>
-          <t>Suite a votre article de [année] sur l'asclepiade</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="M32" s="25" t="inlineStr">
@@ -3337,7 +3337,7 @@
       </c>
       <c r="L33" s="25" t="inlineStr">
         <is>
-          <t>Suite a votre article de [année] sur l'asclepiade</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="M33" s="25" t="inlineStr">
@@ -3401,7 +3401,7 @@
       </c>
       <c r="L34" s="25" t="inlineStr">
         <is>
-          <t>Suite a votre article de [année] sur l'asclepiade</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="M34" s="25" t="inlineStr">
@@ -3465,7 +3465,7 @@
       </c>
       <c r="L35" s="25" t="inlineStr">
         <is>
-          <t>Suite a votre article de [année] sur l'asclepiade</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="M35" s="25" t="inlineStr">
@@ -3535,7 +3535,7 @@
       </c>
       <c r="L36" s="25" t="inlineStr">
         <is>
-          <t>Suite a votre article de 2020 sur l'asclepiade</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="M36" s="25" t="inlineStr">
@@ -3605,7 +3605,7 @@
       </c>
       <c r="L37" s="25" t="inlineStr">
         <is>
-          <t>Suite a votre article de 2021 sur l'asclepiade</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="M37" s="25" t="inlineStr">
@@ -3675,7 +3675,7 @@
       </c>
       <c r="L38" s="25" t="inlineStr">
         <is>
-          <t>Suite a votre article de 2023 sur l'asclepiade</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="M38" s="25" t="inlineStr">
@@ -3894,7 +3894,7 @@
       </c>
       <c r="P2" s="25" t="inlineStr">
         <is>
-          <t>L'asclepiade, huit ans apres l'effondrement de la filiere</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q2" s="25" t="inlineStr">
@@ -3981,7 +3981,7 @@
       </c>
       <c r="P3" s="25" t="inlineStr">
         <is>
-          <t>L'asclepiade, huit ans apres l'effondrement de la filiere</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q3" s="25" t="inlineStr">
@@ -4067,7 +4067,7 @@
       </c>
       <c r="P4" s="25" t="inlineStr">
         <is>
-          <t>Un manteau isole avec une mauvaise herbe, au premier episode de Dragons' Den</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q4" s="25" t="inlineStr">
@@ -4157,7 +4157,7 @@
       </c>
       <c r="P5" s="25" t="inlineStr">
         <is>
-          <t>Capitale-Nationale/Chaudière-Appalaches : Lasclay au premier episode de la 21e saison de Dragons' Den</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q5" s="25" t="inlineStr">
@@ -4242,7 +4242,7 @@
       </c>
       <c r="P6" s="25" t="inlineStr">
         <is>
-          <t>L'asclepiade, huit ans apres l'effondrement de la filiere</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q6" s="25" t="inlineStr">
@@ -4328,7 +4328,7 @@
       </c>
       <c r="P7" s="25" t="inlineStr">
         <is>
-          <t>Capitale-Nationale/Chaudière-Appalaches : Lasclay au premier episode de la 21e saison de Dragons' Den</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q7" s="25" t="inlineStr">
@@ -4414,7 +4414,7 @@
       </c>
       <c r="P8" s="25" t="inlineStr">
         <is>
-          <t>Une PME qui a rapatrie sa production, puis en a delocalise une partie</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q8" s="25" t="inlineStr">
@@ -4504,7 +4504,7 @@
       </c>
       <c r="P9" s="25" t="inlineStr">
         <is>
-          <t>Le monarque, l'asclepiade, et l'idee qu'il faut la rendre payante</t>
+          <t>L'asclépiade et les monarques à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q9" s="25" t="inlineStr">
@@ -4594,7 +4594,7 @@
       </c>
       <c r="P10" s="25" t="inlineStr">
         <is>
-          <t>Capitale-Nationale/Chaudière-Appalaches : Lasclay au premier episode de la 21e saison de Dragons' Den</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q10" s="25" t="inlineStr">
@@ -4679,7 +4679,7 @@
       </c>
       <c r="P11" s="25" t="inlineStr">
         <is>
-          <t>Invite disponible : Lasclay a Dragons' Den le 17 septembre</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
         </is>
       </c>
       <c r="Q11" s="25" t="inlineStr">
@@ -4769,7 +4769,7 @@
       </c>
       <c r="P12" s="25" t="inlineStr">
         <is>
-          <t>Capitale-Nationale/Chaudière-Appalaches : Lasclay au premier episode de la 21e saison de Dragons' Den</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q12" s="25" t="inlineStr">
@@ -4850,7 +4850,7 @@
       </c>
       <c r="P13" s="25" t="inlineStr">
         <is>
-          <t>L'asclepiade contre le duvet, et ce que les tests disent vraiment</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q13" s="25" t="inlineStr">
@@ -4936,7 +4936,7 @@
       </c>
       <c r="P14" s="25" t="inlineStr">
         <is>
-          <t>Montérégie : Lasclay au premier episode de la 21e saison de Dragons' Den</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q14" s="25" t="inlineStr">
@@ -5026,7 +5026,7 @@
       </c>
       <c r="P15" s="25" t="inlineStr">
         <is>
-          <t>L'asclepiade, huit ans apres l'effondrement de la filiere</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q15" s="25" t="inlineStr">
@@ -5116,7 +5116,7 @@
       </c>
       <c r="P16" s="25" t="inlineStr">
         <is>
-          <t>L'asclepiade, huit ans apres l'effondrement de la filiere</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q16" s="25" t="inlineStr">
@@ -5202,7 +5202,7 @@
       </c>
       <c r="P17" s="25" t="inlineStr">
         <is>
-          <t>Saguenay - Lac-Saint-Jean : Lasclay au premier episode de la 21e saison de Dragons' Den</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q17" s="25" t="inlineStr">
@@ -5283,7 +5283,7 @@
       </c>
       <c r="P18" s="25" t="inlineStr">
         <is>
-          <t>L'asclepiade contre le duvet, et ce que les tests disent vraiment</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q18" s="25" t="inlineStr">
@@ -5369,7 +5369,7 @@
       </c>
       <c r="P19" s="25" t="inlineStr">
         <is>
-          <t>L'asclepiade, huit ans apres l'effondrement de la filiere</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q19" s="25" t="inlineStr">
@@ -5459,7 +5459,7 @@
       </c>
       <c r="P20" s="25" t="inlineStr">
         <is>
-          <t>Mauricie : Lasclay au premier episode de la 21e saison de Dragons' Den</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q20" s="25" t="inlineStr">
@@ -5545,7 +5545,7 @@
       </c>
       <c r="P21" s="25" t="inlineStr">
         <is>
-          <t>Le monarque, l'asclepiade, et l'idee qu'il faut la rendre payante</t>
+          <t>L'asclépiade et les monarques à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q21" s="25" t="inlineStr">
@@ -5630,7 +5630,7 @@
       </c>
       <c r="P22" s="25" t="inlineStr">
         <is>
-          <t>L'asclepiade, huit ans apres l'effondrement de la filiere</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q22" s="25" t="inlineStr">
@@ -5720,7 +5720,7 @@
       </c>
       <c r="P23" s="25" t="inlineStr">
         <is>
-          <t>Invite disponible : Lasclay a Dragons' Den le 17 septembre</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
         </is>
       </c>
       <c r="Q23" s="25" t="inlineStr">
@@ -5805,7 +5805,7 @@
       </c>
       <c r="P24" s="25" t="inlineStr">
         <is>
-          <t>Laurentides : Lasclay au premier episode de la 21e saison de Dragons' Den</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q24" s="25" t="inlineStr">
@@ -5890,7 +5890,7 @@
       </c>
       <c r="P25" s="25" t="inlineStr">
         <is>
-          <t>L'asclepiade, huit ans apres l'effondrement de la filiere</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q25" s="25" t="inlineStr">
@@ -5971,7 +5971,7 @@
       </c>
       <c r="P26" s="25" t="inlineStr">
         <is>
-          <t>Invite disponible : Lasclay a Dragons' Den le 17 septembre</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
         </is>
       </c>
       <c r="Q26" s="25" t="inlineStr">
@@ -6056,7 +6056,7 @@
       </c>
       <c r="P27" s="25" t="inlineStr">
         <is>
-          <t>Est-du-Québec : Lasclay au premier episode de la 21e saison de Dragons' Den</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q27" s="25" t="inlineStr">
@@ -6141,7 +6141,7 @@
       </c>
       <c r="P28" s="25" t="inlineStr">
         <is>
-          <t>Le monarque, l'asclepiade, et l'idee qu'il faut la rendre payante</t>
+          <t>L'asclépiade et les monarques à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q28" s="25" t="inlineStr">
@@ -6227,7 +6227,7 @@
       </c>
       <c r="P29" s="25" t="inlineStr">
         <is>
-          <t>Invite disponible : Lasclay a Dragons' Den le 17 septembre</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
         </is>
       </c>
       <c r="Q29" s="25" t="inlineStr">
@@ -6317,7 +6317,7 @@
       </c>
       <c r="P30" s="25" t="inlineStr">
         <is>
-          <t>L'asclepiade contre le duvet, et ce que les tests disent vraiment</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q30" s="25" t="inlineStr">
@@ -6407,7 +6407,7 @@
       </c>
       <c r="P31" s="25" t="inlineStr">
         <is>
-          <t>L'asclepiade contre le duvet, et ce que les tests disent vraiment</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q31" s="25" t="inlineStr">
@@ -6497,7 +6497,7 @@
       </c>
       <c r="P32" s="25" t="inlineStr">
         <is>
-          <t>L'asclepiade, huit ans apres l'effondrement de la filiere</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q32" s="25" t="inlineStr">
@@ -6582,7 +6582,7 @@
       </c>
       <c r="P33" s="25" t="inlineStr">
         <is>
-          <t>Invite disponible : Lasclay a Dragons' Den le 17 septembre</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
         </is>
       </c>
       <c r="Q33" s="25" t="inlineStr">
@@ -6667,7 +6667,7 @@
       </c>
       <c r="P34" s="25" t="inlineStr">
         <is>
-          <t>L'asclepiade, huit ans apres l'effondrement de la filiere</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q34" s="25" t="inlineStr">
@@ -6757,7 +6757,7 @@
       </c>
       <c r="P35" s="25" t="inlineStr">
         <is>
-          <t>Le monarque, l'asclepiade, et l'idee qu'il faut la rendre payante</t>
+          <t>L'asclépiade et les monarques à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q35" s="25" t="inlineStr">
@@ -6843,7 +6843,7 @@
       </c>
       <c r="P36" s="25" t="inlineStr">
         <is>
-          <t>L'asclepiade, huit ans apres l'effondrement de la filiere</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q36" s="25" t="inlineStr">
@@ -6924,7 +6924,7 @@
       </c>
       <c r="P37" s="25" t="inlineStr">
         <is>
-          <t>Invite disponible : Lasclay a Dragons' Den le 17 septembre</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
         </is>
       </c>
       <c r="Q37" s="25" t="inlineStr">
@@ -7009,7 +7009,7 @@
       </c>
       <c r="P38" s="25" t="inlineStr">
         <is>
-          <t>L'asclepiade, huit ans apres l'effondrement de la filiere</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q38" s="25" t="inlineStr">
@@ -7095,7 +7095,7 @@
       </c>
       <c r="P39" s="25" t="inlineStr">
         <is>
-          <t>Invite disponible : Lasclay a Dragons' Den le 17 septembre</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
         </is>
       </c>
       <c r="Q39" s="25" t="inlineStr">
@@ -7176,7 +7176,7 @@
       </c>
       <c r="P40" s="25" t="inlineStr">
         <is>
-          <t>Capitale-Nationale/Chaudière-Appalaches : Lasclay au premier episode de la 21e saison de Dragons' Den</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q40" s="25" t="inlineStr">
@@ -7261,7 +7261,7 @@
       </c>
       <c r="P41" s="25" t="inlineStr">
         <is>
-          <t>Une PME qui a rapatrie sa production, puis en a delocalise une partie</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q41" s="25" t="inlineStr">
@@ -7346,7 +7346,7 @@
       </c>
       <c r="P42" s="25" t="inlineStr">
         <is>
-          <t>L'asclepiade contre le duvet, et ce que les tests disent vraiment</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q42" s="25" t="inlineStr">
@@ -7432,7 +7432,7 @@
       </c>
       <c r="P43" s="25" t="inlineStr">
         <is>
-          <t>L'asclepiade contre le duvet, et ce que les tests disent vraiment</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q43" s="25" t="inlineStr">
@@ -7517,7 +7517,7 @@
       </c>
       <c r="P44" s="25" t="inlineStr">
         <is>
-          <t>L'asclepiade, huit ans apres l'effondrement de la filiere</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q44" s="25" t="inlineStr">
@@ -7607,7 +7607,7 @@
       </c>
       <c r="P45" s="25" t="inlineStr">
         <is>
-          <t>L'asclepiade, huit ans apres l'effondrement de la filiere</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q45" s="25" t="inlineStr">
@@ -7699,7 +7699,7 @@
       </c>
       <c r="P46" s="25" t="inlineStr">
         <is>
-          <t>Le monarque, l'asclepiade, et l'idee qu'il faut la rendre payante</t>
+          <t>L'asclépiade et les monarques à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q46" s="25" t="inlineStr">
@@ -7780,7 +7780,7 @@
       </c>
       <c r="P47" s="25" t="inlineStr">
         <is>
-          <t>L'asclepiade, huit ans apres l'effondrement de la filiere</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q47" s="25" t="inlineStr">
@@ -7870,7 +7870,7 @@
       </c>
       <c r="P48" s="25" t="inlineStr">
         <is>
-          <t>L'asclepiade, huit ans apres l'effondrement de la filiere</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q48" s="25" t="inlineStr">
@@ -7955,7 +7955,7 @@
       </c>
       <c r="P49" s="25" t="inlineStr">
         <is>
-          <t>Invite disponible : Lasclay a Dragons' Den le 17 septembre</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
         </is>
       </c>
       <c r="Q49" s="25" t="inlineStr">
@@ -8040,7 +8040,7 @@
       </c>
       <c r="P50" s="25" t="inlineStr">
         <is>
-          <t>L'asclepiade, huit ans apres l'effondrement de la filiere</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q50" s="25" t="inlineStr">
@@ -8130,7 +8130,7 @@
       </c>
       <c r="P51" s="25" t="inlineStr">
         <is>
-          <t>L'asclepiade, huit ans apres l'effondrement de la filiere</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q51" s="25" t="inlineStr">
@@ -8220,7 +8220,7 @@
       </c>
       <c r="P52" s="25" t="inlineStr">
         <is>
-          <t>L'asclepiade, huit ans apres l'effondrement de la filiere</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q52" s="25" t="inlineStr">
@@ -8305,7 +8305,7 @@
       </c>
       <c r="P53" s="25" t="inlineStr">
         <is>
-          <t>Invite disponible : Lasclay a Dragons' Den le 17 septembre</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
         </is>
       </c>
       <c r="Q53" s="25" t="inlineStr">
@@ -8386,7 +8386,7 @@
       </c>
       <c r="P54" s="25" t="inlineStr">
         <is>
-          <t>Capitale-Nationale/Chaudière-Appalaches : Lasclay au premier episode de la 21e saison de Dragons' Den</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q54" s="25" t="inlineStr">
@@ -8471,7 +8471,7 @@
       </c>
       <c r="P55" s="25" t="inlineStr">
         <is>
-          <t>L'asclepiade contre le duvet, et ce que les tests disent vraiment</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q55" s="25" t="inlineStr">
@@ -8561,7 +8561,7 @@
       </c>
       <c r="P56" s="25" t="inlineStr">
         <is>
-          <t>L'asclepiade contre le duvet, et ce que les tests disent vraiment</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q56" s="25" t="inlineStr">
@@ -8646,7 +8646,7 @@
       </c>
       <c r="P57" s="25" t="inlineStr">
         <is>
-          <t>L'asclepiade contre le duvet, et ce que les tests disent vraiment</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q57" s="25" t="inlineStr">
@@ -8736,7 +8736,7 @@
       </c>
       <c r="P58" s="25" t="inlineStr">
         <is>
-          <t>L'asclepiade, huit ans apres l'effondrement de la filiere</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q58" s="25" t="inlineStr">
@@ -8822,7 +8822,7 @@
       </c>
       <c r="P59" s="25" t="inlineStr">
         <is>
-          <t>L'asclepiade, huit ans apres l'effondrement de la filiere</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q59" s="25" t="inlineStr">
@@ -8912,7 +8912,7 @@
       </c>
       <c r="P60" s="25" t="inlineStr">
         <is>
-          <t>Le monarque, l'asclepiade, et l'idee qu'il faut la rendre payante</t>
+          <t>L'asclépiade et les monarques à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q60" s="25" t="inlineStr">
@@ -9002,7 +9002,7 @@
       </c>
       <c r="P61" s="25" t="inlineStr">
         <is>
-          <t>L'asclepiade contre le duvet, et ce que les tests disent vraiment</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q61" s="25" t="inlineStr">
@@ -9092,7 +9092,7 @@
       </c>
       <c r="P62" s="25" t="inlineStr">
         <is>
-          <t>L'asclepiade, huit ans apres l'effondrement de la filiere</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q62" s="25" t="inlineStr">
@@ -9177,7 +9177,7 @@
       </c>
       <c r="P63" s="25" t="inlineStr">
         <is>
-          <t>Laurentides : Lasclay au premier episode de la 21e saison de Dragons' Den</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q63" s="25" t="inlineStr">
@@ -9262,7 +9262,7 @@
       </c>
       <c r="P64" s="25" t="inlineStr">
         <is>
-          <t>Capitale-Nationale/Chaudière-Appalaches : Lasclay au premier episode de la 21e saison de Dragons' Den</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q64" s="25" t="inlineStr">
@@ -9347,7 +9347,7 @@
       </c>
       <c r="P65" s="25" t="inlineStr">
         <is>
-          <t>L'asclepiade contre le duvet, et ce que les tests disent vraiment</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q65" s="25" t="inlineStr">
@@ -9432,7 +9432,7 @@
       </c>
       <c r="P66" s="25" t="inlineStr">
         <is>
-          <t>L'asclepiade contre le duvet, et ce que les tests disent vraiment</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q66" s="25" t="inlineStr">
@@ -9522,7 +9522,7 @@
       </c>
       <c r="P67" s="25" t="inlineStr">
         <is>
-          <t>L'asclepiade, huit ans apres l'effondrement de la filiere</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q67" s="25" t="inlineStr">
@@ -9612,7 +9612,7 @@
       </c>
       <c r="P68" s="25" t="inlineStr">
         <is>
-          <t>L'asclepiade, huit ans apres l'effondrement de la filiere</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q68" s="25" t="inlineStr">
@@ -9702,7 +9702,7 @@
       </c>
       <c r="P69" s="25" t="inlineStr">
         <is>
-          <t>Invite disponible : Lasclay a Dragons' Den le 17 septembre</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
         </is>
       </c>
       <c r="Q69" s="25" t="inlineStr">
@@ -9792,7 +9792,7 @@
       </c>
       <c r="P70" s="25" t="inlineStr">
         <is>
-          <t>Estrie : Lasclay au premier episode de la 21e saison de Dragons' Den</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q70" s="25" t="inlineStr">
@@ -9873,7 +9873,7 @@
       </c>
       <c r="P71" s="25" t="inlineStr">
         <is>
-          <t>Le monarque, l'asclepiade, et l'idee qu'il faut la rendre payante</t>
+          <t>L'asclépiade et les monarques à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q71" s="25" t="inlineStr">
@@ -9963,7 +9963,7 @@
       </c>
       <c r="P72" s="25" t="inlineStr">
         <is>
-          <t>L'asclepiade contre le duvet, et ce que les tests disent vraiment</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q72" s="25" t="inlineStr">
@@ -10049,7 +10049,7 @@
       </c>
       <c r="P73" s="25" t="inlineStr">
         <is>
-          <t>Un manteau isole avec une mauvaise herbe, au premier episode de Dragons' Den</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q73" s="25" t="inlineStr">
@@ -10139,7 +10139,7 @@
       </c>
       <c r="P74" s="25" t="inlineStr">
         <is>
-          <t>Le monarque, l'asclepiade, et l'idee qu'il faut la rendre payante</t>
+          <t>L'asclépiade et les monarques à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q74" s="25" t="inlineStr">
@@ -10224,7 +10224,7 @@
       </c>
       <c r="P75" s="25" t="inlineStr">
         <is>
-          <t>L'asclepiade, huit ans apres l'effondrement de la filiere</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q75" s="25" t="inlineStr">
@@ -10310,7 +10310,7 @@
       </c>
       <c r="P76" s="25" t="inlineStr">
         <is>
-          <t>Le monarque, l'asclepiade, et l'idee qu'il faut la rendre payante</t>
+          <t>L'asclépiade et les monarques à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q76" s="25" t="inlineStr">
@@ -10396,7 +10396,7 @@
       </c>
       <c r="P77" s="25" t="inlineStr">
         <is>
-          <t>Le monarque, l'asclepiade, et l'idee qu'il faut la rendre payante</t>
+          <t>L'asclépiade et les monarques à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q77" s="25" t="inlineStr">
@@ -10481,7 +10481,7 @@
       </c>
       <c r="P78" s="25" t="inlineStr">
         <is>
-          <t>Le monarque, l'asclepiade, et l'idee qu'il faut la rendre payante</t>
+          <t>L'asclépiade et les monarques à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q78" s="25" t="inlineStr">
@@ -10567,7 +10567,7 @@
       </c>
       <c r="P79" s="25" t="inlineStr">
         <is>
-          <t>Invite disponible : Lasclay a Dragons' Den le 17 septembre</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
         </is>
       </c>
       <c r="Q79" s="25" t="inlineStr">
@@ -10652,7 +10652,7 @@
       </c>
       <c r="P80" s="25" t="inlineStr">
         <is>
-          <t>Invite disponible : Lasclay a Dragons' Den le 17 septembre</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
         </is>
       </c>
       <c r="Q80" s="25" t="inlineStr">
@@ -10737,7 +10737,7 @@
       </c>
       <c r="P81" s="25" t="inlineStr">
         <is>
-          <t>L'asclepiade, huit ans apres l'effondrement de la filiere</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q81" s="25" t="inlineStr">
@@ -10827,7 +10827,7 @@
       </c>
       <c r="P82" s="25" t="inlineStr">
         <is>
-          <t>L'asclepiade, huit ans apres l'effondrement de la filiere</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q82" s="25" t="inlineStr">
@@ -10912,7 +10912,7 @@
       </c>
       <c r="P83" s="25" t="inlineStr">
         <is>
-          <t>Canada anglais : Lasclay au premier episode de la 21e saison de Dragons' Den</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q83" s="25" t="inlineStr">
@@ -10997,7 +10997,7 @@
       </c>
       <c r="P84" s="25" t="inlineStr">
         <is>
-          <t>Le monarque, l'asclepiade, et l'idee qu'il faut la rendre payante</t>
+          <t>L'asclépiade et les monarques à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q84" s="25" t="inlineStr">
@@ -11082,7 +11082,7 @@
       </c>
       <c r="P85" s="25" t="inlineStr">
         <is>
-          <t>L'asclepiade, huit ans apres l'effondrement de la filiere</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q85" s="25" t="inlineStr">
@@ -11167,7 +11167,7 @@
       </c>
       <c r="P86" s="25" t="inlineStr">
         <is>
-          <t>Le monarque, l'asclepiade, et l'idee qu'il faut la rendre payante</t>
+          <t>L'asclépiade et les monarques à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q86" s="25" t="inlineStr">
@@ -11252,7 +11252,7 @@
       </c>
       <c r="P87" s="25" t="inlineStr">
         <is>
-          <t>Le monarque, l'asclepiade, et l'idee qu'il faut la rendre payante</t>
+          <t>L'asclépiade et les monarques à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q87" s="25" t="inlineStr">
@@ -11333,7 +11333,7 @@
       </c>
       <c r="P88" s="25" t="inlineStr">
         <is>
-          <t>Le monarque, l'asclepiade, et l'idee qu'il faut la rendre payante</t>
+          <t>L'asclépiade et les monarques à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q88" s="25" t="inlineStr">
@@ -11418,7 +11418,7 @@
       </c>
       <c r="P89" s="25" t="inlineStr">
         <is>
-          <t>Est-du-Québec : Lasclay au premier episode de la 21e saison de Dragons' Den</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q89" s="25" t="inlineStr">
@@ -11499,7 +11499,7 @@
       </c>
       <c r="P90" s="25" t="inlineStr">
         <is>
-          <t>Le monarque, l'asclepiade, et l'idee qu'il faut la rendre payante</t>
+          <t>L'asclépiade et les monarques à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q90" s="25" t="inlineStr">
@@ -11585,7 +11585,7 @@
       </c>
       <c r="P91" s="25" t="inlineStr">
         <is>
-          <t>Montérégie : Lasclay au premier episode de la 21e saison de Dragons' Den</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q91" s="25" t="inlineStr">
@@ -11670,7 +11670,7 @@
       </c>
       <c r="P92" s="25" t="inlineStr">
         <is>
-          <t>Le monarque, l'asclepiade, et l'idee qu'il faut la rendre payante</t>
+          <t>L'asclépiade et les monarques à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q92" s="25" t="inlineStr">
@@ -11760,7 +11760,7 @@
       </c>
       <c r="P93" s="25" t="inlineStr">
         <is>
-          <t>L'asclepiade, huit ans apres l'effondrement de la filiere</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q93" s="25" t="inlineStr">
@@ -11845,7 +11845,7 @@
       </c>
       <c r="P94" s="25" t="inlineStr">
         <is>
-          <t>Laurentides : Lasclay au premier episode de la 21e saison de Dragons' Den</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q94" s="25" t="inlineStr">
@@ -11930,7 +11930,7 @@
       </c>
       <c r="P95" s="25" t="inlineStr">
         <is>
-          <t>Une PME qui a rapatrie sa production, puis en a delocalise une partie</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q95" s="25" t="inlineStr">
@@ -12015,7 +12015,7 @@
       </c>
       <c r="P96" s="25" t="inlineStr">
         <is>
-          <t>Montérégie : Lasclay au premier episode de la 21e saison de Dragons' Den</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q96" s="25" t="inlineStr">
@@ -12105,7 +12105,7 @@
       </c>
       <c r="P97" s="25" t="inlineStr">
         <is>
-          <t>Une PME qui a rapatrie sa production, puis en a delocalise une partie</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q97" s="25" t="inlineStr">
@@ -12190,7 +12190,7 @@
       </c>
       <c r="P98" s="25" t="inlineStr">
         <is>
-          <t>Invite disponible : Lasclay a Dragons' Den le 17 septembre</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
         </is>
       </c>
       <c r="Q98" s="25" t="inlineStr">
@@ -12280,7 +12280,7 @@
       </c>
       <c r="P99" s="25" t="inlineStr">
         <is>
-          <t>L'asclepiade, huit ans apres l'effondrement de la filiere</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q99" s="25" t="inlineStr">
@@ -12365,7 +12365,7 @@
       </c>
       <c r="P100" s="25" t="inlineStr">
         <is>
-          <t>L'asclepiade contre le duvet, et ce que les tests disent vraiment</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q100" s="25" t="inlineStr">
@@ -12455,7 +12455,7 @@
       </c>
       <c r="P101" s="25" t="inlineStr">
         <is>
-          <t>Une PME qui a rapatrie sa production, puis en a delocalise une partie</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q101" s="25" t="inlineStr">
@@ -12540,7 +12540,7 @@
       </c>
       <c r="P102" s="25" t="inlineStr">
         <is>
-          <t>Le monarque, l'asclepiade, et l'idee qu'il faut la rendre payante</t>
+          <t>L'asclépiade et les monarques à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q102" s="25" t="inlineStr">
@@ -12621,7 +12621,7 @@
       </c>
       <c r="P103" s="25" t="inlineStr">
         <is>
-          <t>Le monarque, l'asclepiade, et l'idee qu'il faut la rendre payante</t>
+          <t>L'asclépiade et les monarques à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q103" s="25" t="inlineStr">
@@ -12706,7 +12706,7 @@
       </c>
       <c r="P104" s="25" t="inlineStr">
         <is>
-          <t>Mauricie : Lasclay au premier episode de la 21e saison de Dragons' Den</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q104" s="25" t="inlineStr">
@@ -12791,7 +12791,7 @@
       </c>
       <c r="P105" s="25" t="inlineStr">
         <is>
-          <t>L'asclepiade contre le duvet, et ce que les tests disent vraiment</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q105" s="25" t="inlineStr">
@@ -12876,7 +12876,7 @@
       </c>
       <c r="P106" s="25" t="inlineStr">
         <is>
-          <t>Une PME qui a rapatrie sa production, puis en a delocalise une partie</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q106" s="25" t="inlineStr">
@@ -12961,7 +12961,7 @@
       </c>
       <c r="P107" s="25" t="inlineStr">
         <is>
-          <t>L'asclepiade contre le duvet, et ce que les tests disent vraiment</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q107" s="25" t="inlineStr">
@@ -13051,7 +13051,7 @@
       </c>
       <c r="P108" s="25" t="inlineStr">
         <is>
-          <t>Une PME qui a rapatrie sa production, puis en a delocalise une partie</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q108" s="25" t="inlineStr">
@@ -13136,7 +13136,7 @@
       </c>
       <c r="P109" s="25" t="inlineStr">
         <is>
-          <t>Montérégie : Lasclay au premier episode de la 21e saison de Dragons' Den</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q109" s="25" t="inlineStr">
@@ -13221,7 +13221,7 @@
       </c>
       <c r="P110" s="25" t="inlineStr">
         <is>
-          <t>Invite disponible : Lasclay a Dragons' Den le 17 septembre</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
         </is>
       </c>
       <c r="Q110" s="25" t="inlineStr">
@@ -13311,7 +13311,7 @@
       </c>
       <c r="P111" s="25" t="inlineStr">
         <is>
-          <t>L'asclepiade, huit ans apres l'effondrement de la filiere</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q111" s="25" t="inlineStr">
@@ -13396,7 +13396,7 @@
       </c>
       <c r="P112" s="25" t="inlineStr">
         <is>
-          <t>Laurentides : Lasclay au premier episode de la 21e saison de Dragons' Den</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q112" s="25" t="inlineStr">
@@ -13477,7 +13477,7 @@
       </c>
       <c r="P113" s="25" t="inlineStr">
         <is>
-          <t>L'asclepiade contre le duvet, et ce que les tests disent vraiment</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q113" s="25" t="inlineStr">
@@ -13567,7 +13567,7 @@
       </c>
       <c r="P114" s="25" t="inlineStr">
         <is>
-          <t>Est-du-Québec : Lasclay au premier episode de la 21e saison de Dragons' Den</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q114" s="25" t="inlineStr">
@@ -13652,7 +13652,7 @@
       </c>
       <c r="P115" s="25" t="inlineStr">
         <is>
-          <t>Montérégie : Lasclay au premier episode de la 21e saison de Dragons' Den</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q115" s="25" t="inlineStr">
@@ -13737,7 +13737,7 @@
       </c>
       <c r="P116" s="25" t="inlineStr">
         <is>
-          <t>Invite disponible : Lasclay a Dragons' Den le 17 septembre</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
         </is>
       </c>
       <c r="Q116" s="25" t="inlineStr">
@@ -13827,7 +13827,7 @@
       </c>
       <c r="P117" s="25" t="inlineStr">
         <is>
-          <t>Le monarque, l'asclepiade, et l'idee qu'il faut la rendre payante</t>
+          <t>L'asclépiade et les monarques à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q117" s="25" t="inlineStr">
@@ -13908,7 +13908,7 @@
       </c>
       <c r="P118" s="25" t="inlineStr">
         <is>
-          <t>Le monarque, l'asclepiade, et l'idee qu'il faut la rendre payante</t>
+          <t>L'asclépiade et les monarques à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q118" s="25" t="inlineStr">
@@ -13989,7 +13989,7 @@
       </c>
       <c r="P119" s="25" t="inlineStr">
         <is>
-          <t>Le monarque, l'asclepiade, et l'idee qu'il faut la rendre payante</t>
+          <t>L'asclépiade et les monarques à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q119" s="25" t="inlineStr">
@@ -14070,7 +14070,7 @@
       </c>
       <c r="P120" s="25" t="inlineStr">
         <is>
-          <t>Le monarque, l'asclepiade, et l'idee qu'il faut la rendre payante</t>
+          <t>L'asclépiade et les monarques à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q120" s="25" t="inlineStr">
@@ -14151,7 +14151,7 @@
       </c>
       <c r="P121" s="25" t="inlineStr">
         <is>
-          <t>L'asclepiade, huit ans apres l'effondrement de la filiere</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q121" s="25" t="inlineStr">
@@ -14232,7 +14232,7 @@
       </c>
       <c r="P122" s="25" t="inlineStr">
         <is>
-          <t>Une PME qui a rapatrie sa production, puis en a delocalise une partie</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q122" s="25" t="inlineStr">
@@ -14317,7 +14317,7 @@
       </c>
       <c r="P123" s="25" t="inlineStr">
         <is>
-          <t>L'asclepiade contre le duvet, et ce que les tests disent vraiment</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q123" s="25" t="inlineStr">
@@ -14407,7 +14407,7 @@
       </c>
       <c r="P124" s="25" t="inlineStr">
         <is>
-          <t>Une PME qui a rapatrie sa production, puis en a delocalise une partie</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q124" s="25" t="inlineStr">
@@ -14488,7 +14488,7 @@
       </c>
       <c r="P125" s="25" t="inlineStr">
         <is>
-          <t>Le monarque, l'asclepiade, et l'idee qu'il faut la rendre payante</t>
+          <t>L'asclépiade et les monarques à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q125" s="25" t="inlineStr">
@@ -14578,7 +14578,7 @@
       </c>
       <c r="P126" s="25" t="inlineStr">
         <is>
-          <t>Le monarque, l'asclepiade, et l'idee qu'il faut la rendre payante</t>
+          <t>L'asclépiade et les monarques à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q126" s="25" t="inlineStr">
@@ -14663,7 +14663,7 @@
       </c>
       <c r="P127" s="25" t="inlineStr">
         <is>
-          <t>Le monarque, l'asclepiade, et l'idee qu'il faut la rendre payante</t>
+          <t>L'asclépiade et les monarques à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q127" s="25" t="inlineStr">
@@ -14749,7 +14749,7 @@
       </c>
       <c r="P128" s="25" t="inlineStr">
         <is>
-          <t>Une PME qui a rapatrie sa production, puis en a delocalise une partie</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q128" s="25" t="inlineStr">
@@ -14839,7 +14839,7 @@
       </c>
       <c r="P129" s="25" t="inlineStr">
         <is>
-          <t>Le monarque, l'asclepiade, et l'idee qu'il faut la rendre payante</t>
+          <t>L'asclépiade et les monarques à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q129" s="25" t="inlineStr">
@@ -14920,7 +14920,7 @@
       </c>
       <c r="P130" s="25" t="inlineStr">
         <is>
-          <t>Un manteau isole avec une mauvaise herbe, au premier episode de Dragons' Den</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q130" s="25" t="inlineStr">
@@ -15010,7 +15010,7 @@
       </c>
       <c r="P131" s="25" t="inlineStr">
         <is>
-          <t>Une PME qui a rapatrie sa production, puis en a delocalise une partie</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q131" s="25" t="inlineStr">
@@ -15096,7 +15096,7 @@
       </c>
       <c r="P132" s="25" t="inlineStr">
         <is>
-          <t>Invite disponible : Lasclay a Dragons' Den le 17 septembre</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
         </is>
       </c>
       <c r="Q132" s="25" t="inlineStr">
@@ -15186,7 +15186,7 @@
       </c>
       <c r="P133" s="25" t="inlineStr">
         <is>
-          <t>Un manteau isole avec une mauvaise herbe, au premier episode de Dragons' Den</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q133" s="25" t="inlineStr">
@@ -15271,7 +15271,7 @@
       </c>
       <c r="P134" s="25" t="inlineStr">
         <is>
-          <t>Outaouais : Lasclay au premier episode de la 21e saison de Dragons' Den</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q134" s="25" t="inlineStr">
@@ -15356,7 +15356,7 @@
       </c>
       <c r="P135" s="25" t="inlineStr">
         <is>
-          <t>L'asclepiade contre le duvet, et ce que les tests disent vraiment</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q135" s="25" t="inlineStr">
@@ -15446,7 +15446,7 @@
       </c>
       <c r="P136" s="25" t="inlineStr">
         <is>
-          <t>Une PME qui a rapatrie sa production, puis en a delocalise une partie</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q136" s="25" t="inlineStr">
@@ -15536,7 +15536,7 @@
       </c>
       <c r="P137" s="25" t="inlineStr">
         <is>
-          <t>Invite disponible : Lasclay a Dragons' Den le 17 septembre</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
         </is>
       </c>
       <c r="Q137" s="25" t="inlineStr">
@@ -15617,7 +15617,7 @@
       </c>
       <c r="P138" s="25" t="inlineStr">
         <is>
-          <t>Invite disponible : Lasclay a Dragons' Den le 17 septembre</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
         </is>
       </c>
       <c r="Q138" s="25" t="inlineStr">
@@ -15707,7 +15707,7 @@
       </c>
       <c r="P139" s="25" t="inlineStr">
         <is>
-          <t>Un manteau isole avec une mauvaise herbe, au premier episode de Dragons' Den</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q139" s="25" t="inlineStr">
@@ -15788,7 +15788,7 @@
       </c>
       <c r="P140" s="25" t="inlineStr">
         <is>
-          <t>Une PME qui a rapatrie sa production, puis en a delocalise une partie</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q140" s="25" t="inlineStr">
@@ -15878,7 +15878,7 @@
       </c>
       <c r="P141" s="25" t="inlineStr">
         <is>
-          <t>Le monarque, l'asclepiade, et l'idee qu'il faut la rendre payante</t>
+          <t>L'asclépiade et les monarques à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q141" s="25" t="inlineStr">
@@ -15968,7 +15968,7 @@
       </c>
       <c r="P142" s="25" t="inlineStr">
         <is>
-          <t>Invite disponible : Lasclay a Dragons' Den le 17 septembre</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
         </is>
       </c>
       <c r="Q142" s="25" t="inlineStr">
@@ -16053,7 +16053,7 @@
       </c>
       <c r="P143" s="25" t="inlineStr">
         <is>
-          <t>Invite disponible : Lasclay a Dragons' Den le 17 septembre</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
         </is>
       </c>
       <c r="Q143" s="25" t="inlineStr">
@@ -16139,7 +16139,7 @@
       </c>
       <c r="P144" s="25" t="inlineStr">
         <is>
-          <t>Invite disponible : Lasclay a Dragons' Den le 17 septembre</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
         </is>
       </c>
       <c r="Q144" s="25" t="inlineStr">
@@ -16229,7 +16229,7 @@
       </c>
       <c r="P145" s="25" t="inlineStr">
         <is>
-          <t>Le monarque, l'asclepiade, et l'idee qu'il faut la rendre payante</t>
+          <t>L'asclépiade et les monarques à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q145" s="25" t="inlineStr">
@@ -16315,7 +16315,7 @@
       </c>
       <c r="P146" s="25" t="inlineStr">
         <is>
-          <t>Montérégie : Lasclay au premier episode de la 21e saison de Dragons' Den</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q146" s="25" t="inlineStr">
@@ -16405,7 +16405,7 @@
       </c>
       <c r="P147" s="25" t="inlineStr">
         <is>
-          <t>Un manteau isole avec une mauvaise herbe, au premier episode de Dragons' Den</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q147" s="25" t="inlineStr">
@@ -16495,7 +16495,7 @@
       </c>
       <c r="P148" s="25" t="inlineStr">
         <is>
-          <t>Un manteau isole avec une mauvaise herbe, au premier episode de Dragons' Den</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q148" s="25" t="inlineStr">
@@ -16576,7 +16576,7 @@
       </c>
       <c r="P149" s="25" t="inlineStr">
         <is>
-          <t>Le monarque, l'asclepiade, et l'idee qu'il faut la rendre payante</t>
+          <t>L'asclépiade et les monarques à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q149" s="25" t="inlineStr">
@@ -16662,7 +16662,7 @@
       </c>
       <c r="P150" s="25" t="inlineStr">
         <is>
-          <t>L'asclepiade contre le duvet, et ce que les tests disent vraiment</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q150" s="25" t="inlineStr">
@@ -16752,7 +16752,7 @@
       </c>
       <c r="P151" s="25" t="inlineStr">
         <is>
-          <t>Une PME qui a rapatrie sa production, puis en a delocalise une partie</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q151" s="25" t="inlineStr">
@@ -16833,7 +16833,7 @@
       </c>
       <c r="P152" s="25" t="inlineStr">
         <is>
-          <t>Un manteau isole avec une mauvaise herbe, au premier episode de Dragons' Den</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q152" s="25" t="inlineStr">
@@ -16923,7 +16923,7 @@
       </c>
       <c r="P153" s="25" t="inlineStr">
         <is>
-          <t>Estrie : Lasclay au premier episode de la 21e saison de Dragons' Den</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q153" s="25" t="inlineStr">
@@ -17008,7 +17008,7 @@
       </c>
       <c r="P154" s="25" t="inlineStr">
         <is>
-          <t>Une PME qui a rapatrie sa production, puis en a delocalise une partie</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q154" s="25" t="inlineStr">
@@ -17094,7 +17094,7 @@
       </c>
       <c r="P155" s="25" t="inlineStr">
         <is>
-          <t>Le monarque, l'asclepiade, et l'idee qu'il faut la rendre payante</t>
+          <t>L'asclépiade et les monarques à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q155" s="25" t="inlineStr">
@@ -17184,7 +17184,7 @@
       </c>
       <c r="P156" s="25" t="inlineStr">
         <is>
-          <t>Laval : Lasclay au premier episode de la 21e saison de Dragons' Den</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q156" s="25" t="inlineStr">
@@ -17274,7 +17274,7 @@
       </c>
       <c r="P157" s="25" t="inlineStr">
         <is>
-          <t>Invite disponible : Lasclay a Dragons' Den le 17 septembre</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
         </is>
       </c>
       <c r="Q157" s="25" t="inlineStr">
@@ -17355,7 +17355,7 @@
       </c>
       <c r="P158" s="25" t="inlineStr">
         <is>
-          <t>Une PME qui a rapatrie sa production, puis en a delocalise une partie</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q158" s="25" t="inlineStr">
@@ -17445,7 +17445,7 @@
       </c>
       <c r="P159" s="25" t="inlineStr">
         <is>
-          <t>Un manteau isole avec une mauvaise herbe, au premier episode de Dragons' Den</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q159" s="25" t="inlineStr">
@@ -17531,7 +17531,7 @@
       </c>
       <c r="P160" s="25" t="inlineStr">
         <is>
-          <t>Le monarque, l'asclepiade, et l'idee qu'il faut la rendre payante</t>
+          <t>L'asclépiade et les monarques à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q160" s="25" t="inlineStr">
@@ -17621,7 +17621,7 @@
       </c>
       <c r="P161" s="25" t="inlineStr">
         <is>
-          <t>Invite disponible : Lasclay a Dragons' Den le 17 septembre</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
         </is>
       </c>
       <c r="Q161" s="25" t="inlineStr">
@@ -17702,7 +17702,7 @@
       </c>
       <c r="P162" s="25" t="inlineStr">
         <is>
-          <t>Une PME qui a rapatrie sa production, puis en a delocalise une partie</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q162" s="25" t="inlineStr">
@@ -17787,7 +17787,7 @@
       </c>
       <c r="P163" s="25" t="inlineStr">
         <is>
-          <t>Le monarque, l'asclepiade, et l'idee qu'il faut la rendre payante</t>
+          <t>L'asclépiade et les monarques à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q163" s="25" t="inlineStr">
@@ -17868,7 +17868,7 @@
       </c>
       <c r="P164" s="25" t="inlineStr">
         <is>
-          <t>Un manteau isole avec une mauvaise herbe, au premier episode de Dragons' Den</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q164" s="25" t="inlineStr">
@@ -17958,7 +17958,7 @@
       </c>
       <c r="P165" s="25" t="inlineStr">
         <is>
-          <t>Un manteau isole avec une mauvaise herbe, au premier episode de Dragons' Den</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q165" s="25" t="inlineStr">
@@ -18043,7 +18043,7 @@
       </c>
       <c r="P166" s="25" t="inlineStr">
         <is>
-          <t>Une PME qui a rapatrie sa production, puis en a delocalise une partie</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q166" s="25" t="inlineStr">
@@ -18209,7 +18209,7 @@
       </c>
       <c r="P168" s="25" t="inlineStr">
         <is>
-          <t>Le monarque, l'asclepiade, et l'idee qu'il faut la rendre payante</t>
+          <t>L'asclépiade et les monarques à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q168" s="25" t="inlineStr">
@@ -18299,7 +18299,7 @@
       </c>
       <c r="P169" s="25" t="inlineStr">
         <is>
-          <t>Un manteau isole avec une mauvaise herbe, au premier episode de Dragons' Den</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q169" s="25" t="inlineStr">
@@ -18389,7 +18389,7 @@
       </c>
       <c r="P170" s="25" t="inlineStr">
         <is>
-          <t>Une PME qui a rapatrie sa production, puis en a delocalise une partie</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q170" s="25" t="inlineStr">
@@ -18474,7 +18474,7 @@
       </c>
       <c r="P171" s="25" t="inlineStr">
         <is>
-          <t>Invite disponible : Lasclay a Dragons' Den le 17 septembre</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
         </is>
       </c>
       <c r="Q171" s="25" t="inlineStr">
@@ -18564,7 +18564,7 @@
       </c>
       <c r="P172" s="25" t="inlineStr">
         <is>
-          <t>Invite disponible : Lasclay a Dragons' Den le 17 septembre</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
         </is>
       </c>
       <c r="Q172" s="25" t="inlineStr">
@@ -18735,7 +18735,7 @@
       </c>
       <c r="P174" s="25" t="inlineStr">
         <is>
-          <t>Un manteau isole avec une mauvaise herbe, au premier episode de Dragons' Den</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q174" s="25" t="inlineStr">
@@ -18821,7 +18821,7 @@
       </c>
       <c r="P175" s="25" t="inlineStr">
         <is>
-          <t>Le monarque, l'asclepiade, et l'idee qu'il faut la rendre payante</t>
+          <t>L'asclépiade et les monarques à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q175" s="25" t="inlineStr">
@@ -18902,7 +18902,7 @@
       </c>
       <c r="P176" s="25" t="inlineStr">
         <is>
-          <t>Le monarque, l'asclepiade, et l'idee qu'il faut la rendre payante</t>
+          <t>L'asclépiade et les monarques à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q176" s="25" t="inlineStr">
@@ -18992,7 +18992,7 @@
       </c>
       <c r="P177" s="25" t="inlineStr">
         <is>
-          <t>Invite disponible : Lasclay a Dragons' Den le 17 septembre</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
         </is>
       </c>
       <c r="Q177" s="25" t="inlineStr">
@@ -19082,7 +19082,7 @@
       </c>
       <c r="P178" s="25" t="inlineStr">
         <is>
-          <t>Le monarque, l'asclepiade, et l'idee qu'il faut la rendre payante</t>
+          <t>L'asclépiade et les monarques à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q178" s="25" t="inlineStr">
@@ -19167,7 +19167,7 @@
       </c>
       <c r="P179" s="25" t="inlineStr">
         <is>
-          <t>Un manteau isole avec une mauvaise herbe, au premier episode de Dragons' Den</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q179" s="25" t="inlineStr">
@@ -19248,7 +19248,7 @@
       </c>
       <c r="P180" s="25" t="inlineStr">
         <is>
-          <t>Une PME qui a rapatrie sa production, puis en a delocalise une partie</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q180" s="25" t="inlineStr">
@@ -19338,7 +19338,7 @@
       </c>
       <c r="P181" s="25" t="inlineStr">
         <is>
-          <t>Une PME qui a rapatrie sa production, puis en a delocalise une partie</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q181" s="25" t="inlineStr">
@@ -19419,7 +19419,7 @@
       </c>
       <c r="P182" s="25" t="inlineStr">
         <is>
-          <t>Invite disponible : Lasclay a Dragons' Den le 17 septembre</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
         </is>
       </c>
       <c r="Q182" s="25" t="inlineStr">
@@ -19505,7 +19505,7 @@
       </c>
       <c r="P183" s="25" t="inlineStr">
         <is>
-          <t>Invite disponible : Lasclay a Dragons' Den le 17 septembre</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
         </is>
       </c>
       <c r="Q183" s="25" t="inlineStr">
@@ -19595,7 +19595,7 @@
       </c>
       <c r="P184" s="25" t="inlineStr">
         <is>
-          <t>Le monarque, l'asclepiade, et l'idee qu'il faut la rendre payante</t>
+          <t>L'asclépiade et les monarques à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q184" s="25" t="inlineStr">
@@ -19685,7 +19685,7 @@
       </c>
       <c r="P185" s="25" t="inlineStr">
         <is>
-          <t>Un manteau isole avec une mauvaise herbe, au premier episode de Dragons' Den</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q185" s="25" t="inlineStr">
@@ -19770,7 +19770,7 @@
       </c>
       <c r="P186" s="25" t="inlineStr">
         <is>
-          <t>Une PME qui a rapatrie sa production, puis en a delocalise une partie</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q186" s="25" t="inlineStr">
@@ -19860,7 +19860,7 @@
       </c>
       <c r="P187" s="25" t="inlineStr">
         <is>
-          <t>Un manteau isole avec une mauvaise herbe, au premier episode de Dragons' Den</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q187" s="25" t="inlineStr">
@@ -19946,7 +19946,7 @@
       </c>
       <c r="P188" s="25" t="inlineStr">
         <is>
-          <t>Invite disponible : Lasclay a Dragons' Den le 17 septembre</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
         </is>
       </c>
       <c r="Q188" s="25" t="inlineStr">
@@ -20036,7 +20036,7 @@
       </c>
       <c r="P189" s="25" t="inlineStr">
         <is>
-          <t>Montérégie : Lasclay au premier episode de la 21e saison de Dragons' Den</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q189" s="25" t="inlineStr">
@@ -20126,7 +20126,7 @@
       </c>
       <c r="P190" s="25" t="inlineStr">
         <is>
-          <t>Centre-du-Québec : Lasclay au premier episode de la 21e saison de Dragons' Den</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q190" s="25" t="inlineStr">
@@ -20211,7 +20211,7 @@
       </c>
       <c r="P191" s="25" t="inlineStr">
         <is>
-          <t>Un manteau isole avec une mauvaise herbe, au premier episode de Dragons' Den</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q191" s="25" t="inlineStr">
@@ -20296,7 +20296,7 @@
       </c>
       <c r="P192" s="25" t="inlineStr">
         <is>
-          <t>Invite disponible : Lasclay a Dragons' Den le 17 septembre</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
         </is>
       </c>
       <c r="Q192" s="25" t="inlineStr">
@@ -20386,7 +20386,7 @@
       </c>
       <c r="P193" s="25" t="inlineStr">
         <is>
-          <t>Canada anglais : Lasclay au premier episode de la 21e saison de Dragons' Den</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q193" s="25" t="inlineStr">
@@ -20471,7 +20471,7 @@
       </c>
       <c r="P194" s="25" t="inlineStr">
         <is>
-          <t>Invite disponible : Lasclay a Dragons' Den le 17 septembre</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
         </is>
       </c>
       <c r="Q194" s="25" t="inlineStr">
@@ -20561,7 +20561,7 @@
       </c>
       <c r="P195" s="25" t="inlineStr">
         <is>
-          <t>Un manteau isole avec une mauvaise herbe, au premier episode de Dragons' Den</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q195" s="25" t="inlineStr">
@@ -20651,7 +20651,7 @@
       </c>
       <c r="P196" s="25" t="inlineStr">
         <is>
-          <t>Un manteau isole avec une mauvaise herbe, au premier episode de Dragons' Den</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q196" s="25" t="inlineStr">
@@ -20741,7 +20741,7 @@
       </c>
       <c r="P197" s="25" t="inlineStr">
         <is>
-          <t>Un manteau isole avec une mauvaise herbe, au premier episode de Dragons' Den</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q197" s="25" t="inlineStr">
@@ -20826,7 +20826,7 @@
       </c>
       <c r="P198" s="25" t="inlineStr">
         <is>
-          <t>Le monarque, l'asclepiade, et l'idee qu'il faut la rendre payante</t>
+          <t>L'asclépiade et les monarques à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q198" s="25" t="inlineStr">
@@ -20912,7 +20912,7 @@
       </c>
       <c r="P199" s="25" t="inlineStr">
         <is>
-          <t>Invite disponible : Lasclay a Dragons' Den le 17 septembre</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
         </is>
       </c>
       <c r="Q199" s="25" t="inlineStr">
@@ -20997,7 +20997,7 @@
       </c>
       <c r="P200" s="25" t="inlineStr">
         <is>
-          <t>Centre-du-Québec : Lasclay au premier episode de la 21e saison de Dragons' Den</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q200" s="25" t="inlineStr">
@@ -21082,7 +21082,7 @@
       </c>
       <c r="P201" s="25" t="inlineStr">
         <is>
-          <t>Un manteau isole avec une mauvaise herbe, au premier episode de Dragons' Den</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q201" s="25" t="inlineStr">
@@ -21163,7 +21163,7 @@
       </c>
       <c r="P202" s="25" t="inlineStr">
         <is>
-          <t>Une PME qui a rapatrie sa production, puis en a delocalise une partie</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q202" s="25" t="inlineStr">
@@ -21244,7 +21244,7 @@
       </c>
       <c r="P203" s="25" t="inlineStr">
         <is>
-          <t>Lanaudière : Lasclay au premier episode de la 21e saison de Dragons' Den</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q203" s="25" t="inlineStr">
@@ -21329,7 +21329,7 @@
       </c>
       <c r="P204" s="25" t="inlineStr">
         <is>
-          <t>Le monarque, l'asclepiade, et l'idee qu'il faut la rendre payante</t>
+          <t>L'asclépiade et les monarques à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q204" s="25" t="inlineStr">
@@ -21410,7 +21410,7 @@
       </c>
       <c r="P205" s="25" t="inlineStr">
         <is>
-          <t>Le monarque, l'asclepiade, et l'idee qu'il faut la rendre payante</t>
+          <t>L'asclépiade et les monarques à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q205" s="25" t="inlineStr">
@@ -21495,7 +21495,7 @@
       </c>
       <c r="P206" s="25" t="inlineStr">
         <is>
-          <t>Invite disponible : Lasclay a Dragons' Den le 17 septembre</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
         </is>
       </c>
       <c r="Q206" s="25" t="inlineStr">
@@ -21581,7 +21581,7 @@
       </c>
       <c r="P207" s="25" t="inlineStr">
         <is>
-          <t>Une PME qui a rapatrie sa production, puis en a delocalise une partie</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q207" s="25" t="inlineStr">
@@ -21671,7 +21671,7 @@
       </c>
       <c r="P208" s="25" t="inlineStr">
         <is>
-          <t>Une PME qui a rapatrie sa production, puis en a delocalise une partie</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q208" s="25" t="inlineStr">
@@ -21752,7 +21752,7 @@
       </c>
       <c r="P209" s="25" t="inlineStr">
         <is>
-          <t>Le monarque, l'asclepiade, et l'idee qu'il faut la rendre payante</t>
+          <t>L'asclépiade et les monarques à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q209" s="25" t="inlineStr">
@@ -21837,7 +21837,7 @@
       </c>
       <c r="P210" s="25" t="inlineStr">
         <is>
-          <t>Invite disponible : Lasclay a Dragons' Den le 17 septembre</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
         </is>
       </c>
       <c r="Q210" s="25" t="inlineStr">
@@ -21922,7 +21922,7 @@
       </c>
       <c r="P211" s="25" t="inlineStr">
         <is>
-          <t>Une PME qui a rapatrie sa production, puis en a delocalise une partie</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q211" s="25" t="inlineStr">
@@ -22003,7 +22003,7 @@
       </c>
       <c r="P212" s="25" t="inlineStr">
         <is>
-          <t>Invite disponible : Lasclay a Dragons' Den le 17 septembre</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
         </is>
       </c>
       <c r="Q212" s="25" t="inlineStr">
@@ -22093,7 +22093,7 @@
       </c>
       <c r="P213" s="25" t="inlineStr">
         <is>
-          <t>Mauricie : Lasclay au premier episode de la 21e saison de Dragons' Den</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q213" s="25" t="inlineStr">
@@ -22178,7 +22178,7 @@
       </c>
       <c r="P214" s="25" t="inlineStr">
         <is>
-          <t>Invite disponible : Lasclay a Dragons' Den le 17 septembre</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre — invité disponible</t>
         </is>
       </c>
       <c r="Q214" s="25" t="inlineStr">
@@ -22263,7 +22263,7 @@
       </c>
       <c r="P215" s="25" t="inlineStr">
         <is>
-          <t>Le monarque, l'asclepiade, et l'idee qu'il faut la rendre payante</t>
+          <t>L'asclépiade et les monarques à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q215" s="25" t="inlineStr">
@@ -22353,7 +22353,7 @@
       </c>
       <c r="P216" s="25" t="inlineStr">
         <is>
-          <t>Canada anglais : Lasclay au premier episode de la 21e saison de Dragons' Den</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q216" s="25" t="inlineStr">
@@ -22438,7 +22438,7 @@
       </c>
       <c r="P217" s="25" t="inlineStr">
         <is>
-          <t>Le monarque, l'asclepiade, et l'idee qu'il faut la rendre payante</t>
+          <t>L'asclépiade et les monarques à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q217" s="25" t="inlineStr">
@@ -22519,7 +22519,7 @@
       </c>
       <c r="P218" s="25" t="inlineStr">
         <is>
-          <t>Le monarque, l'asclepiade, et l'idee qu'il faut la rendre payante</t>
+          <t>L'asclépiade et les monarques à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q218" s="25" t="inlineStr">
@@ -22595,7 +22595,7 @@
       </c>
       <c r="P219" s="25" t="inlineStr">
         <is>
-          <t>Vous couvrez l'asclepiade depuis 2014. Il y a une suite.</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q219" s="25" t="inlineStr">
@@ -22674,7 +22674,7 @@
       </c>
       <c r="P220" s="25" t="inlineStr">
         <is>
-          <t>Vous couvrez l'asclepiade depuis 2015. Il y a une suite.</t>
+          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="Q220" s="25" t="inlineStr">

</xml_diff>

<commit_message>
Adopte l'ouverture de Gabriel, qui porte tout le pitch d'un coup
« On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on
cultive pour sauvegarder un pollinisateur emblématique et menacé: le papillon
monarque. » Le produit, la plante et la mission dans une seule phrase.

Conséquence: le paragraphe « Mes 2 grandes missions » ne faisait plus que
répéter. Il disparaît de toute la liste froide et des quatre contacts chauds
sans historique, et le courriel raccourcit d'autant.

Corrige aussi un détail botanique: les « petits cochons » sont les gousses, pas
la soie. La phrase le dit maintenant dans le bon ordre, sinon elle est fausse
pour quiconque connaît la plante.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015pjLsGPzf1MX1JC7QiKGGk
</commit_message>
<xml_diff>
--- a/communique-dragons/Lasclay_v2.xlsx
+++ b/communique-dragons/Lasclay_v2.xlsx
@@ -3080,8 +3080,7 @@
       <c r="N29" s="46" t="inlineStr">
         <is>
           <t>Bonjour Mme Roberge,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe : l'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque. Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe, qu'on transforme en isolant à Québec.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part : je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
@@ -3144,8 +3143,7 @@
       <c r="N30" s="46" t="inlineStr">
         <is>
           <t>Bonjour Mme Laforest,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe : l'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque. Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe, qu'on transforme en isolant à Québec.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part : je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
@@ -3412,8 +3410,7 @@
       <c r="N34" s="46" t="inlineStr">
         <is>
           <t>Bonjour Mme Goubau,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe. Vous couvrez le textile et la mode, alors voici une matière que peu de gens ont vue de près : la soie d'asclépiade, une fibre creuse et naturellement hydrophobe attachée aux graines d'une plante que les agriculteurs arrachent de leurs champs depuis 50 ans. On la transforme en isolant, et on en fait des manteaux, des mitaines et des tuques.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque. Vous couvrez le textile et la mode, alors voici une matière que peu de gens ont vue de près : la soie d'asclépiade, une fibre creuse et naturellement hydrophobe attachée aux graines d'une plante que les agriculteurs arrachent de leurs champs depuis 50 ans. On la transforme en isolant, et on en fait des manteaux, des mitaines et des tuques.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet.
@@ -3476,8 +3473,7 @@
       <c r="N35" s="46" t="inlineStr">
         <is>
           <t>Bonjour Mme Dostie,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe : l'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans. La soie attachée à ses graines est creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque. Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe, qu'on transforme en isolant à Québec.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet.
@@ -3905,15 +3901,15 @@
       <c r="S2" s="46" t="inlineStr">
         <is>
           <t>Bonjour Marie Allard,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une
-mauvaise herbe.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une
+mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et
+menacé : le papillon monarque.
 Il y a une belle histoire de sciences dans l'asclépiade. La soie attachée à ses graines n'est
 pas un poil : c'est un tube creux enduit d'une cire hydrophobe, et les fibres portent une
 charge qui les fait se repousser. C'est ce qui forme le parachute autour de la graine, et
 c'est ce qui emprisonne l'air. Chaque follicule en produit plus de 200.
-On en fait de l'isolant pour des manteaux et des mitaines. Mes 2 grandes missions : faire
-connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade, parce
-que c'est la seule plante que leurs chenilles peuvent manger.
+On en fait de l'isolant pour des manteaux et des mitaines. Et c'est la seule plante que les
+chenilles du monarque peuvent manger, ce qui est toute la raison d'être de l'entreprise.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de
@@ -3997,9 +3993,8 @@
       <c r="S3" s="46" t="inlineStr">
         <is>
           <t>Bonjour Zoé Allemand,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -4083,9 +4078,8 @@
       <c r="S4" s="46" t="inlineStr">
         <is>
           <t>Bonjour Victoria Bakos,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -4168,9 +4162,8 @@
       <c r="S5" s="46" t="inlineStr">
         <is>
           <t>Bonjour Marie-Émélie Bernier,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -4258,9 +4251,8 @@
       <c r="S6" s="46" t="inlineStr">
         <is>
           <t>Bonjour Normand Blouin,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -4344,9 +4336,8 @@
       <c r="S7" s="46" t="inlineStr">
         <is>
           <t>Bonjour Louise Bourbonnais,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -4430,9 +4421,8 @@
       <c r="S8" s="46" t="inlineStr">
         <is>
           <t>Bonjour Francois Bourque,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -4520,9 +4510,8 @@
       <c r="S9" s="46" t="inlineStr">
         <is>
           <t>Bonjour Ariane Boyer,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -4605,9 +4594,8 @@
       <c r="S10" s="46" t="inlineStr">
         <is>
           <t>Bonjour Gilbert Bégin,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -4695,9 +4683,8 @@
       <c r="S11" s="46" t="inlineStr">
         <is>
           <t>Bonjour Papa Moussa Camara,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -4780,9 +4767,8 @@
       <c r="S12" s="46" t="inlineStr">
         <is>
           <t>Bonjour Victor Carré,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -4866,9 +4852,8 @@
       <c r="S13" s="46" t="inlineStr">
         <is>
           <t>Bonjour Eric Chabot,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez le plein air. À poids égal, la littérature donne la soie d'asclépiade pour environ 10 % plus isolante que le duvet. C'est un repère de laboratoire, pas une promesse de manteau, et c'est exactement pour ça que je préfère qu'on la teste.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -4952,9 +4937,8 @@
       <c r="S14" s="46" t="inlineStr">
         <is>
           <t>Bonjour Tristan Champagne-Lessard,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -5042,9 +5026,8 @@
       <c r="S15" s="46" t="inlineStr">
         <is>
           <t>Bonjour Jean-Marc Chevalier,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -5132,9 +5115,8 @@
       <c r="S16" s="46" t="inlineStr">
         <is>
           <t>Bonjour Simon Chrétien,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -5213,9 +5195,8 @@
       <c r="S17" s="46" t="inlineStr">
         <is>
           <t>Bonjour Maxime Corneau,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce qu'un de nos fournisseurs d'asclépiade cultive au Lac-Saint-Jean depuis nos tout débuts, et qu'il l'est encore aujourd'hui. La fibre de chez vous se retrouve dans nos produits.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -5299,9 +5280,8 @@
       <c r="S18" s="46" t="inlineStr">
         <is>
           <t>Bonjour Aurélia Crémoux,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez le plein air. À poids égal, la littérature donne la soie d'asclépiade pour environ 10 % plus isolante que le duvet. C'est un repère de laboratoire, pas une promesse de manteau, et c'est exactement pour ça que je préfère qu'on la teste.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -5385,9 +5365,8 @@
       <c r="S19" s="46" t="inlineStr">
         <is>
           <t>Bonjour Catherine Dallaire,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce qu'une des premières usines de transformation de la fibre était à Granby, et que l'Estrie compte encore des producteurs d'asclépiade.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -5470,14 +5449,13 @@
       <c r="S20" s="46" t="inlineStr">
         <is>
           <t>Bonjour Gabriel Delisle,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une
-mauvaise herbe.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une
+mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et
+menacé : le papillon monarque.
 L'asclépiade a été une histoire mauricienne avant d'être la nôtre : l'usine de Saint-Tite
 achetait 90 % des récoltes du Québec. On a démarré après la chute de cette filière, et six ans
 plus tard on achète encore de l'asclépiade québécoise et on la
 transforme nous-mêmes à Québec.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la
-culture de l'asclépiade.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet : huit ans après
@@ -5556,9 +5534,8 @@
       <c r="S21" s="46" t="inlineStr">
         <is>
           <t>Bonjour Anaïs Desjardins,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -5646,9 +5623,8 @@
       <c r="S22" s="46" t="inlineStr">
         <is>
           <t>Bonjour Simon Dominé,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -5731,9 +5707,8 @@
       <c r="S23" s="46" t="inlineStr">
         <is>
           <t>Bonjour Karl-Ivann Dubé,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -5816,9 +5791,8 @@
       <c r="S24" s="46" t="inlineStr">
         <is>
           <t>Bonjour André Fauteux,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -5901,9 +5875,8 @@
       <c r="S25" s="46" t="inlineStr">
         <is>
           <t>Bonjour Myriam Fimbry,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -5982,9 +5955,8 @@
       <c r="S26" s="46" t="inlineStr">
         <is>
           <t>Bonjour Étienne Fortin-Gauthier,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -6067,9 +6039,8 @@
       <c r="S27" s="46" t="inlineStr">
         <is>
           <t>Bonjour Johanne Fournier,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -6157,9 +6128,8 @@
       <c r="S28" s="46" t="inlineStr">
         <is>
           <t>Bonjour Jean Garon,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -6243,9 +6213,8 @@
       <c r="S29" s="46" t="inlineStr">
         <is>
           <t>Bonjour Cécile Gladel,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -6333,9 +6302,8 @@
       <c r="S30" s="46" t="inlineStr">
         <is>
           <t>Bonjour Marieke Glorieux-Stryckman,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez le plein air. À poids égal, la littérature donne la soie d'asclépiade pour environ 10 % plus isolante que le duvet. C'est un repère de laboratoire, pas une promesse de manteau, et c'est exactement pour ça que je préfère qu'on la teste.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -6423,9 +6391,8 @@
       <c r="S31" s="46" t="inlineStr">
         <is>
           <t>Bonjour Maude Goyer,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez le plein air. À poids égal, la littérature donne la soie d'asclépiade pour environ 10 % plus isolante que le duvet. C'est un repère de laboratoire, pas une promesse de manteau, et c'est exactement pour ça que je préfère qu'on la teste.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -6508,9 +6475,8 @@
       <c r="S32" s="46" t="inlineStr">
         <is>
           <t>Bonjour Pauline Gravel,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -6593,9 +6559,8 @@
       <c r="S33" s="46" t="inlineStr">
         <is>
           <t>Bonjour Bernard Hervieux,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -6683,9 +6648,8 @@
       <c r="S34" s="46" t="inlineStr">
         <is>
           <t>Bonjour Leïla Jolin-Dahel,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -6773,9 +6737,8 @@
       <c r="S35" s="46" t="inlineStr">
         <is>
           <t>Bonjour Kodjo Edjinam Nulagnon LOGO,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -6854,9 +6817,8 @@
       <c r="S36" s="46" t="inlineStr">
         <is>
           <t>Bonjour Annie Labrecque,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -6935,9 +6897,8 @@
       <c r="S37" s="46" t="inlineStr">
         <is>
           <t>Bonjour Marianne Lachapelle,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce qu'une des premières usines de transformation de la fibre était à Granby, et que l'Estrie compte encore des producteurs d'asclépiade.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -7025,9 +6986,8 @@
       <c r="S38" s="46" t="inlineStr">
         <is>
           <t>Bonjour Sophie Lachapelle,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -7106,9 +7066,8 @@
       <c r="S39" s="46" t="inlineStr">
         <is>
           <t>Bonjour Alain Laforest,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -7187,9 +7146,8 @@
       <c r="S40" s="46" t="inlineStr">
         <is>
           <t>Bonjour Mikaël Lalancette,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -7272,9 +7230,8 @@
       <c r="S41" s="46" t="inlineStr">
         <is>
           <t>Bonjour Jean-Luc Lavallée,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -7362,9 +7319,8 @@
       <c r="S42" s="46" t="inlineStr">
         <is>
           <t>Bonjour Jean-Francois Leblanc,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez le plein air. À poids égal, la littérature donne la soie d'asclépiade pour environ 10 % plus isolante que le duvet. C'est un repère de laboratoire, pas une promesse de manteau, et c'est exactement pour ça que je préfère qu'on la teste.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -7443,9 +7399,8 @@
       <c r="S43" s="46" t="inlineStr">
         <is>
           <t>Bonjour Julie Leduc,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez le plein air. À poids égal, la littérature donne la soie d'asclépiade pour environ 10 % plus isolante que le duvet. C'est un repère de laboratoire, pas une promesse de manteau, et c'est exactement pour ça que je préfère qu'on la teste.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -7533,9 +7488,8 @@
       <c r="S44" s="46" t="inlineStr">
         <is>
           <t>Bonjour Annie Martin,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -7623,14 +7577,14 @@
       <c r="S45" s="46" t="inlineStr">
         <is>
           <t>Bonjour Réjean Martin,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une
-mauvaise herbe.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une
+mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et
+menacé : le papillon monarque.
 Vous couvrez Mékinac, donc Saint-Tite, donc l'endroit où l'asclépiade a eu son grand moment
 industriel au Québec. L'usine achetait 90 % des récoltes de la province avant que la filière
 se casse en 2018.
 On a démarré après. Six ans plus tard, on achète encore de l'asclépiade québécoise et on la
-transforme nous-mêmes à Québec. Mes 2 grandes missions : faire connaître
-l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+transforme nous-mêmes à Québec.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Je voulais vous en faire part parce que vos lecteurs ont vu la promesse de l'asclépiade de
@@ -7710,9 +7664,8 @@
       <c r="S46" s="46" t="inlineStr">
         <is>
           <t>Bonjour Charles Mathieu,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -7796,9 +7749,8 @@
       <c r="S47" s="46" t="inlineStr">
         <is>
           <t>Bonjour Clara Matthey-Jonais,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -7881,9 +7833,8 @@
       <c r="S48" s="46" t="inlineStr">
         <is>
           <t>Bonjour Valérian Mazataud,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -7966,9 +7917,8 @@
       <c r="S49" s="46" t="inlineStr">
         <is>
           <t>Bonjour Lili Mercure,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -8056,9 +8006,8 @@
       <c r="S50" s="46" t="inlineStr">
         <is>
           <t>Bonjour Nicolas Mesly,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -8146,9 +8095,8 @@
       <c r="S51" s="46" t="inlineStr">
         <is>
           <t>Bonjour Nicolas Michaud,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -8231,9 +8179,8 @@
       <c r="S52" s="46" t="inlineStr">
         <is>
           <t>Bonjour Véronique Morin,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -8316,9 +8263,8 @@
       <c r="S53" s="46" t="inlineStr">
         <is>
           <t>Bonjour Lila Mouch,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -8397,9 +8343,8 @@
       <c r="S54" s="46" t="inlineStr">
         <is>
           <t>Bonjour Olivier Mougeot,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -8487,9 +8432,8 @@
       <c r="S55" s="46" t="inlineStr">
         <is>
           <t>Bonjour Emmanuelle Mozayan-Verschaeve,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez le plein air. À poids égal, la littérature donne la soie d'asclépiade pour environ 10 % plus isolante que le duvet. C'est un repère de laboratoire, pas une promesse de manteau, et c'est exactement pour ça que je préfère qu'on la teste.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -8572,9 +8516,8 @@
       <c r="S56" s="46" t="inlineStr">
         <is>
           <t>Bonjour Jean-Benoît Nadeau,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez le plein air. À poids égal, la littérature donne la soie d'asclépiade pour environ 10 % plus isolante que le duvet. C'est un repère de laboratoire, pas une promesse de manteau, et c'est exactement pour ça que je préfère qu'on la teste.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -8662,9 +8605,8 @@
       <c r="S57" s="46" t="inlineStr">
         <is>
           <t>Bonjour Yves Ouellet,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez le plein air. À poids égal, la littérature donne la soie d'asclépiade pour environ 10 % plus isolante que le duvet. C'est un repère de laboratoire, pas une promesse de manteau, et c'est exactement pour ça que je préfère qu'on la teste.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -8752,9 +8694,8 @@
       <c r="S58" s="46" t="inlineStr">
         <is>
           <t>Bonjour Josée Panet-Raymond,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -8838,9 +8779,8 @@
       <c r="S59" s="46" t="inlineStr">
         <is>
           <t>Bonjour Yannick Patelli,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -8928,9 +8868,8 @@
       <c r="S60" s="46" t="inlineStr">
         <is>
           <t>Bonjour Félix Pedneault,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -9018,9 +8957,8 @@
       <c r="S61" s="46" t="inlineStr">
         <is>
           <t>Bonjour Marie-Eve Poulin,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez le plein air. À poids égal, la littérature donne la soie d'asclépiade pour environ 10 % plus isolante que le duvet. C'est un repère de laboratoire, pas une promesse de manteau, et c'est exactement pour ça que je préfère qu'on la teste.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -9103,9 +9041,8 @@
       <c r="S62" s="46" t="inlineStr">
         <is>
           <t>Bonjour Marie-Hélène Proulx,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -9188,9 +9125,8 @@
       <c r="S63" s="46" t="inlineStr">
         <is>
           <t>Bonjour Jean-Hugues Roy,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -9273,9 +9209,8 @@
       <c r="S64" s="46" t="inlineStr">
         <is>
           <t>Bonjour Martin Roy,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -9358,9 +9293,8 @@
       <c r="S65" s="46" t="inlineStr">
         <is>
           <t>Bonjour Sylvain Sarrazin,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez le plein air. À poids égal, la littérature donne la soie d'asclépiade pour environ 10 % plus isolante que le duvet. C'est un repère de laboratoire, pas une promesse de manteau, et c'est exactement pour ça que je préfère qu'on la teste.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -9448,9 +9382,8 @@
       <c r="S66" s="46" t="inlineStr">
         <is>
           <t>Bonjour Pierre Sormany,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez le plein air. À poids égal, la littérature donne la soie d'asclépiade pour environ 10 % plus isolante que le duvet. C'est un repère de laboratoire, pas une promesse de manteau, et c'est exactement pour ça que je préfère qu'on la teste.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -9538,9 +9471,8 @@
       <c r="S67" s="46" t="inlineStr">
         <is>
           <t>Bonjour Scott Stevenson,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce qu'une des premières usines de transformation de la fibre était à Granby, et que l'Estrie compte encore des producteurs d'asclépiade.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -9628,9 +9560,8 @@
       <c r="S68" s="46" t="inlineStr">
         <is>
           <t>Bonjour Michèle Tanganika,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -9718,9 +9649,8 @@
       <c r="S69" s="46" t="inlineStr">
         <is>
           <t>Bonjour Stephane Tellier,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -9803,9 +9733,8 @@
       <c r="S70" s="46" t="inlineStr">
         <is>
           <t>Bonjour Karine Tremblay,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce qu'une des premières usines de transformation de la fibre était à Granby, et que l'Estrie compte encore des producteurs d'asclépiade.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -9889,9 +9818,8 @@
       <c r="S71" s="46" t="inlineStr">
         <is>
           <t>Bonjour Jean-Francois Venne,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -9979,9 +9907,8 @@
       <c r="S72" s="46" t="inlineStr">
         <is>
           <t>Bonjour Shahram Yazdanpanah,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez le plein air. À poids égal, la littérature donne la soie d'asclépiade pour environ 10 % plus isolante que le duvet. C'est un repère de laboratoire, pas une promesse de manteau, et c'est exactement pour ça que je préfère qu'on la teste.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -10065,9 +9992,8 @@
       <c r="S73" s="46" t="inlineStr">
         <is>
           <t>Bonjour Malika Alaoui,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -10150,9 +10076,8 @@
       <c r="S74" s="46" t="inlineStr">
         <is>
           <t>Bonjour Yahia Arkat,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -10240,9 +10165,8 @@
       <c r="S75" s="46" t="inlineStr">
         <is>
           <t>Bonjour MARC-OLIVIER BISSON,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -10326,9 +10250,8 @@
       <c r="S76" s="46" t="inlineStr">
         <is>
           <t>Bonjour Maïté Belmir,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -10407,9 +10330,8 @@
       <c r="S77" s="46" t="inlineStr">
         <is>
           <t>Bonjour André Bernard,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -10497,9 +10419,8 @@
       <c r="S78" s="46" t="inlineStr">
         <is>
           <t>Bonjour Didier Bert,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -10578,9 +10499,8 @@
       <c r="S79" s="46" t="inlineStr">
         <is>
           <t>Bonjour Sophie-Andrée Blondin,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -10663,9 +10583,8 @@
       <c r="S80" s="46" t="inlineStr">
         <is>
           <t>Bonjour Pierre Brochu,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce qu'une des premières usines de transformation de la fibre était à Granby, et que l'Estrie compte encore des producteurs d'asclépiade.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -10753,9 +10672,8 @@
       <c r="S81" s="46" t="inlineStr">
         <is>
           <t>Bonjour Gilles Bérubé,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -10838,9 +10756,8 @@
       <c r="S82" s="46" t="inlineStr">
         <is>
           <t>Bonjour Daphné Cameron,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -10923,9 +10840,8 @@
       <c r="S83" s="46" t="inlineStr">
         <is>
           <t>Bonjour Godefroy Macaire Chabi,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -11008,9 +10924,8 @@
       <c r="S84" s="46" t="inlineStr">
         <is>
           <t>Bonjour Sara Champagne,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -11093,9 +11008,8 @@
       <c r="S85" s="46" t="inlineStr">
         <is>
           <t>Bonjour Sarah Champagne,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -11178,9 +11092,8 @@
       <c r="S86" s="46" t="inlineStr">
         <is>
           <t>Bonjour Éric-Pierre Champagne,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -11263,9 +11176,8 @@
       <c r="S87" s="46" t="inlineStr">
         <is>
           <t>Bonjour Marine Corniou,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -11344,9 +11256,8 @@
       <c r="S88" s="46" t="inlineStr">
         <is>
           <t>Bonjour Catherine Crépeau,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -11429,9 +11340,8 @@
       <c r="S89" s="46" t="inlineStr">
         <is>
           <t>Bonjour Laurence Dami-Houle,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -11515,9 +11425,8 @@
       <c r="S90" s="46" t="inlineStr">
         <is>
           <t>Bonjour Amélie Daoust-Boisvert,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -11596,9 +11505,8 @@
       <c r="S91" s="46" t="inlineStr">
         <is>
           <t>Bonjour Dominique Degré,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -11686,9 +11594,8 @@
       <c r="S92" s="46" t="inlineStr">
         <is>
           <t>Bonjour Quentin Dufranne,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -11771,9 +11678,8 @@
       <c r="S93" s="46" t="inlineStr">
         <is>
           <t>Bonjour Ève Dumas,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -11856,9 +11762,8 @@
       <c r="S94" s="46" t="inlineStr">
         <is>
           <t>Bonjour Michel Fortier,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -11941,9 +11846,8 @@
       <c r="S95" s="46" t="inlineStr">
         <is>
           <t>Bonjour Marie-Eve Fournier,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -12031,9 +11935,8 @@
       <c r="S96" s="46" t="inlineStr">
         <is>
           <t>Bonjour Raymond Fournier,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -12116,9 +12019,8 @@
       <c r="S97" s="46" t="inlineStr">
         <is>
           <t>Bonjour Marie-Pier Frappier,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -12206,9 +12108,8 @@
       <c r="S98" s="46" t="inlineStr">
         <is>
           <t>Bonjour Marie-Julie Gagnon,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -12291,9 +12192,8 @@
       <c r="S99" s="46" t="inlineStr">
         <is>
           <t>Bonjour Chloé Germain-Thérien,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce que l'asclépiade a eu son grand moment industriel chez vous : l'usine de Saint-Tite achetait 90 % des récoltes du Québec avant que la filière se casse en 2018. Des producteurs de la Mauricie cultivent encore, et on continue d'acheter leur récolte.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -12381,9 +12281,8 @@
       <c r="S100" s="46" t="inlineStr">
         <is>
           <t>Bonjour Charlotte Glorieux,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez le plein air. À poids égal, la littérature donne la soie d'asclépiade pour environ 10 % plus isolante que le duvet. C'est un repère de laboratoire, pas une promesse de manteau, et c'est exactement pour ça que je préfère qu'on la teste.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -12466,9 +12365,8 @@
       <c r="S101" s="46" t="inlineStr">
         <is>
           <t>Bonjour Annie Hudon,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -12551,9 +12449,8 @@
       <c r="S102" s="46" t="inlineStr">
         <is>
           <t>Bonjour Ahmed Kouaou,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -12632,9 +12529,8 @@
       <c r="S103" s="46" t="inlineStr">
         <is>
           <t>Bonjour Tania Krywiak,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -12717,9 +12613,8 @@
       <c r="S104" s="46" t="inlineStr">
         <is>
           <t>Bonjour Jacinthe Lafrance,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce que l'asclépiade a eu son grand moment industriel chez vous : l'usine de Saint-Tite achetait 90 % des récoltes du Québec avant que la filière se casse en 2018. Des producteurs de la Mauricie cultivent encore, et on continue d'acheter leur récolte.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -12802,9 +12697,8 @@
       <c r="S105" s="46" t="inlineStr">
         <is>
           <t>Bonjour Bruno Lamolet,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -12887,9 +12781,8 @@
       <c r="S106" s="46" t="inlineStr">
         <is>
           <t>Bonjour Yvan Lamontagne,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce qu'une des premières usines de transformation de la fibre était à Granby, et que l'Estrie compte encore des producteurs d'asclépiade.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -12977,9 +12870,8 @@
       <c r="S107" s="46" t="inlineStr">
         <is>
           <t>Bonjour Yves Langlois,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce qu'une des premières usines de transformation de la fibre était à Granby, et que l'Estrie compte encore des producteurs d'asclépiade.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -13062,9 +12954,8 @@
       <c r="S108" s="46" t="inlineStr">
         <is>
           <t>Bonjour Anne Marie Lecomte,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -13147,9 +13038,8 @@
       <c r="S109" s="46" t="inlineStr">
         <is>
           <t>Bonjour Stéphanie Mac Farlane,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -13237,9 +13127,8 @@
       <c r="S110" s="46" t="inlineStr">
         <is>
           <t>Bonjour Philippe Marois,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -13322,9 +13211,8 @@
       <c r="S111" s="46" t="inlineStr">
         <is>
           <t>Bonjour Gildas Meneu,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -13407,9 +13295,8 @@
       <c r="S112" s="46" t="inlineStr">
         <is>
           <t>Bonjour Louis-Xavier Michaud,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -13493,9 +13380,8 @@
       <c r="S113" s="46" t="inlineStr">
         <is>
           <t>Bonjour Anne Montplaisir,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez le plein air. À poids égal, la littérature donne la soie d'asclépiade pour environ 10 % plus isolante que le duvet. C'est un repère de laboratoire, pas une promesse de manteau, et c'est exactement pour ça que je préfère qu'on la teste.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -13578,9 +13464,8 @@
       <c r="S114" s="46" t="inlineStr">
         <is>
           <t>Bonjour Karianne Nepton-Philippe,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -13663,9 +13548,8 @@
       <c r="S115" s="46" t="inlineStr">
         <is>
           <t>Bonjour Geneviève Normand,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -13753,9 +13637,8 @@
       <c r="S116" s="46" t="inlineStr">
         <is>
           <t>Bonjour Carole Payer,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce que l'asclépiade se cultive dans votre région depuis la première vague de 2013, et que plusieurs des producteurs qui ont tenu bon nous vendent encore leur récolte.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -13838,9 +13721,8 @@
       <c r="S117" s="46" t="inlineStr">
         <is>
           <t>Bonjour Boris Proulx,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -13919,9 +13801,8 @@
       <c r="S118" s="46" t="inlineStr">
         <is>
           <t>Bonjour Philippe Robitaille-Grou,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -14000,9 +13881,8 @@
       <c r="S119" s="46" t="inlineStr">
         <is>
           <t>Bonjour Gwen Roley,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -14081,9 +13961,8 @@
       <c r="S120" s="46" t="inlineStr">
         <is>
           <t>Bonjour Mathieu-Robert Sauvé,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -14162,9 +14041,8 @@
       <c r="S121" s="46" t="inlineStr">
         <is>
           <t>Bonjour Pierre St-Arnaud,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'agriculture. La question qui compte pour les producteurs n'a pas changé depuis l'effondrement de la filière en 2018 : est-ce qu'il y a un acheteur stable au bout du champ. On achète encore la récolte de producteurs d'ici et on la transforme nous-mêmes.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -14243,9 +14121,8 @@
       <c r="S122" s="46" t="inlineStr">
         <is>
           <t>Bonjour Katherine Tremblay,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -14333,9 +14210,8 @@
       <c r="S123" s="46" t="inlineStr">
         <is>
           <t>Bonjour Michel Tremblay,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce que l'asclépiade se cultive dans votre région depuis la première vague de 2013, et que plusieurs des producteurs qui ont tenu bon nous vendent encore leur récolte.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -14418,9 +14294,8 @@
       <c r="S124" s="46" t="inlineStr">
         <is>
           <t>Bonjour Martin Vallières,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -14504,9 +14379,8 @@
       <c r="S125" s="46" t="inlineStr">
         <is>
           <t>Bonjour Yanick Villedieu,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -14589,9 +14463,8 @@
       <c r="S126" s="46" t="inlineStr">
         <is>
           <t>Bonjour Jonathan Allard,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -14679,9 +14552,8 @@
       <c r="S127" s="46" t="inlineStr">
         <is>
           <t>Bonjour Anick Baribeau,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce que l'asclépiade a eu son grand moment industriel chez vous : l'usine de Saint-Tite achetait 90 % des récoltes du Québec avant que la filière se casse en 2018. Des producteurs de la Mauricie cultivent encore, et on continue d'acheter leur récolte.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -14765,9 +14637,8 @@
       <c r="S128" s="46" t="inlineStr">
         <is>
           <t>Bonjour Félix-Antoine Beauchemin,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -14850,9 +14721,8 @@
       <c r="S129" s="46" t="inlineStr">
         <is>
           <t>Bonjour Karim Benessaieh,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -14936,9 +14806,8 @@
       <c r="S130" s="46" t="inlineStr">
         <is>
           <t>Bonjour Julia Bernier,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce que l'asclépiade se cultive dans votre région depuis la première vague de 2013, et que plusieurs des producteurs qui ont tenu bon nous vendent encore leur récolte.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -15026,9 +14895,8 @@
       <c r="S131" s="46" t="inlineStr">
         <is>
           <t>Bonjour Karine Boivin Forcier,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce qu'un de nos fournisseurs d'asclépiade cultive au Lac-Saint-Jean depuis nos tout débuts, et qu'il l'est encore aujourd'hui. La fibre de chez vous se retrouve dans nos produits.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -15112,9 +14980,8 @@
       <c r="S132" s="46" t="inlineStr">
         <is>
           <t>Bonjour Audrey Bonaque,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -15197,9 +15064,8 @@
       <c r="S133" s="46" t="inlineStr">
         <is>
           <t>Bonjour Luc Boulanger,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -15282,9 +15148,8 @@
       <c r="S134" s="46" t="inlineStr">
         <is>
           <t>Bonjour Mario Boulianne,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -15372,9 +15237,8 @@
       <c r="S135" s="46" t="inlineStr">
         <is>
           <t>Bonjour Bernard Brault,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -15462,9 +15326,8 @@
       <c r="S136" s="46" t="inlineStr">
         <is>
           <t>Bonjour Pierre Brisson,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -15547,9 +15410,8 @@
       <c r="S137" s="46" t="inlineStr">
         <is>
           <t>Bonjour Laurence Brisson Dubreuil,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -15633,9 +15495,8 @@
       <c r="S138" s="46" t="inlineStr">
         <is>
           <t>Bonjour Nathaniel Bronner,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -15718,9 +15579,8 @@
       <c r="S139" s="46" t="inlineStr">
         <is>
           <t>Bonjour Marie-France Bélanger,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -15804,9 +15664,8 @@
       <c r="S140" s="46" t="inlineStr">
         <is>
           <t>Bonjour Diane Bérard,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -15894,9 +15753,8 @@
       <c r="S141" s="46" t="inlineStr">
         <is>
           <t>Bonjour Julien Cayouette,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -15979,9 +15837,8 @@
       <c r="S142" s="46" t="inlineStr">
         <is>
           <t>Bonjour Rudy Chabannes,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -16069,9 +15926,8 @@
       <c r="S143" s="46" t="inlineStr">
         <is>
           <t>Bonjour Denis-Martin Chabot,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -16155,9 +16011,8 @@
       <c r="S144" s="46" t="inlineStr">
         <is>
           <t>Bonjour Loubna Majda Chourouk,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -16245,9 +16100,8 @@
       <c r="S145" s="46" t="inlineStr">
         <is>
           <t>Bonjour Sarah Collardey,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -16331,9 +16185,8 @@
       <c r="S146" s="46" t="inlineStr">
         <is>
           <t>Bonjour Kathleen Couillard,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -16421,9 +16274,8 @@
       <c r="S147" s="46" t="inlineStr">
         <is>
           <t>Bonjour Oumou DIAKITÉ,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -16506,9 +16358,8 @@
       <c r="S148" s="46" t="inlineStr">
         <is>
           <t>Bonjour Agnès Delavault,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -16592,9 +16443,8 @@
       <c r="S149" s="46" t="inlineStr">
         <is>
           <t>Bonjour Marcelin Delice,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -16678,9 +16528,8 @@
       <c r="S150" s="46" t="inlineStr">
         <is>
           <t>Bonjour Alain Demers,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez le plein air. À poids égal, la littérature donne la soie d'asclépiade pour environ 10 % plus isolante que le duvet. C'est un repère de laboratoire, pas une promesse de manteau, et c'est exactement pour ça que je préfère qu'on la teste.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -16763,9 +16612,8 @@
       <c r="S151" s="46" t="inlineStr">
         <is>
           <t>Bonjour Ivanoh Demers,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -16849,9 +16697,8 @@
       <c r="S152" s="46" t="inlineStr">
         <is>
           <t>Bonjour Claude Deschênes,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -16934,9 +16781,8 @@
       <c r="S153" s="46" t="inlineStr">
         <is>
           <t>Bonjour Thomas Deshaies,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce qu'une des premières usines de transformation de la fibre était à Granby, et que l'Estrie compte encore des producteurs d'asclépiade.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -17024,9 +16870,8 @@
       <c r="S154" s="46" t="inlineStr">
         <is>
           <t>Bonjour Claude Desjardins,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -17110,9 +16955,8 @@
       <c r="S155" s="46" t="inlineStr">
         <is>
           <t>Bonjour Martine Deslauriers,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -17200,9 +17044,8 @@
       <c r="S156" s="46" t="inlineStr">
         <is>
           <t>Bonjour Marie-Claude Di Lillo,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -17285,9 +17128,8 @@
       <c r="S157" s="46" t="inlineStr">
         <is>
           <t>Bonjour Jean-René Dufort,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -17371,9 +17213,8 @@
       <c r="S158" s="46" t="inlineStr">
         <is>
           <t>Bonjour Richard Dupaul,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -17461,9 +17302,8 @@
       <c r="S159" s="46" t="inlineStr">
         <is>
           <t>Bonjour Stéphanie Dupuis,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -17547,9 +17387,8 @@
       <c r="S160" s="46" t="inlineStr">
         <is>
           <t>Bonjour Maxim Fauteux,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce qu'un de nos fournisseurs d'asclépiade cultive au Lac-Saint-Jean depuis nos tout débuts, et qu'il l'est encore aujourd'hui. La fibre de chez vous se retrouve dans nos produits.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -17632,9 +17471,8 @@
       <c r="S161" s="46" t="inlineStr">
         <is>
           <t>Bonjour Ronald Georges,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -17713,9 +17551,8 @@
       <c r="S162" s="46" t="inlineStr">
         <is>
           <t>Bonjour Stéphane Giroux,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -17798,9 +17635,8 @@
       <c r="S163" s="46" t="inlineStr">
         <is>
           <t>Bonjour Zacharie Goudreault,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -17884,9 +17720,8 @@
       <c r="S164" s="46" t="inlineStr">
         <is>
           <t>Bonjour Isabelle Grégoire,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -17969,9 +17804,8 @@
       <c r="S165" s="46" t="inlineStr">
         <is>
           <t>Bonjour Chantal Guy,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -18054,9 +17888,8 @@
       <c r="S166" s="46" t="inlineStr">
         <is>
           <t>Bonjour Matthieu Hains,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -18225,9 +18058,8 @@
       <c r="S168" s="46" t="inlineStr">
         <is>
           <t>Bonjour ANGELO JEAN-BAPTISTE,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -18315,9 +18147,8 @@
       <c r="S169" s="46" t="inlineStr">
         <is>
           <t>Bonjour Andréanne Joly,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -18400,9 +18231,8 @@
       <c r="S170" s="46" t="inlineStr">
         <is>
           <t>Bonjour Hugo Joncas,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -18490,9 +18320,8 @@
       <c r="S171" s="46" t="inlineStr">
         <is>
           <t>Bonjour Philémon La Frenière-Prémont,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -18580,9 +18409,8 @@
       <c r="S172" s="46" t="inlineStr">
         <is>
           <t>Bonjour Henri Laban,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -18751,9 +18579,8 @@
       <c r="S174" s="46" t="inlineStr">
         <is>
           <t>Bonjour Joannie Lafrenière,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -18832,9 +18659,8 @@
       <c r="S175" s="46" t="inlineStr">
         <is>
           <t>Bonjour Angie Landry,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -18918,9 +18744,8 @@
       <c r="S176" s="46" t="inlineStr">
         <is>
           <t>Bonjour Camille Langlade,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -19008,9 +18833,8 @@
       <c r="S177" s="46" t="inlineStr">
         <is>
           <t>Bonjour Claudia Larochelle,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -19093,9 +18917,8 @@
       <c r="S178" s="46" t="inlineStr">
         <is>
           <t>Bonjour Étienne Leblanc,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -19178,9 +19001,8 @@
       <c r="S179" s="46" t="inlineStr">
         <is>
           <t>Bonjour Louise Leduc,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -19264,9 +19086,8 @@
       <c r="S180" s="46" t="inlineStr">
         <is>
           <t>Bonjour Guillaume Longuépée,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -19349,9 +19170,8 @@
       <c r="S181" s="46" t="inlineStr">
         <is>
           <t>Bonjour Roxane Léouzon,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -19435,9 +19255,8 @@
       <c r="S182" s="46" t="inlineStr">
         <is>
           <t>Bonjour Ève Lévesque,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -19521,9 +19340,8 @@
       <c r="S183" s="46" t="inlineStr">
         <is>
           <t>Bonjour Sophie Mangado,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -19611,9 +19429,8 @@
       <c r="S184" s="46" t="inlineStr">
         <is>
           <t>Bonjour Colin McGregor,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -19696,9 +19513,8 @@
       <c r="S185" s="46" t="inlineStr">
         <is>
           <t>Bonjour Isabelle Morin,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -19786,9 +19602,8 @@
       <c r="S186" s="46" t="inlineStr">
         <is>
           <t>Bonjour Timothy Morson,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce que l'asclépiade se cultive dans votre région depuis la première vague de 2013, et que plusieurs des producteurs qui ont tenu bon nous vendent encore leur récolte.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -19876,9 +19691,8 @@
       <c r="S187" s="46" t="inlineStr">
         <is>
           <t>Bonjour Rachid Najahi,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -19962,9 +19776,8 @@
       <c r="S188" s="46" t="inlineStr">
         <is>
           <t>Bonjour Richard Olivier,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -20052,9 +19865,8 @@
       <c r="S189" s="46" t="inlineStr">
         <is>
           <t>Bonjour MELISSA PELLETIER,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -20137,9 +19949,8 @@
       <c r="S190" s="46" t="inlineStr">
         <is>
           <t>Bonjour Isaac Peltz,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce que l'asclépiade se cultive dans votre région depuis la première vague de 2013, et que plusieurs des producteurs qui ont tenu bon nous vendent encore leur récolte.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -20222,9 +20033,8 @@
       <c r="S191" s="46" t="inlineStr">
         <is>
           <t>Bonjour Frédéric Perron,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -20312,9 +20122,8 @@
       <c r="S192" s="46" t="inlineStr">
         <is>
           <t>Bonjour Nathalie Petrowski,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -20397,9 +20206,8 @@
       <c r="S193" s="46" t="inlineStr">
         <is>
           <t>Bonjour Francis Plourde,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -20487,9 +20295,8 @@
       <c r="S194" s="46" t="inlineStr">
         <is>
           <t>Bonjour Raymonde Provencher,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -20577,9 +20384,8 @@
       <c r="S195" s="46" t="inlineStr">
         <is>
           <t>Bonjour Richard Prudhomme,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -20667,9 +20473,8 @@
       <c r="S196" s="46" t="inlineStr">
         <is>
           <t>Bonjour Pascale Renaud,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -20752,9 +20557,8 @@
       <c r="S197" s="46" t="inlineStr">
         <is>
           <t>Bonjour Marc Sony Ricot,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -20842,9 +20646,8 @@
       <c r="S198" s="46" t="inlineStr">
         <is>
           <t>Bonjour Marie-Paul Rouleau,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -20923,9 +20726,8 @@
       <c r="S199" s="46" t="inlineStr">
         <is>
           <t>Bonjour Emmalie Ruest,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -21008,9 +20810,8 @@
       <c r="S200" s="46" t="inlineStr">
         <is>
           <t>Bonjour Louis-Philippe Samson,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce que l'asclépiade se cultive dans votre région depuis la première vague de 2013, et que plusieurs des producteurs qui ont tenu bon nous vendent encore leur récolte.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -21093,9 +20894,8 @@
       <c r="S201" s="46" t="inlineStr">
         <is>
           <t>Bonjour Catherine Schlager,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -21174,9 +20974,8 @@
       <c r="S202" s="46" t="inlineStr">
         <is>
           <t>Bonjour Olivier Schmouker,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -21255,9 +21054,8 @@
       <c r="S203" s="46" t="inlineStr">
         <is>
           <t>Bonjour Jacques Sennechael,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -21340,9 +21138,8 @@
       <c r="S204" s="46" t="inlineStr">
         <is>
           <t>Bonjour Alexandre Shields,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -21421,9 +21218,8 @@
       <c r="S205" s="46" t="inlineStr">
         <is>
           <t>Bonjour Chloé Sondervorst,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -21511,9 +21307,8 @@
       <c r="S206" s="46" t="inlineStr">
         <is>
           <t>Bonjour Kimberley Sullivan,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -21597,9 +21392,8 @@
       <c r="S207" s="46" t="inlineStr">
         <is>
           <t>Bonjour William Thériault,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce que la Montérégie est une des régions où l'asclépiade se cultive encore, et que c'est de champs comme ceux-là que vient la fibre qu'on transforme.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -21682,9 +21476,8 @@
       <c r="S208" s="46" t="inlineStr">
         <is>
           <t>Bonjour Katia Tobar,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -21763,9 +21556,8 @@
       <c r="S209" s="46" t="inlineStr">
         <is>
           <t>Bonjour Martin Tremblay,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -21848,9 +21640,8 @@
       <c r="S210" s="46" t="inlineStr">
         <is>
           <t>Bonjour Marie-Christine Trottier,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -21933,9 +21724,8 @@
       <c r="S211" s="46" t="inlineStr">
         <is>
           <t>Bonjour Pierre-Luc Trudel,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'économie. On a bâti nos propres procédés de transformation parce qu'aucun sous-traitant ne voulait toucher à l'asclépiade, puis on a changé de modèle manufacturier l'an dernier pour rendre un manteau accessible à 300 $. J'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -22019,9 +21809,8 @@
       <c r="S212" s="46" t="inlineStr">
         <is>
           <t>Bonjour David Turbis,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -22104,9 +21893,8 @@
       <c r="S213" s="46" t="inlineStr">
         <is>
           <t>Bonjour Paule Vermot-Desroches,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris entre autres parce que l'asclépiade a eu son grand moment industriel chez vous : l'usine de Saint-Tite achetait 90 % des récoltes du Québec avant que la filière se casse en 2018. Des producteurs de la Mauricie cultivent encore, et on continue d'acheter leur récolte.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -22189,9 +21977,8 @@
       <c r="S214" s="46" t="inlineStr">
         <is>
           <t>Bonjour Alexandra Viau,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que le sujet se raconte bien en ondes : une entreprise de Québec qui va expliquer à un auditoire pancanadien pourquoi la mauvaise herbe des champs de maïs peut isoler un manteau.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -22279,9 +22066,8 @@
       <c r="S215" s="46" t="inlineStr">
         <is>
           <t>Bonjour Raymond Viger,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -22364,9 +22150,8 @@
       <c r="S216" s="46" t="inlineStr">
         <is>
           <t>Bonjour Paul Émile d'Entremont,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que c'est une nouvelle de chez nous qui passe au national.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -22449,9 +22234,8 @@
       <c r="S217" s="46" t="inlineStr">
         <is>
           <t>Bonjour Augustin de Baudinière,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -22530,9 +22314,8 @@
       <c r="S218" s="46" t="inlineStr">
         <is>
           <t>Bonjour Ivan de Jacquelin-Dulphe,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une mauvaise herbe.
-L'asclépiade, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, produit une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis. C'est aussi la seule plante que les chenilles du papillon monarque peuvent manger.
-Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
+Ses gousses, les « petits cochons » que les agriculteurs arrachent de leurs champs depuis 50 ans, sont remplies d'une soie creuse, très légère et naturellement hydrophobe. On la transforme en isolant à Québec, et on en fait des manteaux, des mitaines, des tuques et des sacs isothermes vendus au Canada et aux États-Unis.
 Je vous écris parce que vous couvrez l'environnement. Notre pari est économique avant d'être militant : si l'asclépiade devient payante, les agriculteurs la gardent dans leurs champs, et les monarques retrouvent de l'habitat de reproduction.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -22606,15 +22389,15 @@
       <c r="S219" s="46" t="inlineStr">
         <is>
           <t>Bonjour Jean-Michel Leprince,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une
-mauvaise herbe.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une
+mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et
+menacé : le papillon monarque.
 Vous couvrez l'asclépiade depuis au moins 2014 : le Téléjournal, la soie d'Amérique partie
 sur l'Everest, le pouvoir absorbant de la fibre sur les hydrocarbures, le lien avec le
 monarque. Vous avez suivi cette histoire plus longtemps que la plupart des entreprises qui
 s'y sont essayées.
 On a démarré après la chute de la première filière. Six ans plus tard, on achète encore de l'asclépiade québécoise et on transforme l'isolant nous-mêmes à
-Limoilou. Mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques
-par la culture de l'asclépiade.
+Limoilou.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Vous êtes probablement la personne au Québec qui a le plus longtemps suivi cette plante-là.
@@ -22690,8 +22473,9 @@
       <c r="S220" s="46" t="inlineStr">
         <is>
           <t>Bonjour Antoine Stab,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des manteaux avec une
-mauvaise herbe.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une
+mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et
+menacé : le papillon monarque.
 Vous aviez écrit sur le soyer du Québec dans Espaces en février 2015, à l'époque où la fibre
 devait remplacer le duvet.
 On a démarré après la chute de cette première filière. Six ans plus tard, on achète encore de l'asclépiade québécoise, on transforme l'isolant nous-mêmes, et il

</xml_diff>

<commit_message>
Retire Julia Haurio et Protégez-Vous de la liste chaude
Leurs lignes sont supprimées du chiffrier, pas seulement marquées. Justine
Friis, l'autre contact d'Unpointcinq, reste.

La liste chaude passe de 37 à 35 contacts, le total de 256 à 254.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015pjLsGPzf1MX1JC7QiKGGk
</commit_message>
<xml_diff>
--- a/communique-dragons/Lasclay_v2.xlsx
+++ b/communique-dragons/Lasclay_v2.xlsx
@@ -990,7 +990,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O38"/>
+  <dimension ref="A1:O36"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="26" customWidth="1" style="25" min="1" max="1"/>
@@ -2182,30 +2182,30 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="240" customHeight="1" s="26">
+    <row r="17" ht="15" customHeight="1" s="26">
       <c r="A17" s="36" t="inlineStr">
         <is>
-          <t>Julia Haurio</t>
+          <t>Marc Tison</t>
         </is>
       </c>
       <c r="B17" s="36" t="inlineStr">
         <is>
-          <t>Unpointcinq</t>
+          <t>La Presse</t>
         </is>
       </c>
       <c r="C17" s="36" t="inlineStr">
         <is>
-          <t>jhaurio@unpointcinq.ca</t>
+          <t>mtison1@lapresse.ca</t>
         </is>
       </c>
       <c r="D17" s="36" t="inlineStr">
         <is>
-          <t>2022-01-21</t>
+          <t>2021-09-20</t>
         </is>
       </c>
       <c r="E17" s="37" t="inlineStr">
         <is>
-          <t>Impact climatique asclépiade</t>
+          <t>Entrevue — section Affaires</t>
         </is>
       </c>
       <c r="F17" s="36" t="inlineStr">
@@ -2233,17 +2233,17 @@
       </c>
       <c r="M17" s="25" t="inlineStr">
         <is>
-          <t>Bonjour Julia,</t>
+          <t>Bonjour Marc,</t>
         </is>
       </c>
       <c r="N17" s="46" t="inlineStr">
         <is>
-          <t>Bonjour Mme Haurio,
-On avait creusé l'impact climatique de l'asclépiade ensemble en janvier 2022.
-Depuis, tout mon temps va à mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+          <t>Bonjour M. Tison,
+On s'était parlé pour la section Affaires en septembre 2021, à l'époque où on venait de rapatrier notre production faute de sous-traitant prêt à toucher à la fibre. Le modèle a changé depuis : la vidéo est ici, https://www.youtube.com/watch?v=GKyHh-Ok9JU, et Sylvain Larocque en a parlé en mai.
+Parmi les raisons de ce changement, il y avait clairement que j'avais besoin de temps pour me recentrer sur mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer une suite à votre dernier article.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -2254,30 +2254,30 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="240" customHeight="1" s="26">
+    <row r="18" ht="15" customHeight="1" s="26">
       <c r="A18" s="36" t="inlineStr">
         <is>
-          <t>Protégez-Vous (contact général)</t>
+          <t>Valérie Simard</t>
         </is>
       </c>
       <c r="B18" s="36" t="inlineStr">
         <is>
-          <t>Protégez-Vous</t>
+          <t>La Presse</t>
         </is>
       </c>
       <c r="C18" s="36" t="inlineStr">
         <is>
-          <t>contact@protegez-vous.ca</t>
+          <t>vsimard@lapresse.ca</t>
         </is>
       </c>
       <c r="D18" s="36" t="inlineStr">
         <is>
-          <t>2021-11-19</t>
+          <t>2021-09-17</t>
         </is>
       </c>
       <c r="E18" s="37" t="inlineStr">
         <is>
-          <t>Étude de marché sur les glacières</t>
+          <t>Demande média</t>
         </is>
       </c>
       <c r="F18" s="36" t="inlineStr">
@@ -2305,17 +2305,17 @@
       </c>
       <c r="M18" s="25" t="inlineStr">
         <is>
-          <t>Bonjour Protégez-Vous,</t>
+          <t>Bonjour Valérie,</t>
         </is>
       </c>
       <c r="N18" s="46" t="inlineStr">
         <is>
-          <t>Bonjour,
-En novembre 2021, votre équipe nous avait contactés pour une étude de marché sur les glacières. Nos sacs isothermes et nos glacières souples sont isolés à la soie d'asclépiade, une fibre creuse et naturellement hydrophobe.
+          <t>Bonjour Mme Simard,
+Vous aviez présenté nos moufles isolées à l'asclépiade le 17 septembre 2021. Drôle de coïncidence : la diffusion tombe cinq ans jour pour jour après votre article.
 Depuis, tout mon temps va à mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer une suite à votre dernier article.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -2329,27 +2329,27 @@
     <row r="19" ht="240" customHeight="1" s="26">
       <c r="A19" s="36" t="inlineStr">
         <is>
-          <t>Marc Tison</t>
+          <t>Justine Friis</t>
         </is>
       </c>
       <c r="B19" s="36" t="inlineStr">
         <is>
-          <t>La Presse</t>
+          <t>Unpointcinq</t>
         </is>
       </c>
       <c r="C19" s="36" t="inlineStr">
         <is>
-          <t>mtison1@lapresse.ca</t>
+          <t>jfriis@unpointcinq.ca</t>
         </is>
       </c>
       <c r="D19" s="36" t="inlineStr">
         <is>
-          <t>2021-09-20</t>
+          <t>2021-09-08</t>
         </is>
       </c>
       <c r="E19" s="37" t="inlineStr">
         <is>
-          <t>Entrevue — section Affaires</t>
+          <t>Impact climatique asclépiade</t>
         </is>
       </c>
       <c r="F19" s="36" t="inlineStr">
@@ -2377,17 +2377,17 @@
       </c>
       <c r="M19" s="25" t="inlineStr">
         <is>
-          <t>Bonjour Marc,</t>
+          <t>Bonjour Justine,</t>
         </is>
       </c>
       <c r="N19" s="46" t="inlineStr">
         <is>
-          <t>Bonjour M. Tison,
-On s'était parlé pour la section Affaires en septembre 2021, à l'époque où on venait de rapatrier notre production faute de sous-traitant prêt à toucher à la fibre. Le modèle a changé depuis : la vidéo est ici, https://www.youtube.com/watch?v=GKyHh-Ok9JU, et Sylvain Larocque en a parlé en mai.
-Parmi les raisons de ce changement, il y avait clairement que j'avais besoin de temps pour me recentrer sur mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+          <t>Bonjour Mme Friis,
+Vous aviez travaillé sur l'impact climatique de l'asclépiade en septembre 2021.
+Depuis, tout mon temps va à mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer une suite à votre dernier article.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -2401,27 +2401,27 @@
     <row r="20" ht="240" customHeight="1" s="26">
       <c r="A20" s="36" t="inlineStr">
         <is>
-          <t>Valérie Simard</t>
+          <t>Alex Perreault</t>
         </is>
       </c>
       <c r="B20" s="36" t="inlineStr">
         <is>
-          <t>La Presse</t>
+          <t>Radio-Canada</t>
         </is>
       </c>
       <c r="C20" s="36" t="inlineStr">
         <is>
-          <t>vsimard@lapresse.ca</t>
+          <t>alex.perreault@radio-canada.ca</t>
         </is>
       </c>
       <c r="D20" s="36" t="inlineStr">
         <is>
-          <t>2021-09-17</t>
+          <t>2021-07-22</t>
         </is>
       </c>
       <c r="E20" s="37" t="inlineStr">
         <is>
-          <t>Demande média</t>
+          <t>Entrevue Radio-Canada</t>
         </is>
       </c>
       <c r="F20" s="36" t="inlineStr">
@@ -2449,17 +2449,17 @@
       </c>
       <c r="M20" s="25" t="inlineStr">
         <is>
-          <t>Bonjour Valérie,</t>
+          <t>Bonjour Alex,</t>
         </is>
       </c>
       <c r="N20" s="46" t="inlineStr">
         <is>
-          <t>Bonjour Mme Simard,
-Vous aviez présenté nos moufles isolées à l'asclépiade le 17 septembre 2021. Drôle de coïncidence : la diffusion tombe cinq ans jour pour jour après votre article.
+          <t>Bonjour M. Perreault,
+On s'était parlé en juillet 2021.
 Depuis, tout mon temps va à mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer une suite à votre dernier article.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part : je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -2473,27 +2473,27 @@
     <row r="21" ht="240" customHeight="1" s="26">
       <c r="A21" s="36" t="inlineStr">
         <is>
-          <t>Justine Friis</t>
+          <t>Francis Higgins</t>
         </is>
       </c>
       <c r="B21" s="36" t="inlineStr">
         <is>
-          <t>Unpointcinq</t>
+          <t>Le Soleil</t>
         </is>
       </c>
       <c r="C21" s="36" t="inlineStr">
         <is>
-          <t>jfriis@unpointcinq.ca</t>
+          <t>fhiggins@lesoleil.com</t>
         </is>
       </c>
       <c r="D21" s="36" t="inlineStr">
         <is>
-          <t>2021-09-08</t>
+          <t>2021-07-07</t>
         </is>
       </c>
       <c r="E21" s="37" t="inlineStr">
         <is>
-          <t>Impact climatique asclépiade</t>
+          <t>Demande de presse — Le Soleil de Québec</t>
         </is>
       </c>
       <c r="F21" s="36" t="inlineStr">
@@ -2521,17 +2521,17 @@
       </c>
       <c r="M21" s="25" t="inlineStr">
         <is>
-          <t>Bonjour Justine,</t>
+          <t>Bonjour Francis,</t>
         </is>
       </c>
       <c r="N21" s="46" t="inlineStr">
         <is>
-          <t>Bonjour Mme Friis,
-Vous aviez travaillé sur l'impact climatique de l'asclépiade en septembre 2021.
+          <t>Bonjour M. Higgins,
+On s'était parlé pour Le Soleil en juillet 2021. L'atelier est toujours dans Limoilou.
 Depuis, tout mon temps va à mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer une suite à votre dernier article.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -2545,7 +2545,7 @@
     <row r="22" ht="240" customHeight="1" s="26">
       <c r="A22" s="36" t="inlineStr">
         <is>
-          <t>Alex Perreault</t>
+          <t>Fanny Samson</t>
         </is>
       </c>
       <c r="B22" s="36" t="inlineStr">
@@ -2555,17 +2555,17 @@
       </c>
       <c r="C22" s="36" t="inlineStr">
         <is>
-          <t>alex.perreault@radio-canada.ca</t>
+          <t>fanny.samson@radio-canada.ca</t>
         </is>
       </c>
       <c r="D22" s="36" t="inlineStr">
         <is>
-          <t>2021-07-22</t>
+          <t>2021-03-13</t>
         </is>
       </c>
       <c r="E22" s="37" t="inlineStr">
         <is>
-          <t>Entrevue Radio-Canada</t>
+          <t>Reportage</t>
         </is>
       </c>
       <c r="F22" s="36" t="inlineStr">
@@ -2593,17 +2593,17 @@
       </c>
       <c r="M22" s="25" t="inlineStr">
         <is>
-          <t>Bonjour Alex,</t>
+          <t>Bonjour Fanny,</t>
         </is>
       </c>
       <c r="N22" s="46" t="inlineStr">
         <is>
-          <t>Bonjour M. Perreault,
-On s'était parlé en juillet 2021.
+          <t>Bonjour Mme Samson,
+En mars 2021, vous aviez signé « Les grandes promesses de l'asclépiade, la soie d'Amérique ». Cinq ans plus tard, je peux vous dire lesquelles ont été tenues : il y a des produits finis, l'isolant se transforme toujours au Québec, on achète encore de l'asclépiade québécoise, et un manteau se vend autour de 300 $.
 Depuis, tout mon temps va à mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part : je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer une suite à votre dernier article.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -2617,27 +2617,27 @@
     <row r="23" ht="240" customHeight="1" s="26">
       <c r="A23" s="36" t="inlineStr">
         <is>
-          <t>Francis Higgins</t>
+          <t>Martin Ménard</t>
         </is>
       </c>
       <c r="B23" s="36" t="inlineStr">
         <is>
-          <t>Le Soleil</t>
+          <t>La Terre de chez nous</t>
         </is>
       </c>
       <c r="C23" s="36" t="inlineStr">
         <is>
-          <t>fhiggins@lesoleil.com</t>
+          <t>mmenard@laterre.ca</t>
         </is>
       </c>
       <c r="D23" s="36" t="inlineStr">
         <is>
-          <t>2021-07-07</t>
+          <t>2021-01-26</t>
         </is>
       </c>
       <c r="E23" s="37" t="inlineStr">
         <is>
-          <t>Demande de presse — Le Soleil de Québec</t>
+          <t>Entrevue La Terre</t>
         </is>
       </c>
       <c r="F23" s="36" t="inlineStr">
@@ -2665,13 +2665,13 @@
       </c>
       <c r="M23" s="25" t="inlineStr">
         <is>
-          <t>Bonjour Francis,</t>
+          <t>Bonjour Martin,</t>
         </is>
       </c>
       <c r="N23" s="46" t="inlineStr">
         <is>
-          <t>Bonjour M. Higgins,
-On s'était parlé pour Le Soleil en juillet 2021. L'atelier est toujours dans Limoilou.
+          <t>Bonjour M. Ménard,
+On s'était parlé à La Terre en janvier 2021. Cinq ans plus tard, on achète encore de l'asclépiade québécoise et on la transforme nous-mêmes à Québec.
 Depuis, tout mon temps va à mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -2689,27 +2689,27 @@
     <row r="24" ht="240" customHeight="1" s="26">
       <c r="A24" s="36" t="inlineStr">
         <is>
-          <t>Fanny Samson</t>
+          <t>Anne-Sophie Roy</t>
         </is>
       </c>
       <c r="B24" s="36" t="inlineStr">
         <is>
-          <t>Radio-Canada</t>
+          <t>Québecor Média</t>
         </is>
       </c>
       <c r="C24" s="36" t="inlineStr">
         <is>
-          <t>fanny.samson@radio-canada.ca</t>
+          <t>anne-sophie.roy@quebecormedia.com</t>
         </is>
       </c>
       <c r="D24" s="36" t="inlineStr">
         <is>
-          <t>2021-03-13</t>
+          <t>2020-12-13</t>
         </is>
       </c>
       <c r="E24" s="37" t="inlineStr">
         <is>
-          <t>Reportage</t>
+          <t>Série d'articles</t>
         </is>
       </c>
       <c r="F24" s="36" t="inlineStr">
@@ -2732,56 +2732,49 @@
       </c>
       <c r="L24" s="25" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M24" s="25" t="inlineStr">
         <is>
-          <t>Bonjour Fanny,</t>
+          <t>Bonjour Anne-Sophie,</t>
         </is>
       </c>
       <c r="N24" s="46" t="inlineStr">
         <is>
-          <t>Bonjour Mme Samson,
-En mars 2021, vous aviez signé « Les grandes promesses de l'asclépiade, la soie d'Amérique ». Cinq ans plus tard, je peux vous dire lesquelles ont été tenues : il y a des produits finis, l'isolant se transforme toujours au Québec, on achète encore de l'asclépiade québécoise, et un manteau se vend autour de 300 $.
-Depuis, tout mon temps va à mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
-Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
-Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer une suite à votre dernier article.
-J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
-Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
+          <t>NE PAS ENVOYER — même journaliste que la ligne Radio-Canada, à une ancienne adresse. Écrire à anne-sophie.roy@radio-canada.ca. Garder cette adresse en réserve si l'autre rebondit.</t>
         </is>
       </c>
       <c r="O24" s="25" t="inlineStr">
         <is>
-          <t>vous</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="25" ht="240" customHeight="1" s="26">
       <c r="A25" s="36" t="inlineStr">
         <is>
-          <t>Martin Ménard</t>
+          <t>Raphaëlle Drouin</t>
         </is>
       </c>
       <c r="B25" s="36" t="inlineStr">
         <is>
-          <t>La Terre de chez nous</t>
+          <t>URBANIA</t>
         </is>
       </c>
       <c r="C25" s="36" t="inlineStr">
         <is>
-          <t>mmenard@laterre.ca</t>
+          <t>raphaelle.drouin@urbania.ca</t>
         </is>
       </c>
       <c r="D25" s="36" t="inlineStr">
         <is>
-          <t>2021-01-26</t>
+          <t>2020-11-24</t>
         </is>
       </c>
       <c r="E25" s="37" t="inlineStr">
         <is>
-          <t>Entrevue La Terre</t>
+          <t>Entrevue URBANIA</t>
         </is>
       </c>
       <c r="F25" s="36" t="inlineStr">
@@ -2809,13 +2802,13 @@
       </c>
       <c r="M25" s="25" t="inlineStr">
         <is>
-          <t>Bonjour Martin,</t>
+          <t>Bonjour Raphaëlle,</t>
         </is>
       </c>
       <c r="N25" s="46" t="inlineStr">
         <is>
-          <t>Bonjour M. Ménard,
-On s'était parlé à La Terre en janvier 2021. Cinq ans plus tard, on achète encore de l'asclépiade québécoise et on la transforme nous-mêmes à Québec.
+          <t>Bonjour Mme Drouin,
+En janvier 2021, vous aviez écrit « Devenir viral avant même de se lancer en affaires ». Six ans plus tard, l'entreprise existe pour vrai, avec plus de 40 produits.
 Depuis, tout mon temps va à mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -2833,37 +2826,29 @@
     <row r="26" ht="15" customHeight="1" s="26">
       <c r="A26" s="36" t="inlineStr">
         <is>
-          <t>Anne-Sophie Roy</t>
+          <t>G. Roy</t>
         </is>
       </c>
       <c r="B26" s="36" t="inlineStr">
         <is>
-          <t>Québecor Média</t>
+          <t>Le Quotidien</t>
         </is>
       </c>
       <c r="C26" s="36" t="inlineStr">
         <is>
-          <t>anne-sophie.roy@quebecormedia.com</t>
-        </is>
-      </c>
-      <c r="D26" s="36" t="inlineStr">
-        <is>
-          <t>2020-12-13</t>
-        </is>
-      </c>
-      <c r="E26" s="37" t="inlineStr">
-        <is>
-          <t>Série d'articles</t>
-        </is>
-      </c>
+          <t>groy@lequotidien.com</t>
+        </is>
+      </c>
+      <c r="D26" s="36" t="n"/>
+      <c r="E26" s="37" t="n"/>
       <c r="F26" s="36" t="inlineStr">
         <is>
-          <t>Missive — boîte LAS Media</t>
-        </is>
-      </c>
-      <c r="G26" s="36" t="inlineStr">
-        <is>
-          <t>Correspondance confirmée</t>
+          <t>Fournie par Gabriel</t>
+        </is>
+      </c>
+      <c r="G26" s="40" t="inlineStr">
+        <is>
+          <t>Non recoupée dans Missive</t>
         </is>
       </c>
       <c r="H26" s="38" t="n"/>
@@ -2876,59 +2861,58 @@
       </c>
       <c r="L26" s="25" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="M26" s="25" t="inlineStr">
         <is>
-          <t>Bonjour Anne-Sophie,</t>
+          <t>Bonjour,</t>
         </is>
       </c>
       <c r="N26" s="46" t="inlineStr">
         <is>
-          <t>NE PAS ENVOYER — même journaliste que la ligne Radio-Canada, à une ancienne adresse. Écrire à anne-sophie.roy@radio-canada.ca. Garder cette adresse en réserve si l'autre rebondit.</t>
+          <t>Bonjour M. Roy,
+En octobre 2020, vous avez écrit « La deuxième vie de l'asclépiade ». Vous avez été le tout premier journaliste à parler de nous. Et l'agriculteur du Lac-Saint-Jean qui vous avait donné envie du sujet est encore notre fournisseur aujourd'hui : six ans plus tard, l'asclépiade de chez vous se retrouve toujours dans nos produits.
+Depuis, tout mon temps va à mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
+Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer une suite à votre dernier article.
+J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
+Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
       </c>
       <c r="O26" s="25" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>vous</t>
         </is>
       </c>
     </row>
     <row r="27" ht="240" customHeight="1" s="26">
       <c r="A27" s="36" t="inlineStr">
         <is>
-          <t>Raphaëlle Drouin</t>
+          <t>Mireille Roberge</t>
         </is>
       </c>
       <c r="B27" s="36" t="inlineStr">
         <is>
-          <t>URBANIA</t>
+          <t>Radio-Canada</t>
         </is>
       </c>
       <c r="C27" s="36" t="inlineStr">
         <is>
-          <t>raphaelle.drouin@urbania.ca</t>
-        </is>
-      </c>
-      <c r="D27" s="36" t="inlineStr">
-        <is>
-          <t>2020-11-24</t>
-        </is>
-      </c>
-      <c r="E27" s="37" t="inlineStr">
-        <is>
-          <t>Entrevue URBANIA</t>
-        </is>
-      </c>
+          <t>mireille.roberge@radio-canada.ca</t>
+        </is>
+      </c>
+      <c r="D27" s="36" t="n"/>
+      <c r="E27" s="37" t="n"/>
       <c r="F27" s="36" t="inlineStr">
         <is>
-          <t>Missive — boîte LAS Media</t>
-        </is>
-      </c>
-      <c r="G27" s="36" t="inlineStr">
-        <is>
-          <t>Correspondance confirmée</t>
+          <t>Fournie par Gabriel</t>
+        </is>
+      </c>
+      <c r="G27" s="40" t="inlineStr">
+        <is>
+          <t>Non recoupée dans Missive</t>
         </is>
       </c>
       <c r="H27" s="38" t="n"/>
@@ -2946,17 +2930,16 @@
       </c>
       <c r="M27" s="25" t="inlineStr">
         <is>
-          <t>Bonjour Raphaëlle,</t>
+          <t>Bonjour Mireille,</t>
         </is>
       </c>
       <c r="N27" s="46" t="inlineStr">
         <is>
-          <t>Bonjour Mme Drouin,
-En janvier 2021, vous aviez écrit « Devenir viral avant même de se lancer en affaires ». Six ans plus tard, l'entreprise existe pour vrai, avec plus de 40 produits.
-Depuis, tout mon temps va à mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
-Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
-Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer une suite à votre dernier article.
+          <t>Bonjour Mme Roberge,
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque. Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe, qu'on transforme en isolant à Québec.
+Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
+Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part : je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -2970,17 +2953,17 @@
     <row r="28" ht="240" customHeight="1" s="26">
       <c r="A28" s="36" t="inlineStr">
         <is>
-          <t>G. Roy</t>
+          <t>Sophie Laforest</t>
         </is>
       </c>
       <c r="B28" s="36" t="inlineStr">
         <is>
-          <t>Le Quotidien</t>
+          <t>Radio-Canada</t>
         </is>
       </c>
       <c r="C28" s="36" t="inlineStr">
         <is>
-          <t>groy@lequotidien.com</t>
+          <t>sophie.laforest@radio-canada.ca</t>
         </is>
       </c>
       <c r="D28" s="36" t="n"/>
@@ -3010,13 +2993,88 @@
       </c>
       <c r="M28" s="25" t="inlineStr">
         <is>
-          <t>Bonjour,</t>
+          <t>Bonjour Sophie,</t>
         </is>
       </c>
       <c r="N28" s="46" t="inlineStr">
         <is>
-          <t>Bonjour M. Roy,
-En octobre 2020, vous avez écrit « La deuxième vie de l'asclépiade ». Vous avez été le tout premier journaliste à parler de nous. Et l'agriculteur du Lac-Saint-Jean qui vous avait donné envie du sujet est encore notre fournisseur aujourd'hui : six ans plus tard, l'asclépiade de chez vous se retrouve toujours dans nos produits.
+          <t>Bonjour Mme Laforest,
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque. Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe, qu'on transforme en isolant à Québec.
+Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
+Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part : je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
+J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
+Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
+        </is>
+      </c>
+      <c r="O28" s="25" t="inlineStr">
+        <is>
+          <t>vous</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="240" customHeight="1" s="26">
+      <c r="A29" s="36" t="inlineStr">
+        <is>
+          <t>Alain McKenna</t>
+        </is>
+      </c>
+      <c r="B29" s="36" t="inlineStr">
+        <is>
+          <t>Le Devoir</t>
+        </is>
+      </c>
+      <c r="C29" s="36" t="inlineStr">
+        <is>
+          <t>amckenna@ledevoir.com</t>
+        </is>
+      </c>
+      <c r="D29" s="36" t="inlineStr">
+        <is>
+          <t>2021-12-24</t>
+        </is>
+      </c>
+      <c r="E29" s="37" t="inlineStr">
+        <is>
+          <t>Des écouteurs de Québec pour oublier les AirPods (Sounds Good)</t>
+        </is>
+      </c>
+      <c r="F29" s="36" t="inlineStr">
+        <is>
+          <t>Lien fourni par Gabriel</t>
+        </is>
+      </c>
+      <c r="G29" s="40" t="inlineStr">
+        <is>
+          <t>Correspondance confirmée</t>
+        </is>
+      </c>
+      <c r="H29" s="38" t="n"/>
+      <c r="I29" s="38" t="n"/>
+      <c r="J29" s="39" t="inlineStr">
+        <is>
+          <t>A couvert Sounds Good, la première entreprise de Gabriel, à l'époque des trois associés. Gabriel a vendu ses parts en 2022 : le dire d'entrée, McKenna suit encore Sounds Good.</t>
+        </is>
+      </c>
+      <c r="K29" s="25" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="L29" s="25" t="inlineStr">
+        <is>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
+        </is>
+      </c>
+      <c r="M29" s="25" t="inlineStr">
+        <is>
+          <t>Bonjour Alain,</t>
+        </is>
+      </c>
+      <c r="N29" s="46" t="inlineStr">
+        <is>
+          <t>Bonjour M. McKenna,
+En décembre 2021, vous aviez écrit « Des écouteurs de Québec pour oublier les AirPods », sur Sounds Good. J'étais un des trois. J'ai vendu mes parts en 2022 pour me consacrer entièrement à Lasclay, l'autre entreprise que j'avais démarrée entretemps, qui transforme la soie d'asclépiade en isolant textile.
 Depuis, tout mon temps va à mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -3025,69 +3083,6 @@
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
       </c>
-      <c r="O28" s="25" t="inlineStr">
-        <is>
-          <t>vous</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="240" customHeight="1" s="26">
-      <c r="A29" s="36" t="inlineStr">
-        <is>
-          <t>Mireille Roberge</t>
-        </is>
-      </c>
-      <c r="B29" s="36" t="inlineStr">
-        <is>
-          <t>Radio-Canada</t>
-        </is>
-      </c>
-      <c r="C29" s="36" t="inlineStr">
-        <is>
-          <t>mireille.roberge@radio-canada.ca</t>
-        </is>
-      </c>
-      <c r="D29" s="36" t="n"/>
-      <c r="E29" s="37" t="n"/>
-      <c r="F29" s="36" t="inlineStr">
-        <is>
-          <t>Fournie par Gabriel</t>
-        </is>
-      </c>
-      <c r="G29" s="40" t="inlineStr">
-        <is>
-          <t>Non recoupée dans Missive</t>
-        </is>
-      </c>
-      <c r="H29" s="38" t="n"/>
-      <c r="I29" s="38" t="n"/>
-      <c r="J29" s="39" t="n"/>
-      <c r="K29" s="25" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="L29" s="25" t="inlineStr">
-        <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
-        </is>
-      </c>
-      <c r="M29" s="25" t="inlineStr">
-        <is>
-          <t>Bonjour Mireille,</t>
-        </is>
-      </c>
-      <c r="N29" s="46" t="inlineStr">
-        <is>
-          <t>Bonjour Mme Roberge,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque. Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe, qu'on transforme en isolant à Québec.
-Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
-Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part : je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
-J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
-Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
-        </is>
-      </c>
       <c r="O29" s="25" t="inlineStr">
         <is>
           <t>vous</t>
@@ -3097,17 +3092,17 @@
     <row r="30" ht="240" customHeight="1" s="26">
       <c r="A30" s="36" t="inlineStr">
         <is>
-          <t>Sophie Laforest</t>
+          <t>Sylvie Lemieux</t>
         </is>
       </c>
       <c r="B30" s="36" t="inlineStr">
         <is>
-          <t>Radio-Canada</t>
+          <t>Pigiste</t>
         </is>
       </c>
       <c r="C30" s="36" t="inlineStr">
         <is>
-          <t>sophie.laforest@radio-canada.ca</t>
+          <t>sylvielemieux16@gmail.com</t>
         </is>
       </c>
       <c r="D30" s="36" t="n"/>
@@ -3137,16 +3132,17 @@
       </c>
       <c r="M30" s="25" t="inlineStr">
         <is>
-          <t>Bonjour Sophie,</t>
+          <t>Bonjour Sylvie,</t>
         </is>
       </c>
       <c r="N30" s="46" t="inlineStr">
         <is>
-          <t>Bonjour Mme Laforest,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque. Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe, qu'on transforme en isolant à Québec.
-Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
-Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part : je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
+          <t>Bonjour Mme Lemieux,
+En décembre 2021, vous aviez écrit « Les deux mains dans l'écoresponsabilité » pour le Journal de Montréal. Notre modèle manufacturier a changé depuis, et j'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
+Parmi les raisons de ce changement, il y avait clairement que j'avais besoin de temps pour me recentrer sur mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
+Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer une suite à votre dernier article.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -3160,46 +3156,34 @@
     <row r="31" ht="240" customHeight="1" s="26">
       <c r="A31" s="36" t="inlineStr">
         <is>
-          <t>Alain McKenna</t>
+          <t>Sophie Grenier-Héroux</t>
         </is>
       </c>
       <c r="B31" s="36" t="inlineStr">
         <is>
-          <t>Le Devoir</t>
+          <t>Pigiste</t>
         </is>
       </c>
       <c r="C31" s="36" t="inlineStr">
         <is>
-          <t>amckenna@ledevoir.com</t>
-        </is>
-      </c>
-      <c r="D31" s="36" t="inlineStr">
-        <is>
-          <t>2021-12-24</t>
-        </is>
-      </c>
-      <c r="E31" s="37" t="inlineStr">
-        <is>
-          <t>Des écouteurs de Québec pour oublier les AirPods (Sounds Good)</t>
-        </is>
-      </c>
+          <t>sophiegrenierheroux@hotmail.com</t>
+        </is>
+      </c>
+      <c r="D31" s="36" t="n"/>
+      <c r="E31" s="37" t="n"/>
       <c r="F31" s="36" t="inlineStr">
         <is>
-          <t>Lien fourni par Gabriel</t>
+          <t>Fournie par Gabriel</t>
         </is>
       </c>
       <c r="G31" s="40" t="inlineStr">
         <is>
-          <t>Correspondance confirmée</t>
+          <t>Non recoupée dans Missive</t>
         </is>
       </c>
       <c r="H31" s="38" t="n"/>
       <c r="I31" s="38" t="n"/>
-      <c r="J31" s="39" t="inlineStr">
-        <is>
-          <t>A couvert Sounds Good, la première entreprise de Gabriel, à l'époque des trois associés. Gabriel a vendu ses parts en 2022 : le dire d'entrée, McKenna suit encore Sounds Good.</t>
-        </is>
-      </c>
+      <c r="J31" s="39" t="n"/>
       <c r="K31" s="25" t="inlineStr">
         <is>
           <t>A</t>
@@ -3212,13 +3196,13 @@
       </c>
       <c r="M31" s="25" t="inlineStr">
         <is>
-          <t>Bonjour Alain,</t>
+          <t>Bonjour Sophie,</t>
         </is>
       </c>
       <c r="N31" s="46" t="inlineStr">
         <is>
-          <t>Bonjour M. McKenna,
-En décembre 2021, vous aviez écrit « Des écouteurs de Québec pour oublier les AirPods », sur Sounds Good. J'étais un des trois. J'ai vendu mes parts en 2022 pour me consacrer entièrement à Lasclay, l'autre entreprise que j'avais démarrée entretemps, qui transforme la soie d'asclépiade en isolant textile.
+          <t>Bonjour Mme Grenier-Héroux,
+En janvier 2021, vous aviez écrit « La soie d'Amérique, le pari de deux ambitieux » dans Le Devoir. Le pari a six ans, et il tient : plus de 40 produits, environ 10 millions de graines distribuées, et un isolant toujours transformé à Limoilou.
 Depuis, tout mon temps va à mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -3236,7 +3220,7 @@
     <row r="32" ht="240" customHeight="1" s="26">
       <c r="A32" s="36" t="inlineStr">
         <is>
-          <t>Sylvie Lemieux</t>
+          <t>Madeleine Goubau</t>
         </is>
       </c>
       <c r="B32" s="36" t="inlineStr">
@@ -3246,7 +3230,7 @@
       </c>
       <c r="C32" s="36" t="inlineStr">
         <is>
-          <t>sylvielemieux16@gmail.com</t>
+          <t>madeleine.goubau@gmail.com</t>
         </is>
       </c>
       <c r="D32" s="36" t="n"/>
@@ -3276,17 +3260,16 @@
       </c>
       <c r="M32" s="25" t="inlineStr">
         <is>
-          <t>Bonjour Sylvie,</t>
+          <t>Bonjour Madeleine,</t>
         </is>
       </c>
       <c r="N32" s="46" t="inlineStr">
         <is>
-          <t>Bonjour Mme Lemieux,
-En décembre 2021, vous aviez écrit « Les deux mains dans l'écoresponsabilité » pour le Journal de Montréal. Notre modèle manufacturier a changé depuis, et j'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
-Parmi les raisons de ce changement, il y avait clairement que j'avais besoin de temps pour me recentrer sur mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
-Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
-Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer une suite à votre dernier article.
+          <t>Bonjour Mme Goubau,
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque. Vous couvrez le textile et la mode, alors voici une matière que peu de gens ont vue de près : la soie d'asclépiade, une fibre creuse et naturellement hydrophobe attachée aux graines d'une plante que les agriculteurs arrachent de leurs champs depuis 50 ans. On la transforme en isolant, et on en fait des manteaux, des mitaines et des tuques.
+Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
+Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet.
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -3300,7 +3283,7 @@
     <row r="33" ht="240" customHeight="1" s="26">
       <c r="A33" s="36" t="inlineStr">
         <is>
-          <t>Sophie Grenier-Héroux</t>
+          <t>Jessica Dostie</t>
         </is>
       </c>
       <c r="B33" s="36" t="inlineStr">
@@ -3310,7 +3293,7 @@
       </c>
       <c r="C33" s="36" t="inlineStr">
         <is>
-          <t>sophiegrenierheroux@hotmail.com</t>
+          <t>jessica.dostie@gmail.com</t>
         </is>
       </c>
       <c r="D33" s="36" t="n"/>
@@ -3340,137 +3323,10 @@
       </c>
       <c r="M33" s="25" t="inlineStr">
         <is>
-          <t>Bonjour Sophie,</t>
+          <t>Bonjour Jessica,</t>
         </is>
       </c>
       <c r="N33" s="46" t="inlineStr">
-        <is>
-          <t>Bonjour Mme Grenier-Héroux,
-En janvier 2021, vous aviez écrit « La soie d'Amérique, le pari de deux ambitieux » dans Le Devoir. Le pari a six ans, et il tient : plus de 40 produits, environ 10 millions de graines distribuées, et un isolant toujours transformé à Limoilou.
-Depuis, tout mon temps va à mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
-Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
-Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer une suite à votre dernier article.
-J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
-Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
-        </is>
-      </c>
-      <c r="O33" s="25" t="inlineStr">
-        <is>
-          <t>vous</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="240" customHeight="1" s="26">
-      <c r="A34" s="36" t="inlineStr">
-        <is>
-          <t>Madeleine Goubau</t>
-        </is>
-      </c>
-      <c r="B34" s="36" t="inlineStr">
-        <is>
-          <t>Pigiste</t>
-        </is>
-      </c>
-      <c r="C34" s="36" t="inlineStr">
-        <is>
-          <t>madeleine.goubau@gmail.com</t>
-        </is>
-      </c>
-      <c r="D34" s="36" t="n"/>
-      <c r="E34" s="37" t="n"/>
-      <c r="F34" s="36" t="inlineStr">
-        <is>
-          <t>Fournie par Gabriel</t>
-        </is>
-      </c>
-      <c r="G34" s="40" t="inlineStr">
-        <is>
-          <t>Non recoupée dans Missive</t>
-        </is>
-      </c>
-      <c r="H34" s="38" t="n"/>
-      <c r="I34" s="38" t="n"/>
-      <c r="J34" s="39" t="n"/>
-      <c r="K34" s="25" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="L34" s="25" t="inlineStr">
-        <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
-        </is>
-      </c>
-      <c r="M34" s="25" t="inlineStr">
-        <is>
-          <t>Bonjour Madeleine,</t>
-        </is>
-      </c>
-      <c r="N34" s="46" t="inlineStr">
-        <is>
-          <t>Bonjour Mme Goubau,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque. Vous couvrez le textile et la mode, alors voici une matière que peu de gens ont vue de près : la soie d'asclépiade, une fibre creuse et naturellement hydrophobe attachée aux graines d'une plante que les agriculteurs arrachent de leurs champs depuis 50 ans. On la transforme en isolant, et on en fait des manteaux, des mitaines et des tuques.
-Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
-Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet.
-J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
-Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
-        </is>
-      </c>
-      <c r="O34" s="25" t="inlineStr">
-        <is>
-          <t>vous</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="240" customHeight="1" s="26">
-      <c r="A35" s="36" t="inlineStr">
-        <is>
-          <t>Jessica Dostie</t>
-        </is>
-      </c>
-      <c r="B35" s="36" t="inlineStr">
-        <is>
-          <t>Pigiste</t>
-        </is>
-      </c>
-      <c r="C35" s="36" t="inlineStr">
-        <is>
-          <t>jessica.dostie@gmail.com</t>
-        </is>
-      </c>
-      <c r="D35" s="36" t="n"/>
-      <c r="E35" s="37" t="n"/>
-      <c r="F35" s="36" t="inlineStr">
-        <is>
-          <t>Fournie par Gabriel</t>
-        </is>
-      </c>
-      <c r="G35" s="40" t="inlineStr">
-        <is>
-          <t>Non recoupée dans Missive</t>
-        </is>
-      </c>
-      <c r="H35" s="38" t="n"/>
-      <c r="I35" s="38" t="n"/>
-      <c r="J35" s="39" t="n"/>
-      <c r="K35" s="25" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="L35" s="25" t="inlineStr">
-        <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
-        </is>
-      </c>
-      <c r="M35" s="25" t="inlineStr">
-        <is>
-          <t>Bonjour Jessica,</t>
-        </is>
-      </c>
-      <c r="N35" s="46" t="inlineStr">
         <is>
           <t>Bonjour Mme Dostie,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque. Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe, qu'on transforme en isolant à Québec.
@@ -3481,65 +3337,65 @@
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
       </c>
-      <c r="O35" s="25" t="inlineStr">
+      <c r="O33" s="25" t="inlineStr">
         <is>
           <t>vous</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="240" customHeight="1" s="26">
-      <c r="A36" s="25" t="inlineStr">
+    <row r="34" ht="240" customHeight="1" s="26">
+      <c r="A34" s="25" t="inlineStr">
         <is>
           <t>Sophie Poisson</t>
         </is>
       </c>
-      <c r="B36" s="25" t="inlineStr">
+      <c r="B34" s="25" t="inlineStr">
         <is>
           <t>Baron Mag</t>
         </is>
       </c>
-      <c r="C36" s="25" t="inlineStr"/>
-      <c r="D36" s="25" t="inlineStr">
+      <c r="C34" s="25" t="inlineStr"/>
+      <c r="D34" s="25" t="inlineStr">
         <is>
           <t>2020-11-10</t>
         </is>
       </c>
-      <c r="E36" s="25" t="inlineStr">
+      <c r="E34" s="25" t="inlineStr">
         <is>
           <t>Lasclay : des accessoires d'hiver isoles a l'asclepiade</t>
         </is>
       </c>
-      <c r="F36" s="25" t="inlineStr">
+      <c r="F34" s="25" t="inlineStr">
         <is>
           <t>Depouillement web (page medias de lasclay.com)</t>
         </is>
       </c>
-      <c r="G36" s="25" t="inlineStr">
+      <c r="G34" s="25" t="inlineStr">
         <is>
           <t>A verifier</t>
         </is>
       </c>
-      <c r="J36" s="25" t="inlineStr">
+      <c r="J34" s="25" t="inlineStr">
         <is>
           <t>A mentionne Lasclay. Absente des 34. Courriel a trouver.</t>
         </is>
       </c>
-      <c r="K36" s="25" t="inlineStr">
+      <c r="K34" s="25" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="L36" s="25" t="inlineStr">
+      <c r="L34" s="25" t="inlineStr">
         <is>
           <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
-      <c r="M36" s="25" t="inlineStr">
+      <c r="M34" s="25" t="inlineStr">
         <is>
           <t>Bonjour Sophie,</t>
         </is>
       </c>
-      <c r="N36" s="46" t="inlineStr">
+      <c r="N34" s="46" t="inlineStr">
         <is>
           <t>Bonjour Mme Poisson,
 En novembre 2020, vous aviez présenté nos accessoires d'hiver isolés à l'asclépiade, quand il y en avait trois. Il y en a maintenant plus de 40, dont des manteaux et des vestes à inserts amovibles.
@@ -3551,65 +3407,65 @@
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
       </c>
-      <c r="O36" s="25" t="inlineStr">
+      <c r="O34" s="25" t="inlineStr">
         <is>
           <t>vous</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="240" customHeight="1" s="26">
-      <c r="A37" s="25" t="inlineStr">
+    <row r="35" ht="240" customHeight="1" s="26">
+      <c r="A35" s="25" t="inlineStr">
         <is>
           <t>Caroline Bertrand</t>
         </is>
       </c>
-      <c r="B37" s="25" t="inlineStr">
+      <c r="B35" s="25" t="inlineStr">
         <is>
           <t>ICI Explora</t>
         </is>
       </c>
-      <c r="C37" s="25" t="inlineStr"/>
-      <c r="D37" s="25" t="inlineStr">
+      <c r="C35" s="25" t="inlineStr"/>
+      <c r="D35" s="25" t="inlineStr">
         <is>
           <t>2021-09-28</t>
         </is>
       </c>
-      <c r="E37" s="25" t="inlineStr">
+      <c r="E35" s="25" t="inlineStr">
         <is>
           <t>L'asclepiade pour braver le froid</t>
         </is>
       </c>
-      <c r="F37" s="25" t="inlineStr">
+      <c r="F35" s="25" t="inlineStr">
         <is>
           <t>Depouillement web (page medias de lasclay.com)</t>
         </is>
       </c>
-      <c r="G37" s="25" t="inlineStr">
+      <c r="G35" s="25" t="inlineStr">
         <is>
           <t>A verifier</t>
         </is>
       </c>
-      <c r="J37" s="25" t="inlineStr">
+      <c r="J35" s="25" t="inlineStr">
         <is>
           <t>A mentionne Lasclay. Absente des 34. Courriel a trouver.</t>
         </is>
       </c>
-      <c r="K37" s="25" t="inlineStr">
+      <c r="K35" s="25" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="L37" s="25" t="inlineStr">
+      <c r="L35" s="25" t="inlineStr">
         <is>
           <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
-      <c r="M37" s="25" t="inlineStr">
+      <c r="M35" s="25" t="inlineStr">
         <is>
           <t>Bonjour Caroline,</t>
         </is>
       </c>
-      <c r="N37" s="46" t="inlineStr">
+      <c r="N35" s="46" t="inlineStr">
         <is>
           <t>Bonjour Mme Bertrand,
 En septembre 2021, vous aviez écrit « L'asclépiade pour braver le froid » pour ICI Explora. Depuis, le statut du monarque comme espèce en voie de disparition a été confirmé au Canada, et les États-Unis ont proposé de l'inscrire comme menacée.
@@ -3621,65 +3477,65 @@
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
       </c>
-      <c r="O37" s="25" t="inlineStr">
+      <c r="O35" s="25" t="inlineStr">
         <is>
           <t>vous</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="240" customHeight="1" s="26">
-      <c r="A38" s="25" t="inlineStr">
+    <row r="36" ht="240" customHeight="1" s="26">
+      <c r="A36" s="25" t="inlineStr">
         <is>
           <t>Karine Benoist</t>
         </is>
       </c>
-      <c r="B38" s="25" t="inlineStr">
+      <c r="B36" s="25" t="inlineStr">
         <is>
           <t>Chatelaine</t>
         </is>
       </c>
-      <c r="C38" s="25" t="inlineStr"/>
-      <c r="D38" s="25" t="inlineStr">
+      <c r="C36" s="25" t="inlineStr"/>
+      <c r="D36" s="25" t="inlineStr">
         <is>
           <t>2023-11-29</t>
         </is>
       </c>
-      <c r="E38" s="25" t="inlineStr">
+      <c r="E36" s="25" t="inlineStr">
         <is>
           <t>Cadeaux faits au Quebec : foulard d'asclepiade</t>
         </is>
       </c>
-      <c r="F38" s="25" t="inlineStr">
+      <c r="F36" s="25" t="inlineStr">
         <is>
           <t>Depouillement web (page medias de lasclay.com)</t>
         </is>
       </c>
-      <c r="G38" s="25" t="inlineStr">
+      <c r="G36" s="25" t="inlineStr">
         <is>
           <t>A verifier</t>
         </is>
       </c>
-      <c r="J38" s="25" t="inlineStr">
+      <c r="J36" s="25" t="inlineStr">
         <is>
           <t>A mentionne Lasclay. Absente des 34. Courriel a trouver.</t>
         </is>
       </c>
-      <c r="K38" s="25" t="inlineStr">
+      <c r="K36" s="25" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="L38" s="25" t="inlineStr">
+      <c r="L36" s="25" t="inlineStr">
         <is>
           <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
-      <c r="M38" s="25" t="inlineStr">
+      <c r="M36" s="25" t="inlineStr">
         <is>
           <t>Bonjour Karine,</t>
         </is>
       </c>
-      <c r="N38" s="46" t="inlineStr">
+      <c r="N36" s="46" t="inlineStr">
         <is>
           <t>Bonjour Mme Benoist,
 En novembre 2023, vous aviez retenu notre foulard d'asclépiade dans vos cadeaux faits au Québec. Une précision utile pour la prochaine fois : notre modèle manufacturier a changé en 2025, et l'assemblage des produits finis se fait maintenant en Tunisie. L'asclépiade est cultivée au Québec et l'isolant transformé à Limoilou.
@@ -3691,12 +3547,14 @@
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
       </c>
-      <c r="O38" s="25" t="inlineStr">
+      <c r="O36" s="25" t="inlineStr">
         <is>
           <t>vous</t>
         </is>
       </c>
     </row>
+    <row r="37" ht="240" customHeight="1" s="26"/>
+    <row r="38" ht="240" customHeight="1" s="26"/>
   </sheetData>
   <autoFilter ref="A1:J35"/>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>

</xml_diff>

<commit_message>
Retire les contacts sans adresse et relance Goubau sur son propre segment
Sophie Poisson, Caroline Bertrand et Karine Benoist sortent de la liste chaude,
faute d'adresse courriel. Leurs brouillons restent dans le code si leurs
adresses refont surface. La liste chaude passe à 32 contacts, toutes adresses
remplies.

Madeleine Goubau connaît l'asclépiade: elle en avait parlé à Moteur de
recherche le 9 février 2023. Son courriel le reconnaît d'entrée plutôt que de
lui présenter la plante, puis enchaîne sur ce qu'elle n'a peut-être pas vu, la
fibre une fois transformée en isolant.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015pjLsGPzf1MX1JC7QiKGGk
</commit_message>
<xml_diff>
--- a/communique-dragons/Lasclay_v2.xlsx
+++ b/communique-dragons/Lasclay_v2.xlsx
@@ -990,7 +990,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O36"/>
+  <dimension ref="A1:O33"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="26" customWidth="1" style="25" min="1" max="1"/>
@@ -3266,7 +3266,8 @@
       <c r="N32" s="46" t="inlineStr">
         <is>
           <t>Bonjour Mme Goubau,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque. Vous couvrez le textile et la mode, alors voici une matière que peu de gens ont vue de près : la soie d'asclépiade, une fibre creuse et naturellement hydrophobe attachée aux graines d'une plante que les agriculteurs arrachent de leurs champs depuis 50 ans. On la transforme en isolant, et on en fait des manteaux, des mitaines et des tuques.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe : l'asclépiade, que vous connaissez bien, puisque vous en aviez parlé à Moteur de recherche en février 2023. On la cultive pour sauvegarder un pollinisateur emblématique et menacé, le papillon monarque.
+Ce que vous n'avez peut-être pas vu de près, c'est ce que la fibre donne une fois transformée. Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe, qu'on transforme en isolant à Québec, et qui se retrouve dans des manteaux, des mitaines et des tuques.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet.
@@ -3343,218 +3344,8 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="240" customHeight="1" s="26">
-      <c r="A34" s="25" t="inlineStr">
-        <is>
-          <t>Sophie Poisson</t>
-        </is>
-      </c>
-      <c r="B34" s="25" t="inlineStr">
-        <is>
-          <t>Baron Mag</t>
-        </is>
-      </c>
-      <c r="C34" s="25" t="inlineStr"/>
-      <c r="D34" s="25" t="inlineStr">
-        <is>
-          <t>2020-11-10</t>
-        </is>
-      </c>
-      <c r="E34" s="25" t="inlineStr">
-        <is>
-          <t>Lasclay : des accessoires d'hiver isoles a l'asclepiade</t>
-        </is>
-      </c>
-      <c r="F34" s="25" t="inlineStr">
-        <is>
-          <t>Depouillement web (page medias de lasclay.com)</t>
-        </is>
-      </c>
-      <c r="G34" s="25" t="inlineStr">
-        <is>
-          <t>A verifier</t>
-        </is>
-      </c>
-      <c r="J34" s="25" t="inlineStr">
-        <is>
-          <t>A mentionne Lasclay. Absente des 34. Courriel a trouver.</t>
-        </is>
-      </c>
-      <c r="K34" s="25" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="L34" s="25" t="inlineStr">
-        <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
-        </is>
-      </c>
-      <c r="M34" s="25" t="inlineStr">
-        <is>
-          <t>Bonjour Sophie,</t>
-        </is>
-      </c>
-      <c r="N34" s="46" t="inlineStr">
-        <is>
-          <t>Bonjour Mme Poisson,
-En novembre 2020, vous aviez présenté nos accessoires d'hiver isolés à l'asclépiade, quand il y en avait trois. Il y en a maintenant plus de 40, dont des manteaux et des vestes à inserts amovibles.
-Depuis, tout mon temps va à mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
-Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
-Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer une suite à votre dernier article.
-J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
-Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
-        </is>
-      </c>
-      <c r="O34" s="25" t="inlineStr">
-        <is>
-          <t>vous</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="240" customHeight="1" s="26">
-      <c r="A35" s="25" t="inlineStr">
-        <is>
-          <t>Caroline Bertrand</t>
-        </is>
-      </c>
-      <c r="B35" s="25" t="inlineStr">
-        <is>
-          <t>ICI Explora</t>
-        </is>
-      </c>
-      <c r="C35" s="25" t="inlineStr"/>
-      <c r="D35" s="25" t="inlineStr">
-        <is>
-          <t>2021-09-28</t>
-        </is>
-      </c>
-      <c r="E35" s="25" t="inlineStr">
-        <is>
-          <t>L'asclepiade pour braver le froid</t>
-        </is>
-      </c>
-      <c r="F35" s="25" t="inlineStr">
-        <is>
-          <t>Depouillement web (page medias de lasclay.com)</t>
-        </is>
-      </c>
-      <c r="G35" s="25" t="inlineStr">
-        <is>
-          <t>A verifier</t>
-        </is>
-      </c>
-      <c r="J35" s="25" t="inlineStr">
-        <is>
-          <t>A mentionne Lasclay. Absente des 34. Courriel a trouver.</t>
-        </is>
-      </c>
-      <c r="K35" s="25" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="L35" s="25" t="inlineStr">
-        <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
-        </is>
-      </c>
-      <c r="M35" s="25" t="inlineStr">
-        <is>
-          <t>Bonjour Caroline,</t>
-        </is>
-      </c>
-      <c r="N35" s="46" t="inlineStr">
-        <is>
-          <t>Bonjour Mme Bertrand,
-En septembre 2021, vous aviez écrit « L'asclépiade pour braver le froid » pour ICI Explora. Depuis, le statut du monarque comme espèce en voie de disparition a été confirmé au Canada, et les États-Unis ont proposé de l'inscrire comme menacée.
-Depuis, tout mon temps va à mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
-Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
-Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer une suite à votre dernier article.
-J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
-Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
-        </is>
-      </c>
-      <c r="O35" s="25" t="inlineStr">
-        <is>
-          <t>vous</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="240" customHeight="1" s="26">
-      <c r="A36" s="25" t="inlineStr">
-        <is>
-          <t>Karine Benoist</t>
-        </is>
-      </c>
-      <c r="B36" s="25" t="inlineStr">
-        <is>
-          <t>Chatelaine</t>
-        </is>
-      </c>
-      <c r="C36" s="25" t="inlineStr"/>
-      <c r="D36" s="25" t="inlineStr">
-        <is>
-          <t>2023-11-29</t>
-        </is>
-      </c>
-      <c r="E36" s="25" t="inlineStr">
-        <is>
-          <t>Cadeaux faits au Quebec : foulard d'asclepiade</t>
-        </is>
-      </c>
-      <c r="F36" s="25" t="inlineStr">
-        <is>
-          <t>Depouillement web (page medias de lasclay.com)</t>
-        </is>
-      </c>
-      <c r="G36" s="25" t="inlineStr">
-        <is>
-          <t>A verifier</t>
-        </is>
-      </c>
-      <c r="J36" s="25" t="inlineStr">
-        <is>
-          <t>A mentionne Lasclay. Absente des 34. Courriel a trouver.</t>
-        </is>
-      </c>
-      <c r="K36" s="25" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="L36" s="25" t="inlineStr">
-        <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
-        </is>
-      </c>
-      <c r="M36" s="25" t="inlineStr">
-        <is>
-          <t>Bonjour Karine,</t>
-        </is>
-      </c>
-      <c r="N36" s="46" t="inlineStr">
-        <is>
-          <t>Bonjour Mme Benoist,
-En novembre 2023, vous aviez retenu notre foulard d'asclépiade dans vos cadeaux faits au Québec. Une précision utile pour la prochaine fois : notre modèle manufacturier a changé en 2025, et l'assemblage des produits finis se fait maintenant en Tunisie. L'asclépiade est cultivée au Québec et l'isolant transformé à Limoilou.
-Parmi les raisons de ce changement, il y avait clairement que j'avais besoin de temps pour me recentrer sur mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
-Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
-Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer une suite à votre dernier article.
-J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
-Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
-        </is>
-      </c>
-      <c r="O36" s="25" t="inlineStr">
-        <is>
-          <t>vous</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="240" customHeight="1" s="26"/>
-    <row r="38" ht="240" customHeight="1" s="26"/>
+    <row r="34" ht="240" customHeight="1" s="26"/>
+    <row r="35" ht="240" customHeight="1" s="26"/>
   </sheetData>
   <autoFilter ref="A1:J35"/>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>

</xml_diff>

<commit_message>
Ajoute le lien du média kit aux 247 brouillons
Le lien du dossier Drive se place juste avant la chaîne de bénéfices : un
journaliste qui envisage un sujet veut savoir tout de suite s'il aura des
images, et la question ne doit pas lui coûter un courriel.

L'offre de l'angle art de vivre devient une invitation à l'atelier — « j'ai
du matériel photo » ne veut plus rien dire une fois le dossier lié.

Les deux scripts de livraison, jusqu'ici écrits à la volée, sont versionnés :
livrable.py reconstruit le chiffrier à éditer en reprenant les colonnes que
Gabriel a remplies, artefact.py recharge les fiches dans le navigateur.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015pjLsGPzf1MX1JC7QiKGGk
</commit_message>
<xml_diff>
--- a/communique-dragons/Lasclay_v2.xlsx
+++ b/communique-dragons/Lasclay_v2.xlsx
@@ -1150,7 +1150,10 @@
 et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité
 qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer
-une suite au dernier article. J'espère vraiment un boom des ventes avec cette visibilité, ce
+une suite au dernier article.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise :
+https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+J'espère vraiment un boom des ventes avec cette visibilité, ce
 qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec
 chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se
 reproduire dans leurs plantations.
@@ -1225,6 +1228,7 @@
 Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer une suite à votre dernier article.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -1307,7 +1311,10 @@
 et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité
 qui arrive bien rarement. Je voulais t'en faire part et qui sait, peut-être t'inspirer une
-suite à ton dernier article. J'espère vraiment un boom des ventes avec cette visibilité, ce
+suite à ton dernier article.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise :
+https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+J'espère vraiment un boom des ventes avec cette visibilité, ce
 qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec
 chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se
 reproduire dans leurs plantations.
@@ -1381,6 +1388,7 @@
 Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part : je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -1453,6 +1461,7 @@
 Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer une suite à votre dernier article.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -1525,6 +1534,7 @@
 Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer une suite à votre dernier article.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -1597,6 +1607,7 @@
 Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer une suite à votre dernier article.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -1669,6 +1680,7 @@
 Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -1741,6 +1753,7 @@
 Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -1813,6 +1826,7 @@
 Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer une suite à votre dernier article.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -1885,6 +1899,7 @@
 Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -1957,6 +1972,7 @@
 Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer une suite à votre dernier article.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -2029,6 +2045,7 @@
 Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -2101,6 +2118,7 @@
 Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -2172,6 +2190,7 @@
 Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part : je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -2244,6 +2263,7 @@
 Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer une suite à votre dernier article.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -2316,6 +2336,7 @@
 Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer une suite à votre dernier article.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -2388,6 +2409,7 @@
 Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -2460,6 +2482,7 @@
 Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part : je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -2532,6 +2555,7 @@
 Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer une suite à votre dernier article.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -2604,6 +2628,7 @@
 Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer une suite à votre dernier article.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -2676,6 +2701,7 @@
 Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer une suite à votre dernier article.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -2813,6 +2839,7 @@
 Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer une suite à votre dernier article.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -2877,6 +2904,7 @@
 Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer une suite à votre dernier article.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -2940,6 +2968,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part : je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -3003,6 +3032,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part : je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -3079,6 +3109,7 @@
 Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer une suite à votre dernier article.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -3143,6 +3174,7 @@
 Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer une suite à votre dernier article.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -3207,6 +3239,7 @@
 Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer une suite à votre dernier article.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -3271,6 +3304,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -3334,6 +3368,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -3563,6 +3598,7 @@
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de
 Limoilou est ouvert si vos lecteurs aimeraient voir comment une gousse devient un manteau.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -3648,6 +3684,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -3732,7 +3769,8 @@
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière, et j'ai du matériel photo.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière de vos yeux.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -3817,6 +3855,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -3906,6 +3945,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -3991,6 +4031,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -4076,6 +4117,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -4165,6 +4207,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -4249,6 +4292,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -4338,6 +4382,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -4422,6 +4467,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -4507,6 +4553,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -4592,6 +4639,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -4681,6 +4729,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -4770,6 +4819,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -4850,6 +4900,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -4935,6 +4986,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -5020,6 +5072,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -5109,6 +5162,7 @@
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet : huit ans après
 Saint-Tite, il reste quelque chose de cette promesse-là, et ça se raconte.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -5189,6 +5243,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -5278,6 +5333,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -5362,6 +5418,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -5446,6 +5503,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -5530,6 +5588,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -5610,6 +5669,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -5694,6 +5754,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -5783,6 +5844,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -5868,6 +5930,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -5957,6 +6020,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -6046,6 +6110,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -6130,6 +6195,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -6214,6 +6280,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -6303,6 +6370,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -6392,6 +6460,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -6472,6 +6541,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -6552,6 +6622,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -6641,6 +6712,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -6721,6 +6793,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -6801,6 +6874,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -6885,6 +6959,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -6974,6 +7049,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -7054,6 +7130,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -7143,6 +7220,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -7239,6 +7317,7 @@
 Je voulais vous en faire part parce que vos lecteurs ont vu la promesse de l'asclépiade de
 plus près que n'importe qui. Qui sait, peut-être vous inspirer un sujet sur ce que la plante
 est devenue depuis. Je peux parler des volumes, de la récolte, et de ce qui reste à régler.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -7319,6 +7398,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -7404,6 +7484,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -7488,6 +7569,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -7572,6 +7654,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -7661,6 +7744,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -7750,6 +7834,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -7834,6 +7919,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -7918,6 +8004,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -7998,6 +8085,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -8087,6 +8175,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -8171,6 +8260,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -8260,6 +8350,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -8349,6 +8440,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -8434,6 +8526,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -8523,6 +8616,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -8612,6 +8706,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -8696,6 +8791,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -8780,6 +8876,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -8864,6 +8961,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -8948,6 +9046,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -9037,6 +9136,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -9126,6 +9226,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -9215,6 +9316,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -9304,6 +9406,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -9388,6 +9491,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -9473,6 +9577,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -9562,6 +9667,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -9646,7 +9752,8 @@
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière, et j'ai du matériel photo.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière de vos yeux.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -9731,6 +9838,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -9820,6 +9928,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -9905,6 +10014,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -9985,6 +10095,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -10074,6 +10185,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -10154,6 +10266,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -10238,6 +10351,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -10327,6 +10441,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -10411,6 +10526,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -10495,6 +10611,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -10579,6 +10696,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -10663,6 +10781,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -10747,6 +10866,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -10831,6 +10951,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -10911,6 +11032,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -10995,6 +11117,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -11080,6 +11203,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -11160,6 +11284,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -11249,6 +11374,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -11333,6 +11459,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -11417,6 +11544,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -11501,6 +11629,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -11590,6 +11719,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -11674,6 +11804,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -11763,6 +11894,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -11847,6 +11979,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -11936,6 +12069,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -12020,6 +12154,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -12104,6 +12239,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -12184,6 +12320,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -12268,6 +12405,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -12352,6 +12490,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -12436,6 +12575,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -12525,6 +12665,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -12609,6 +12750,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -12693,6 +12835,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -12782,6 +12925,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -12866,6 +13010,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -12950,6 +13095,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -13035,6 +13181,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -13119,6 +13266,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -13203,6 +13351,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -13292,6 +13441,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -13376,6 +13526,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -13456,6 +13607,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -13536,6 +13688,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -13616,6 +13769,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -13696,6 +13850,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler des volumes, de la fenêtre de récolte et de ce qui reste à régler côté mécanisation, sans rien promettre que je ne peux pas tenir.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -13776,6 +13931,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -13865,6 +14021,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -13949,6 +14106,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -14034,6 +14192,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -14118,6 +14277,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -14207,6 +14367,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -14292,6 +14453,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -14376,6 +14538,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -14460,7 +14623,8 @@
 Je vous écris entre autres parce que l'asclépiade se cultive dans votre région depuis la première vague de 2013, et que plusieurs des producteurs qui ont tenu bon nous vendent encore leur récolte.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière, et j'ai du matériel photo.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière de vos yeux.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -14550,6 +14714,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -14635,6 +14800,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -14718,7 +14884,8 @@
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière, et j'ai du matériel photo.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière de vos yeux.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -14803,6 +14970,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -14892,6 +15060,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -14981,6 +15150,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -15065,6 +15235,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -15150,6 +15321,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -15233,7 +15405,8 @@
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière, et j'ai du matériel photo.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière de vos yeux.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -15319,6 +15492,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -15408,6 +15582,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -15492,6 +15667,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -15581,6 +15757,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -15666,6 +15843,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -15755,6 +15933,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -15840,6 +16019,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -15928,7 +16108,8 @@
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière, et j'ai du matériel photo.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière de vos yeux.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -16012,7 +16193,8 @@
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière, et j'ai du matériel photo.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière de vos yeux.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -16098,6 +16280,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -16183,6 +16366,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Et si vous voulez tester plutôt que me croire sur parole, je vous envoie un produit avec plaisir.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -16267,6 +16451,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -16351,7 +16536,8 @@
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière, et j'ai du matériel photo.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière de vos yeux.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -16436,6 +16622,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -16525,6 +16712,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -16610,6 +16798,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -16699,6 +16888,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -16783,6 +16973,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -16868,6 +17059,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -16956,7 +17148,8 @@
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière, et j'ai du matériel photo.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière de vos yeux.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -17042,6 +17235,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -17126,6 +17320,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -17206,6 +17401,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -17290,6 +17486,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -17374,7 +17571,8 @@
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière, et j'ai du matériel photo.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière de vos yeux.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -17458,7 +17656,8 @@
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière, et j'ai du matériel photo.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière de vos yeux.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -17543,6 +17742,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -17713,6 +17913,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -17801,7 +18002,8 @@
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière, et j'ai du matériel photo.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière de vos yeux.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -17886,6 +18088,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -17975,6 +18178,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -18064,6 +18268,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -18233,7 +18438,8 @@
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière, et j'ai du matériel photo.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière de vos yeux.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -18314,6 +18520,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -18399,6 +18606,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -18488,6 +18696,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -18572,6 +18781,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -18655,7 +18865,8 @@
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière, et j'ai du matériel photo.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière de vos yeux.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -18741,6 +18952,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -18825,6 +19037,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -18910,6 +19123,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -18995,6 +19209,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -19084,6 +19299,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -19167,7 +19383,8 @@
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière, et j'ai du matériel photo.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière de vos yeux.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -19257,6 +19474,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -19345,7 +19563,8 @@
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière, et j'ai du matériel photo.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière de vos yeux.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -19431,6 +19650,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -19520,6 +19740,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -19604,6 +19825,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -19687,7 +19909,8 @@
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière, et j'ai du matériel photo.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière de vos yeux.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -19777,6 +20000,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -19861,6 +20085,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -19950,6 +20175,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -20038,7 +20264,8 @@
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière, et j'ai du matériel photo.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière de vos yeux.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -20127,7 +20354,8 @@
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière, et j'ai du matériel photo.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière de vos yeux.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -20211,7 +20439,8 @@
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière, et j'ai du matériel photo.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière de vos yeux.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -20301,6 +20530,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -20381,6 +20611,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -20465,6 +20696,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -20548,7 +20780,8 @@
 Je vous écris parce que vous couvrez l'art de vivre et la consommation. Le contraste se photographie bien : la gousse dans le champ, la soie blanche dans la main, le manteau porté en ville.
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière, et j'ai du matériel photo.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. L'atelier de Limoilou est ouvert si vous voulez voir la matière de vos yeux.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -20629,6 +20862,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -20709,6 +20943,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -20793,6 +21028,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -20873,6 +21109,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -20962,6 +21199,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -21047,6 +21285,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -21131,6 +21370,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -21211,6 +21451,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -21295,6 +21536,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -21379,6 +21621,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux parler de ce que ça demande d'industrialiser une matière qui n'a aucune chaîne d'approvisionnement.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -21464,6 +21707,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -21548,6 +21792,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -21632,6 +21877,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -21721,6 +21967,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -21805,6 +22052,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je suis disponible pour une entrevue avant ou après la diffusion.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -21889,6 +22137,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -21969,6 +22218,7 @@
 Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet. Je peux aussi parler de notre campagne de plantation, qui en est à sa 5e édition et qui a distribué environ 10 millions de graines en Amérique du Nord.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
@@ -22052,6 +22302,7 @@
 Vous êtes probablement la personne au Québec qui a le plus longtemps suivi cette plante-là.
 Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet : ce serait la
 première fois qu'on raconte ce que la filière est devenue après la chute.
+Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>

</xml_diff>

<commit_message>
Retire Mireille Roberge de la liste chaude
Elle n'avait aucun historique connu et sortait donc déjà sans remerciement.
Il reste 31 contacts chauds, dont 30 brouillons, et 249 contacts en tout.

Le compte des brouillons affiché dans la page se calcule maintenant à partir
des données au lieu d'être écrit dans le texte : un retrait de plus le
laissait faux.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015pjLsGPzf1MX1JC7QiKGGk
</commit_message>
<xml_diff>
--- a/communique-dragons/Lasclay_v2.xlsx
+++ b/communique-dragons/Lasclay_v2.xlsx
@@ -990,7 +990,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O33"/>
+  <dimension ref="A1:O32"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="26" customWidth="1" style="25" min="1" max="1"/>
@@ -2918,7 +2918,7 @@
     <row r="27" ht="240" customHeight="1" s="26">
       <c r="A27" s="36" t="inlineStr">
         <is>
-          <t>Mireille Roberge</t>
+          <t>Sophie Laforest</t>
         </is>
       </c>
       <c r="B27" s="36" t="inlineStr">
@@ -2928,7 +2928,7 @@
       </c>
       <c r="C27" s="36" t="inlineStr">
         <is>
-          <t>mireille.roberge@radio-canada.ca</t>
+          <t>sophie.laforest@radio-canada.ca</t>
         </is>
       </c>
       <c r="D27" s="36" t="n"/>
@@ -2958,74 +2958,10 @@
       </c>
       <c r="M27" s="25" t="inlineStr">
         <is>
-          <t>Bonjour Mireille,</t>
+          <t>Bonjour Sophie,</t>
         </is>
       </c>
       <c r="N27" s="46" t="inlineStr">
-        <is>
-          <t>Bonjour Mme Roberge,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque. Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe, qu'on transforme en isolant à Québec.
-Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
-Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part : je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
-Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
-J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
-Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
-        </is>
-      </c>
-      <c r="O27" s="25" t="inlineStr">
-        <is>
-          <t>vous</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="240" customHeight="1" s="26">
-      <c r="A28" s="36" t="inlineStr">
-        <is>
-          <t>Sophie Laforest</t>
-        </is>
-      </c>
-      <c r="B28" s="36" t="inlineStr">
-        <is>
-          <t>Radio-Canada</t>
-        </is>
-      </c>
-      <c r="C28" s="36" t="inlineStr">
-        <is>
-          <t>sophie.laforest@radio-canada.ca</t>
-        </is>
-      </c>
-      <c r="D28" s="36" t="n"/>
-      <c r="E28" s="37" t="n"/>
-      <c r="F28" s="36" t="inlineStr">
-        <is>
-          <t>Fournie par Gabriel</t>
-        </is>
-      </c>
-      <c r="G28" s="40" t="inlineStr">
-        <is>
-          <t>Non recoupée dans Missive</t>
-        </is>
-      </c>
-      <c r="H28" s="38" t="n"/>
-      <c r="I28" s="38" t="n"/>
-      <c r="J28" s="39" t="n"/>
-      <c r="K28" s="25" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="L28" s="25" t="inlineStr">
-        <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
-        </is>
-      </c>
-      <c r="M28" s="25" t="inlineStr">
-        <is>
-          <t>Bonjour Sophie,</t>
-        </is>
-      </c>
-      <c r="N28" s="46" t="inlineStr">
         <is>
           <t>Bonjour Mme Laforest,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque. Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe, qu'on transforme en isolant à Québec.
@@ -3037,71 +2973,71 @@
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
       </c>
-      <c r="O28" s="25" t="inlineStr">
+      <c r="O27" s="25" t="inlineStr">
         <is>
           <t>vous</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="240" customHeight="1" s="26">
-      <c r="A29" s="36" t="inlineStr">
+    <row r="28" ht="240" customHeight="1" s="26">
+      <c r="A28" s="36" t="inlineStr">
         <is>
           <t>Alain McKenna</t>
         </is>
       </c>
-      <c r="B29" s="36" t="inlineStr">
+      <c r="B28" s="36" t="inlineStr">
         <is>
           <t>Le Devoir</t>
         </is>
       </c>
-      <c r="C29" s="36" t="inlineStr">
+      <c r="C28" s="36" t="inlineStr">
         <is>
           <t>amckenna@ledevoir.com</t>
         </is>
       </c>
-      <c r="D29" s="36" t="inlineStr">
+      <c r="D28" s="36" t="inlineStr">
         <is>
           <t>2021-12-24</t>
         </is>
       </c>
-      <c r="E29" s="37" t="inlineStr">
+      <c r="E28" s="37" t="inlineStr">
         <is>
           <t>Des écouteurs de Québec pour oublier les AirPods (Sounds Good)</t>
         </is>
       </c>
-      <c r="F29" s="36" t="inlineStr">
+      <c r="F28" s="36" t="inlineStr">
         <is>
           <t>Lien fourni par Gabriel</t>
         </is>
       </c>
-      <c r="G29" s="40" t="inlineStr">
+      <c r="G28" s="40" t="inlineStr">
         <is>
           <t>Correspondance confirmée</t>
         </is>
       </c>
-      <c r="H29" s="38" t="n"/>
-      <c r="I29" s="38" t="n"/>
-      <c r="J29" s="39" t="inlineStr">
+      <c r="H28" s="38" t="n"/>
+      <c r="I28" s="38" t="n"/>
+      <c r="J28" s="39" t="inlineStr">
         <is>
           <t>A couvert Sounds Good, la première entreprise de Gabriel, à l'époque des trois associés. Gabriel a vendu ses parts en 2022 : le dire d'entrée, McKenna suit encore Sounds Good.</t>
         </is>
       </c>
-      <c r="K29" s="25" t="inlineStr">
+      <c r="K28" s="25" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="L29" s="25" t="inlineStr">
+      <c r="L28" s="25" t="inlineStr">
         <is>
           <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
-      <c r="M29" s="25" t="inlineStr">
+      <c r="M28" s="25" t="inlineStr">
         <is>
           <t>Bonjour Alain,</t>
         </is>
       </c>
-      <c r="N29" s="46" t="inlineStr">
+      <c r="N28" s="46" t="inlineStr">
         <is>
           <t>Bonjour M. McKenna,
 En décembre 2021, vous aviez écrit « Des écouteurs de Québec pour oublier les AirPods », sur Sounds Good. J'étais un des trois. J'ai vendu mes parts en 2022 pour me consacrer entièrement à Lasclay, l'autre entreprise que j'avais démarrée entretemps, qui transforme la soie d'asclépiade en isolant textile.
@@ -3115,59 +3051,59 @@
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
       </c>
-      <c r="O29" s="25" t="inlineStr">
+      <c r="O28" s="25" t="inlineStr">
         <is>
           <t>vous</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="240" customHeight="1" s="26">
-      <c r="A30" s="36" t="inlineStr">
+    <row r="29" ht="240" customHeight="1" s="26">
+      <c r="A29" s="36" t="inlineStr">
         <is>
           <t>Sylvie Lemieux</t>
         </is>
       </c>
-      <c r="B30" s="36" t="inlineStr">
+      <c r="B29" s="36" t="inlineStr">
         <is>
           <t>Pigiste</t>
         </is>
       </c>
-      <c r="C30" s="36" t="inlineStr">
+      <c r="C29" s="36" t="inlineStr">
         <is>
           <t>sylvielemieux16@gmail.com</t>
         </is>
       </c>
-      <c r="D30" s="36" t="n"/>
-      <c r="E30" s="37" t="n"/>
-      <c r="F30" s="36" t="inlineStr">
+      <c r="D29" s="36" t="n"/>
+      <c r="E29" s="37" t="n"/>
+      <c r="F29" s="36" t="inlineStr">
         <is>
           <t>Fournie par Gabriel</t>
         </is>
       </c>
-      <c r="G30" s="40" t="inlineStr">
+      <c r="G29" s="40" t="inlineStr">
         <is>
           <t>Non recoupée dans Missive</t>
         </is>
       </c>
-      <c r="H30" s="38" t="n"/>
-      <c r="I30" s="38" t="n"/>
-      <c r="J30" s="39" t="n"/>
-      <c r="K30" s="25" t="inlineStr">
+      <c r="H29" s="38" t="n"/>
+      <c r="I29" s="38" t="n"/>
+      <c r="J29" s="39" t="n"/>
+      <c r="K29" s="25" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="L30" s="25" t="inlineStr">
+      <c r="L29" s="25" t="inlineStr">
         <is>
           <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
-      <c r="M30" s="25" t="inlineStr">
+      <c r="M29" s="25" t="inlineStr">
         <is>
           <t>Bonjour Sylvie,</t>
         </is>
       </c>
-      <c r="N30" s="46" t="inlineStr">
+      <c r="N29" s="46" t="inlineStr">
         <is>
           <t>Bonjour Mme Lemieux,
 En décembre 2021, vous aviez écrit « Les deux mains dans l'écoresponsabilité » pour le Journal de Montréal. Notre modèle manufacturier a changé depuis, et j'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
@@ -3181,59 +3117,59 @@
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
       </c>
-      <c r="O30" s="25" t="inlineStr">
+      <c r="O29" s="25" t="inlineStr">
         <is>
           <t>vous</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="240" customHeight="1" s="26">
-      <c r="A31" s="36" t="inlineStr">
+    <row r="30" ht="240" customHeight="1" s="26">
+      <c r="A30" s="36" t="inlineStr">
         <is>
           <t>Sophie Grenier-Héroux</t>
         </is>
       </c>
-      <c r="B31" s="36" t="inlineStr">
+      <c r="B30" s="36" t="inlineStr">
         <is>
           <t>Pigiste</t>
         </is>
       </c>
-      <c r="C31" s="36" t="inlineStr">
+      <c r="C30" s="36" t="inlineStr">
         <is>
           <t>sophiegrenierheroux@hotmail.com</t>
         </is>
       </c>
-      <c r="D31" s="36" t="n"/>
-      <c r="E31" s="37" t="n"/>
-      <c r="F31" s="36" t="inlineStr">
+      <c r="D30" s="36" t="n"/>
+      <c r="E30" s="37" t="n"/>
+      <c r="F30" s="36" t="inlineStr">
         <is>
           <t>Fournie par Gabriel</t>
         </is>
       </c>
-      <c r="G31" s="40" t="inlineStr">
+      <c r="G30" s="40" t="inlineStr">
         <is>
           <t>Non recoupée dans Missive</t>
         </is>
       </c>
-      <c r="H31" s="38" t="n"/>
-      <c r="I31" s="38" t="n"/>
-      <c r="J31" s="39" t="n"/>
-      <c r="K31" s="25" t="inlineStr">
+      <c r="H30" s="38" t="n"/>
+      <c r="I30" s="38" t="n"/>
+      <c r="J30" s="39" t="n"/>
+      <c r="K30" s="25" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="L31" s="25" t="inlineStr">
+      <c r="L30" s="25" t="inlineStr">
         <is>
           <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
-      <c r="M31" s="25" t="inlineStr">
+      <c r="M30" s="25" t="inlineStr">
         <is>
           <t>Bonjour Sophie,</t>
         </is>
       </c>
-      <c r="N31" s="46" t="inlineStr">
+      <c r="N30" s="46" t="inlineStr">
         <is>
           <t>Bonjour Mme Grenier-Héroux,
 En janvier 2021, vous aviez écrit « La soie d'Amérique, le pari de deux ambitieux » dans Le Devoir. Le pari a six ans, et il tient : plus de 40 produits, environ 10 millions de graines distribuées, et un isolant toujours transformé à Limoilou.
@@ -3247,59 +3183,59 @@
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
       </c>
-      <c r="O31" s="25" t="inlineStr">
+      <c r="O30" s="25" t="inlineStr">
         <is>
           <t>vous</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="240" customHeight="1" s="26">
-      <c r="A32" s="36" t="inlineStr">
+    <row r="31" ht="240" customHeight="1" s="26">
+      <c r="A31" s="36" t="inlineStr">
         <is>
           <t>Madeleine Goubau</t>
         </is>
       </c>
-      <c r="B32" s="36" t="inlineStr">
+      <c r="B31" s="36" t="inlineStr">
         <is>
           <t>Pigiste</t>
         </is>
       </c>
-      <c r="C32" s="36" t="inlineStr">
+      <c r="C31" s="36" t="inlineStr">
         <is>
           <t>madeleine.goubau@gmail.com</t>
         </is>
       </c>
-      <c r="D32" s="36" t="n"/>
-      <c r="E32" s="37" t="n"/>
-      <c r="F32" s="36" t="inlineStr">
+      <c r="D31" s="36" t="n"/>
+      <c r="E31" s="37" t="n"/>
+      <c r="F31" s="36" t="inlineStr">
         <is>
           <t>Fournie par Gabriel</t>
         </is>
       </c>
-      <c r="G32" s="40" t="inlineStr">
+      <c r="G31" s="40" t="inlineStr">
         <is>
           <t>Non recoupée dans Missive</t>
         </is>
       </c>
-      <c r="H32" s="38" t="n"/>
-      <c r="I32" s="38" t="n"/>
-      <c r="J32" s="39" t="n"/>
-      <c r="K32" s="25" t="inlineStr">
+      <c r="H31" s="38" t="n"/>
+      <c r="I31" s="38" t="n"/>
+      <c r="J31" s="39" t="n"/>
+      <c r="K31" s="25" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="L32" s="25" t="inlineStr">
+      <c r="L31" s="25" t="inlineStr">
         <is>
           <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
-      <c r="M32" s="25" t="inlineStr">
+      <c r="M31" s="25" t="inlineStr">
         <is>
           <t>Bonjour Madeleine,</t>
         </is>
       </c>
-      <c r="N32" s="46" t="inlineStr">
+      <c r="N31" s="46" t="inlineStr">
         <is>
           <t>Bonjour Mme Goubau,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe : l'asclépiade, que vous connaissez bien, puisque vous en aviez parlé à Moteur de recherche en février 2023. On la cultive pour sauvegarder un pollinisateur emblématique et menacé, le papillon monarque.
@@ -3313,59 +3249,59 @@
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
       </c>
-      <c r="O32" s="25" t="inlineStr">
+      <c r="O31" s="25" t="inlineStr">
         <is>
           <t>vous</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="240" customHeight="1" s="26">
-      <c r="A33" s="36" t="inlineStr">
+    <row r="32" ht="240" customHeight="1" s="26">
+      <c r="A32" s="36" t="inlineStr">
         <is>
           <t>Jessica Dostie</t>
         </is>
       </c>
-      <c r="B33" s="36" t="inlineStr">
+      <c r="B32" s="36" t="inlineStr">
         <is>
           <t>Pigiste</t>
         </is>
       </c>
-      <c r="C33" s="36" t="inlineStr">
+      <c r="C32" s="36" t="inlineStr">
         <is>
           <t>jessica.dostie@gmail.com</t>
         </is>
       </c>
-      <c r="D33" s="36" t="n"/>
-      <c r="E33" s="37" t="n"/>
-      <c r="F33" s="36" t="inlineStr">
+      <c r="D32" s="36" t="n"/>
+      <c r="E32" s="37" t="n"/>
+      <c r="F32" s="36" t="inlineStr">
         <is>
           <t>Fournie par Gabriel</t>
         </is>
       </c>
-      <c r="G33" s="40" t="inlineStr">
+      <c r="G32" s="40" t="inlineStr">
         <is>
           <t>Non recoupée dans Missive</t>
         </is>
       </c>
-      <c r="H33" s="38" t="n"/>
-      <c r="I33" s="38" t="n"/>
-      <c r="J33" s="39" t="n"/>
-      <c r="K33" s="25" t="inlineStr">
+      <c r="H32" s="38" t="n"/>
+      <c r="I32" s="38" t="n"/>
+      <c r="J32" s="39" t="n"/>
+      <c r="K32" s="25" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="L33" s="25" t="inlineStr">
+      <c r="L32" s="25" t="inlineStr">
         <is>
           <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
-      <c r="M33" s="25" t="inlineStr">
+      <c r="M32" s="25" t="inlineStr">
         <is>
           <t>Bonjour Jessica,</t>
         </is>
       </c>
-      <c r="N33" s="46" t="inlineStr">
+      <c r="N32" s="46" t="inlineStr">
         <is>
           <t>Bonjour Mme Dostie,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque. Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe, qu'on transforme en isolant à Québec.
@@ -3377,12 +3313,13 @@
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
       </c>
-      <c r="O33" s="25" t="inlineStr">
+      <c r="O32" s="25" t="inlineStr">
         <is>
           <t>vous</t>
         </is>
       </c>
     </row>
+    <row r="33" ht="240" customHeight="1" s="26"/>
     <row r="34" ht="240" customHeight="1" s="26"/>
     <row r="35" ht="240" customHeight="1" s="26"/>
   </sheetData>

</xml_diff>

<commit_message>
Reprend la version de Gabriel pour Goubau et retire Jessica Dostie
Troisième courriel réécrit par Gabriel, et la leçon dépasse le destinataire :
sans historique connu, la présentation tient en une phrase. Le paragraphe des
deux missions saute au profit de « depuis 5 ans, on travaille fort à la faire
connaître », celui sur la fibre transformée disparaît, et le remerciement
forcé aussi — on ne remercie pas quelqu'un pour un segment de radio quand le
courriel sert à annoncer une nouvelle.

Sophie Laforest, le dernier contact sans historique, est réécrite sur ce même
squelette, avec sa demande d'entrevue plutôt que de sujet.

Il reste 30 contacts chauds, 29 brouillons, 248 contacts en tout.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015pjLsGPzf1MX1JC7QiKGGk
</commit_message>
<xml_diff>
--- a/communique-dragons/Lasclay_v2.xlsx
+++ b/communique-dragons/Lasclay_v2.xlsx
@@ -990,7 +990,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O32"/>
+  <dimension ref="A1:O31"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="26" customWidth="1" style="25" min="1" max="1"/>
@@ -2964,10 +2964,10 @@
       <c r="N27" s="46" t="inlineStr">
         <is>
           <t>Bonjour Mme Laforest,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque. Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe, qu'on transforme en isolant à Québec.
-Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
-Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part : je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe : l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé, le papillon monarque.
+Depuis 5 ans, on travaille fort à la faire connaître et le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
+Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
+Aller parler de cette fibre québécoise unique à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part : je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
 Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
@@ -3238,12 +3238,10 @@
       <c r="N31" s="46" t="inlineStr">
         <is>
           <t>Bonjour Mme Goubau,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe : l'asclépiade, que vous connaissez bien, puisque vous en aviez parlé à Moteur de recherche en février 2023. On la cultive pour sauvegarder un pollinisateur emblématique et menacé, le papillon monarque.
-Ce que vous n'avez peut-être pas vu de près, c'est ce que la fibre donne une fois transformée. Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe, qu'on transforme en isolant à Québec, et qui se retrouve dans des manteaux, des mitaines et des tuques.
-Merci d'en avoir parlé en ondes, d'ailleurs : c'est rare qu'on explique la plante avant de vendre quoi que ce soit.
-Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
-Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet.
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe : l'asclépiade, que vous connaissez bien je pense.
+Depuis 5 ans, on travaille fort à la faire connaître et le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
+Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
+Aller parler de cette fibre québécoise unique à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet.
 Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
@@ -3255,70 +3253,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="240" customHeight="1" s="26">
-      <c r="A32" s="36" t="inlineStr">
-        <is>
-          <t>Jessica Dostie</t>
-        </is>
-      </c>
-      <c r="B32" s="36" t="inlineStr">
-        <is>
-          <t>Pigiste</t>
-        </is>
-      </c>
-      <c r="C32" s="36" t="inlineStr">
-        <is>
-          <t>jessica.dostie@gmail.com</t>
-        </is>
-      </c>
-      <c r="D32" s="36" t="n"/>
-      <c r="E32" s="37" t="n"/>
-      <c r="F32" s="36" t="inlineStr">
-        <is>
-          <t>Fournie par Gabriel</t>
-        </is>
-      </c>
-      <c r="G32" s="40" t="inlineStr">
-        <is>
-          <t>Non recoupée dans Missive</t>
-        </is>
-      </c>
-      <c r="H32" s="38" t="n"/>
-      <c r="I32" s="38" t="n"/>
-      <c r="J32" s="39" t="n"/>
-      <c r="K32" s="25" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="L32" s="25" t="inlineStr">
-        <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
-        </is>
-      </c>
-      <c r="M32" s="25" t="inlineStr">
-        <is>
-          <t>Bonjour Jessica,</t>
-        </is>
-      </c>
-      <c r="N32" s="46" t="inlineStr">
-        <is>
-          <t>Bonjour Mme Dostie,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque. Ses gousses sont remplies d'une soie creuse, très légère et naturellement hydrophobe, qu'on transforme en isolant à Québec.
-Le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
-Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet.
-Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
-J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
-Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
-        </is>
-      </c>
-      <c r="O32" s="25" t="inlineStr">
-        <is>
-          <t>vous</t>
-        </is>
-      </c>
-    </row>
+    <row r="32" ht="240" customHeight="1" s="26"/>
     <row r="33" ht="240" customHeight="1" s="26"/>
     <row r="34" ht="240" customHeight="1" s="26"/>
     <row r="35" ht="240" customHeight="1" s="26"/>

</xml_diff>

<commit_message>
Retire Raphaëlle Drouin de la liste chaude
247 contacts, 28 brouillons chauds, 244 liens du média kit.

Les comptes du sommaire du chiffrier se calculent maintenant à partir des
données. Trois sorties de suite les avaient laissés faux, et un chiffre faux
dans un sommaire vaut moins que pas de sommaire.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015pjLsGPzf1MX1JC7QiKGGk
</commit_message>
<xml_diff>
--- a/communique-dragons/Lasclay_v2.xlsx
+++ b/communique-dragons/Lasclay_v2.xlsx
@@ -990,7 +990,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O31"/>
+  <dimension ref="A1:O30"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="26" customWidth="1" style="25" min="1" max="1"/>
@@ -2778,37 +2778,29 @@
     <row r="25" ht="240" customHeight="1" s="26">
       <c r="A25" s="36" t="inlineStr">
         <is>
-          <t>Raphaëlle Drouin</t>
+          <t>G. Roy</t>
         </is>
       </c>
       <c r="B25" s="36" t="inlineStr">
         <is>
-          <t>URBANIA</t>
+          <t>Le Quotidien</t>
         </is>
       </c>
       <c r="C25" s="36" t="inlineStr">
         <is>
-          <t>raphaelle.drouin@urbania.ca</t>
-        </is>
-      </c>
-      <c r="D25" s="36" t="inlineStr">
-        <is>
-          <t>2020-11-24</t>
-        </is>
-      </c>
-      <c r="E25" s="37" t="inlineStr">
-        <is>
-          <t>Entrevue URBANIA</t>
-        </is>
-      </c>
+          <t>groy@lequotidien.com</t>
+        </is>
+      </c>
+      <c r="D25" s="36" t="n"/>
+      <c r="E25" s="37" t="n"/>
       <c r="F25" s="36" t="inlineStr">
         <is>
-          <t>Missive — boîte LAS Media</t>
-        </is>
-      </c>
-      <c r="G25" s="36" t="inlineStr">
-        <is>
-          <t>Correspondance confirmée</t>
+          <t>Fournie par Gabriel</t>
+        </is>
+      </c>
+      <c r="G25" s="40" t="inlineStr">
+        <is>
+          <t>Non recoupée dans Missive</t>
         </is>
       </c>
       <c r="H25" s="38" t="n"/>
@@ -2826,76 +2818,10 @@
       </c>
       <c r="M25" s="25" t="inlineStr">
         <is>
-          <t>Bonjour Raphaëlle,</t>
+          <t>Bonjour,</t>
         </is>
       </c>
       <c r="N25" s="46" t="inlineStr">
-        <is>
-          <t>Bonjour Mme Drouin,
-En janvier 2021, vous aviez écrit « Devenir viral avant même de se lancer en affaires ». Six ans plus tard, l'entreprise existe pour vrai, avec plus de 40 produits.
-Merci d'avoir écrit sur nous quand il n'y avait littéralement rien à acheter. Vous nous avez pris au sérieux avant tout le monde.
-Depuis, tout mon temps va à mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
-Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
-Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer une suite à votre dernier article.
-Notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
-J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
-Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
-        </is>
-      </c>
-      <c r="O25" s="25" t="inlineStr">
-        <is>
-          <t>vous</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="240" customHeight="1" s="26">
-      <c r="A26" s="36" t="inlineStr">
-        <is>
-          <t>G. Roy</t>
-        </is>
-      </c>
-      <c r="B26" s="36" t="inlineStr">
-        <is>
-          <t>Le Quotidien</t>
-        </is>
-      </c>
-      <c r="C26" s="36" t="inlineStr">
-        <is>
-          <t>groy@lequotidien.com</t>
-        </is>
-      </c>
-      <c r="D26" s="36" t="n"/>
-      <c r="E26" s="37" t="n"/>
-      <c r="F26" s="36" t="inlineStr">
-        <is>
-          <t>Fournie par Gabriel</t>
-        </is>
-      </c>
-      <c r="G26" s="40" t="inlineStr">
-        <is>
-          <t>Non recoupée dans Missive</t>
-        </is>
-      </c>
-      <c r="H26" s="38" t="n"/>
-      <c r="I26" s="38" t="n"/>
-      <c r="J26" s="39" t="n"/>
-      <c r="K26" s="25" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="L26" s="25" t="inlineStr">
-        <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
-        </is>
-      </c>
-      <c r="M26" s="25" t="inlineStr">
-        <is>
-          <t>Bonjour,</t>
-        </is>
-      </c>
-      <c r="N26" s="46" t="inlineStr">
         <is>
           <t>Bonjour M. Roy,
 En octobre 2020, vous avez écrit « La deuxième vie de l'asclépiade ». Vous avez été le tout premier journaliste à parler de nous. Et l'agriculteur du Lac-Saint-Jean qui vous avait donné envie du sujet est encore notre fournisseur aujourd'hui : six ans plus tard, l'asclépiade de chez vous se retrouve toujours dans nos produits.
@@ -2909,59 +2835,59 @@
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
       </c>
-      <c r="O26" s="25" t="inlineStr">
+      <c r="O25" s="25" t="inlineStr">
         <is>
           <t>vous</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="240" customHeight="1" s="26">
-      <c r="A27" s="36" t="inlineStr">
+    <row r="26" ht="240" customHeight="1" s="26">
+      <c r="A26" s="36" t="inlineStr">
         <is>
           <t>Sophie Laforest</t>
         </is>
       </c>
-      <c r="B27" s="36" t="inlineStr">
+      <c r="B26" s="36" t="inlineStr">
         <is>
           <t>Radio-Canada</t>
         </is>
       </c>
-      <c r="C27" s="36" t="inlineStr">
+      <c r="C26" s="36" t="inlineStr">
         <is>
           <t>sophie.laforest@radio-canada.ca</t>
         </is>
       </c>
-      <c r="D27" s="36" t="n"/>
-      <c r="E27" s="37" t="n"/>
-      <c r="F27" s="36" t="inlineStr">
+      <c r="D26" s="36" t="n"/>
+      <c r="E26" s="37" t="n"/>
+      <c r="F26" s="36" t="inlineStr">
         <is>
           <t>Fournie par Gabriel</t>
         </is>
       </c>
-      <c r="G27" s="40" t="inlineStr">
+      <c r="G26" s="40" t="inlineStr">
         <is>
           <t>Non recoupée dans Missive</t>
         </is>
       </c>
-      <c r="H27" s="38" t="n"/>
-      <c r="I27" s="38" t="n"/>
-      <c r="J27" s="39" t="n"/>
-      <c r="K27" s="25" t="inlineStr">
+      <c r="H26" s="38" t="n"/>
+      <c r="I26" s="38" t="n"/>
+      <c r="J26" s="39" t="n"/>
+      <c r="K26" s="25" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="L27" s="25" t="inlineStr">
+      <c r="L26" s="25" t="inlineStr">
         <is>
           <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
-      <c r="M27" s="25" t="inlineStr">
+      <c r="M26" s="25" t="inlineStr">
         <is>
           <t>Bonjour Sophie,</t>
         </is>
       </c>
-      <c r="N27" s="46" t="inlineStr">
+      <c r="N26" s="46" t="inlineStr">
         <is>
           <t>Bonjour Mme Laforest,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe : l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé, le papillon monarque.
@@ -2973,71 +2899,71 @@
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
       </c>
-      <c r="O27" s="25" t="inlineStr">
+      <c r="O26" s="25" t="inlineStr">
         <is>
           <t>vous</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="240" customHeight="1" s="26">
-      <c r="A28" s="36" t="inlineStr">
+    <row r="27" ht="240" customHeight="1" s="26">
+      <c r="A27" s="36" t="inlineStr">
         <is>
           <t>Alain McKenna</t>
         </is>
       </c>
-      <c r="B28" s="36" t="inlineStr">
+      <c r="B27" s="36" t="inlineStr">
         <is>
           <t>Le Devoir</t>
         </is>
       </c>
-      <c r="C28" s="36" t="inlineStr">
+      <c r="C27" s="36" t="inlineStr">
         <is>
           <t>amckenna@ledevoir.com</t>
         </is>
       </c>
-      <c r="D28" s="36" t="inlineStr">
+      <c r="D27" s="36" t="inlineStr">
         <is>
           <t>2021-12-24</t>
         </is>
       </c>
-      <c r="E28" s="37" t="inlineStr">
+      <c r="E27" s="37" t="inlineStr">
         <is>
           <t>Des écouteurs de Québec pour oublier les AirPods (Sounds Good)</t>
         </is>
       </c>
-      <c r="F28" s="36" t="inlineStr">
+      <c r="F27" s="36" t="inlineStr">
         <is>
           <t>Lien fourni par Gabriel</t>
         </is>
       </c>
-      <c r="G28" s="40" t="inlineStr">
+      <c r="G27" s="40" t="inlineStr">
         <is>
           <t>Correspondance confirmée</t>
         </is>
       </c>
-      <c r="H28" s="38" t="n"/>
-      <c r="I28" s="38" t="n"/>
-      <c r="J28" s="39" t="inlineStr">
+      <c r="H27" s="38" t="n"/>
+      <c r="I27" s="38" t="n"/>
+      <c r="J27" s="39" t="inlineStr">
         <is>
           <t>A couvert Sounds Good, la première entreprise de Gabriel, à l'époque des trois associés. Gabriel a vendu ses parts en 2022 : le dire d'entrée, McKenna suit encore Sounds Good.</t>
         </is>
       </c>
-      <c r="K28" s="25" t="inlineStr">
+      <c r="K27" s="25" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="L28" s="25" t="inlineStr">
+      <c r="L27" s="25" t="inlineStr">
         <is>
           <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
-      <c r="M28" s="25" t="inlineStr">
+      <c r="M27" s="25" t="inlineStr">
         <is>
           <t>Bonjour Alain,</t>
         </is>
       </c>
-      <c r="N28" s="46" t="inlineStr">
+      <c r="N27" s="46" t="inlineStr">
         <is>
           <t>Bonjour M. McKenna,
 En décembre 2021, vous aviez écrit « Des écouteurs de Québec pour oublier les AirPods », sur Sounds Good. J'étais un des trois. J'ai vendu mes parts en 2022 pour me consacrer entièrement à Lasclay, l'autre entreprise que j'avais démarrée entretemps, qui transforme la soie d'asclépiade en isolant textile.
@@ -3051,59 +2977,59 @@
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
       </c>
-      <c r="O28" s="25" t="inlineStr">
+      <c r="O27" s="25" t="inlineStr">
         <is>
           <t>vous</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="240" customHeight="1" s="26">
-      <c r="A29" s="36" t="inlineStr">
+    <row r="28" ht="240" customHeight="1" s="26">
+      <c r="A28" s="36" t="inlineStr">
         <is>
           <t>Sylvie Lemieux</t>
         </is>
       </c>
-      <c r="B29" s="36" t="inlineStr">
+      <c r="B28" s="36" t="inlineStr">
         <is>
           <t>Pigiste</t>
         </is>
       </c>
-      <c r="C29" s="36" t="inlineStr">
+      <c r="C28" s="36" t="inlineStr">
         <is>
           <t>sylvielemieux16@gmail.com</t>
         </is>
       </c>
-      <c r="D29" s="36" t="n"/>
-      <c r="E29" s="37" t="n"/>
-      <c r="F29" s="36" t="inlineStr">
+      <c r="D28" s="36" t="n"/>
+      <c r="E28" s="37" t="n"/>
+      <c r="F28" s="36" t="inlineStr">
         <is>
           <t>Fournie par Gabriel</t>
         </is>
       </c>
-      <c r="G29" s="40" t="inlineStr">
+      <c r="G28" s="40" t="inlineStr">
         <is>
           <t>Non recoupée dans Missive</t>
         </is>
       </c>
-      <c r="H29" s="38" t="n"/>
-      <c r="I29" s="38" t="n"/>
-      <c r="J29" s="39" t="n"/>
-      <c r="K29" s="25" t="inlineStr">
+      <c r="H28" s="38" t="n"/>
+      <c r="I28" s="38" t="n"/>
+      <c r="J28" s="39" t="n"/>
+      <c r="K28" s="25" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="L29" s="25" t="inlineStr">
+      <c r="L28" s="25" t="inlineStr">
         <is>
           <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
-      <c r="M29" s="25" t="inlineStr">
+      <c r="M28" s="25" t="inlineStr">
         <is>
           <t>Bonjour Sylvie,</t>
         </is>
       </c>
-      <c r="N29" s="46" t="inlineStr">
+      <c r="N28" s="46" t="inlineStr">
         <is>
           <t>Bonjour Mme Lemieux,
 En décembre 2021, vous aviez écrit « Les deux mains dans l'écoresponsabilité » pour le Journal de Montréal. Notre modèle manufacturier a changé depuis, et j'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
@@ -3117,59 +3043,59 @@
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
       </c>
-      <c r="O29" s="25" t="inlineStr">
+      <c r="O28" s="25" t="inlineStr">
         <is>
           <t>vous</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="240" customHeight="1" s="26">
-      <c r="A30" s="36" t="inlineStr">
+    <row r="29" ht="240" customHeight="1" s="26">
+      <c r="A29" s="36" t="inlineStr">
         <is>
           <t>Sophie Grenier-Héroux</t>
         </is>
       </c>
-      <c r="B30" s="36" t="inlineStr">
+      <c r="B29" s="36" t="inlineStr">
         <is>
           <t>Pigiste</t>
         </is>
       </c>
-      <c r="C30" s="36" t="inlineStr">
+      <c r="C29" s="36" t="inlineStr">
         <is>
           <t>sophiegrenierheroux@hotmail.com</t>
         </is>
       </c>
-      <c r="D30" s="36" t="n"/>
-      <c r="E30" s="37" t="n"/>
-      <c r="F30" s="36" t="inlineStr">
+      <c r="D29" s="36" t="n"/>
+      <c r="E29" s="37" t="n"/>
+      <c r="F29" s="36" t="inlineStr">
         <is>
           <t>Fournie par Gabriel</t>
         </is>
       </c>
-      <c r="G30" s="40" t="inlineStr">
+      <c r="G29" s="40" t="inlineStr">
         <is>
           <t>Non recoupée dans Missive</t>
         </is>
       </c>
-      <c r="H30" s="38" t="n"/>
-      <c r="I30" s="38" t="n"/>
-      <c r="J30" s="39" t="n"/>
-      <c r="K30" s="25" t="inlineStr">
+      <c r="H29" s="38" t="n"/>
+      <c r="I29" s="38" t="n"/>
+      <c r="J29" s="39" t="n"/>
+      <c r="K29" s="25" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="L30" s="25" t="inlineStr">
+      <c r="L29" s="25" t="inlineStr">
         <is>
           <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
-      <c r="M30" s="25" t="inlineStr">
+      <c r="M29" s="25" t="inlineStr">
         <is>
           <t>Bonjour Sophie,</t>
         </is>
       </c>
-      <c r="N30" s="46" t="inlineStr">
+      <c r="N29" s="46" t="inlineStr">
         <is>
           <t>Bonjour Mme Grenier-Héroux,
 En janvier 2021, vous aviez écrit « La soie d'Amérique, le pari de deux ambitieux » dans Le Devoir. Le pari a six ans, et il tient : plus de 40 produits, environ 10 millions de graines distribuées, et un isolant toujours transformé à Limoilou.
@@ -3183,59 +3109,59 @@
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
       </c>
-      <c r="O30" s="25" t="inlineStr">
+      <c r="O29" s="25" t="inlineStr">
         <is>
           <t>vous</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="240" customHeight="1" s="26">
-      <c r="A31" s="36" t="inlineStr">
+    <row r="30" ht="240" customHeight="1" s="26">
+      <c r="A30" s="36" t="inlineStr">
         <is>
           <t>Madeleine Goubau</t>
         </is>
       </c>
-      <c r="B31" s="36" t="inlineStr">
+      <c r="B30" s="36" t="inlineStr">
         <is>
           <t>Pigiste</t>
         </is>
       </c>
-      <c r="C31" s="36" t="inlineStr">
+      <c r="C30" s="36" t="inlineStr">
         <is>
           <t>madeleine.goubau@gmail.com</t>
         </is>
       </c>
-      <c r="D31" s="36" t="n"/>
-      <c r="E31" s="37" t="n"/>
-      <c r="F31" s="36" t="inlineStr">
+      <c r="D30" s="36" t="n"/>
+      <c r="E30" s="37" t="n"/>
+      <c r="F30" s="36" t="inlineStr">
         <is>
           <t>Fournie par Gabriel</t>
         </is>
       </c>
-      <c r="G31" s="40" t="inlineStr">
+      <c r="G30" s="40" t="inlineStr">
         <is>
           <t>Non recoupée dans Missive</t>
         </is>
       </c>
-      <c r="H31" s="38" t="n"/>
-      <c r="I31" s="38" t="n"/>
-      <c r="J31" s="39" t="n"/>
-      <c r="K31" s="25" t="inlineStr">
+      <c r="H30" s="38" t="n"/>
+      <c r="I30" s="38" t="n"/>
+      <c r="J30" s="39" t="n"/>
+      <c r="K30" s="25" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="L31" s="25" t="inlineStr">
+      <c r="L30" s="25" t="inlineStr">
         <is>
           <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
-      <c r="M31" s="25" t="inlineStr">
+      <c r="M30" s="25" t="inlineStr">
         <is>
           <t>Bonjour Madeleine,</t>
         </is>
       </c>
-      <c r="N31" s="46" t="inlineStr">
+      <c r="N30" s="46" t="inlineStr">
         <is>
           <t>Bonjour Mme Goubau,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe : l'asclépiade, que vous connaissez bien je pense.
@@ -3247,12 +3173,13 @@
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
       </c>
-      <c r="O31" s="25" t="inlineStr">
+      <c r="O30" s="25" t="inlineStr">
         <is>
           <t>vous</t>
         </is>
       </c>
     </row>
+    <row r="31" ht="240" customHeight="1" s="26"/>
     <row r="32" ht="240" customHeight="1" s="26"/>
     <row r="33" ht="240" customHeight="1" s="26"/>
     <row r="34" ht="240" customHeight="1" s="26"/>

</xml_diff>

<commit_message>
Retire Rhéane Portelance et Anaïs Elboujdaini de la liste chaude
24 brouillons chauds, 242 contacts.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015pjLsGPzf1MX1JC7QiKGGk
</commit_message>
<xml_diff>
--- a/communique-dragons/Lasclay_v2.xlsx
+++ b/communique-dragons/Lasclay_v2.xlsx
@@ -990,7 +990,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O28"/>
+  <dimension ref="A1:O26"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="26" customWidth="1" style="25" min="1" max="1"/>
@@ -1958,27 +1958,27 @@
     <row r="14" ht="240" customHeight="1" s="26">
       <c r="A14" s="36" t="inlineStr">
         <is>
-          <t>Rhéane Portelance</t>
+          <t>Marc Tison</t>
         </is>
       </c>
       <c r="B14" s="36" t="inlineStr">
         <is>
-          <t>Le Devoir</t>
+          <t>La Presse</t>
         </is>
       </c>
       <c r="C14" s="36" t="inlineStr">
         <is>
-          <t>rportelance@ledevoir.com</t>
+          <t>mtison1@lapresse.ca</t>
         </is>
       </c>
       <c r="D14" s="36" t="inlineStr">
         <is>
-          <t>2022-07-26</t>
+          <t>2021-09-20</t>
         </is>
       </c>
       <c r="E14" s="37" t="inlineStr">
         <is>
-          <t>Cahier spécial Action climatique</t>
+          <t>Entrevue — section Affaires</t>
         </is>
       </c>
       <c r="F14" s="36" t="inlineStr">
@@ -2006,17 +2006,17 @@
       </c>
       <c r="M14" s="25" t="inlineStr">
         <is>
-          <t>Bonjour Rhéane,</t>
+          <t>Bonjour Marc,</t>
         </is>
       </c>
       <c r="N14" s="46" t="inlineStr">
         <is>
-          <t>Bonjour Mme Portelance,
-On avait échangé en juillet 2022 pour le cahier Action climatique. L'asclépiade est une vivace indigène qui se cultive avec peu d'intrants et qui stocke du carbone dans un système racinaire pérenne. Merci de l'intérêt que vous nous aviez porté.
-On se concentre sur nos 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+          <t>Bonjour M. Tison,
+On s'était parlé pour la section Affaires en septembre 2021, à l'époque où on venait de rapatrier notre production faute de sous-traitant prêt à toucher à la fibre. Le modèle a changé depuis : la vidéo est ici, https://www.youtube.com/watch?v=GKyHh-Ok9JU, et Sylvain Larocque en a parlé en mai. Merci encore : le texte a beaucoup circulé chez nos clients.
+Parmi les raisons de ce changement, il y avait clairement que j'avais besoin de temps pour me recentrer sur mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer une suite à votre dernier article.
 Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
@@ -2031,27 +2031,27 @@
     <row r="15" ht="240" customHeight="1" s="26">
       <c r="A15" s="36" t="inlineStr">
         <is>
-          <t>Anaïs Elboujdaini</t>
+          <t>Valérie Simard</t>
         </is>
       </c>
       <c r="B15" s="36" t="inlineStr">
         <is>
-          <t>Bell Média</t>
+          <t>La Presse</t>
         </is>
       </c>
       <c r="C15" s="36" t="inlineStr">
         <is>
-          <t>anais.elboujdaini@bellmedia.ca</t>
+          <t>vsimard@lapresse.ca</t>
         </is>
       </c>
       <c r="D15" s="36" t="inlineStr">
         <is>
-          <t>2022-05-10</t>
+          <t>2021-09-17</t>
         </is>
       </c>
       <c r="E15" s="37" t="inlineStr">
         <is>
-          <t>Entrevue — programme de semences d'asclépiade</t>
+          <t>Demande média</t>
         </is>
       </c>
       <c r="F15" s="36" t="inlineStr">
@@ -2069,26 +2069,25 @@
       <c r="J15" s="39" t="n"/>
       <c r="K15" s="25" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>A</t>
         </is>
       </c>
       <c r="L15" s="25" t="inlineStr">
         <is>
-          <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="M15" s="25" t="inlineStr">
         <is>
-          <t>Bonjour Anaïs,</t>
+          <t>Bonjour Valérie,</t>
         </is>
       </c>
       <c r="N15" s="46" t="inlineStr">
         <is>
-          <t>Bonjour Mme Elboujdaini,
-On s'était parlé du programme de semences en mai 2022. La Campagne nationale de plantation en est à sa 5e édition, et on a distribué environ 10 millions de graines d'asclépiade en Amérique du Nord. Merci d'avoir parlé du programme de semences.
-Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
-Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part : je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
+          <t>Bonjour Mme Simard,
+Vous aviez présenté nos mitaines isolées à l'asclépiade le 17 septembre 2021. Merci pour ce coup de pouce de la première heure.
+Nous avons fait beaucoup de chemin depuis et le 17 septembre prochain, on va faire un autre énorme pas dans la bonne direction : Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer une suite à votre dernier article.
 Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
@@ -2103,27 +2102,27 @@
     <row r="16" ht="240" customHeight="1" s="26">
       <c r="A16" s="36" t="inlineStr">
         <is>
-          <t>Marc Tison</t>
+          <t>Alex Perreault</t>
         </is>
       </c>
       <c r="B16" s="36" t="inlineStr">
         <is>
-          <t>La Presse</t>
+          <t>Radio-Canada</t>
         </is>
       </c>
       <c r="C16" s="36" t="inlineStr">
         <is>
-          <t>mtison1@lapresse.ca</t>
+          <t>alex.perreault@radio-canada.ca</t>
         </is>
       </c>
       <c r="D16" s="36" t="inlineStr">
         <is>
-          <t>2021-09-20</t>
+          <t>2021-07-22</t>
         </is>
       </c>
       <c r="E16" s="37" t="inlineStr">
         <is>
-          <t>Entrevue — section Affaires</t>
+          <t>Entrevue Radio-Canada</t>
         </is>
       </c>
       <c r="F16" s="36" t="inlineStr">
@@ -2151,17 +2150,17 @@
       </c>
       <c r="M16" s="25" t="inlineStr">
         <is>
-          <t>Bonjour Marc,</t>
+          <t>Bonjour Alex,</t>
         </is>
       </c>
       <c r="N16" s="46" t="inlineStr">
         <is>
-          <t>Bonjour M. Tison,
-On s'était parlé pour la section Affaires en septembre 2021, à l'époque où on venait de rapatrier notre production faute de sous-traitant prêt à toucher à la fibre. Le modèle a changé depuis : la vidéo est ici, https://www.youtube.com/watch?v=GKyHh-Ok9JU, et Sylvain Larocque en a parlé en mai. Merci encore : le texte a beaucoup circulé chez nos clients.
-Parmi les raisons de ce changement, il y avait clairement que j'avais besoin de temps pour me recentrer sur mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+          <t>Bonjour M. Perreault,
+On s'était parlé en juillet 2021. Merci de l'intérêt que vous nous aviez porté à l'époque : on partait de zéro.
+On se concentre sur nos 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer une suite à votre dernier article.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part : je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
 Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
@@ -2176,27 +2175,27 @@
     <row r="17" ht="240" customHeight="1" s="26">
       <c r="A17" s="36" t="inlineStr">
         <is>
-          <t>Valérie Simard</t>
+          <t>Fanny Samson</t>
         </is>
       </c>
       <c r="B17" s="36" t="inlineStr">
         <is>
-          <t>La Presse</t>
+          <t>Radio-Canada</t>
         </is>
       </c>
       <c r="C17" s="36" t="inlineStr">
         <is>
-          <t>vsimard@lapresse.ca</t>
+          <t>fanny.samson@radio-canada.ca</t>
         </is>
       </c>
       <c r="D17" s="36" t="inlineStr">
         <is>
-          <t>2021-09-17</t>
+          <t>2021-03-13</t>
         </is>
       </c>
       <c r="E17" s="37" t="inlineStr">
         <is>
-          <t>Demande média</t>
+          <t>Reportage</t>
         </is>
       </c>
       <c r="F17" s="36" t="inlineStr">
@@ -2224,14 +2223,16 @@
       </c>
       <c r="M17" s="25" t="inlineStr">
         <is>
-          <t>Bonjour Valérie,</t>
+          <t>Bonjour Fanny,</t>
         </is>
       </c>
       <c r="N17" s="46" t="inlineStr">
         <is>
-          <t>Bonjour Mme Simard,
-Vous aviez présenté nos mitaines isolées à l'asclépiade le 17 septembre 2021. Merci pour ce coup de pouce de la première heure.
-Nous avons fait beaucoup de chemin depuis et le 17 septembre prochain, on va faire un autre énorme pas dans la bonne direction : Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
+          <t>Bonjour Mme Samson,
+En mars 2021, vous aviez signé « Les grandes promesses de l'asclépiade, la soie d'Amérique ». Cinq ans plus tard, je peux vous dire lesquelles ont été tenues : il y a des produits finis, l'isolant se transforme toujours au Québec, on achète encore de l'asclépiade québécoise, et un manteau Lasclay se vend au prix très abordable de 300 $.
+On se concentre sur nos 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
+Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer une suite à votre dernier article.
 Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
@@ -2247,27 +2248,27 @@
     <row r="18" ht="240" customHeight="1" s="26">
       <c r="A18" s="36" t="inlineStr">
         <is>
-          <t>Alex Perreault</t>
+          <t>Martin Ménard</t>
         </is>
       </c>
       <c r="B18" s="36" t="inlineStr">
         <is>
-          <t>Radio-Canada</t>
+          <t>La Terre de chez nous</t>
         </is>
       </c>
       <c r="C18" s="36" t="inlineStr">
         <is>
-          <t>alex.perreault@radio-canada.ca</t>
+          <t>mmenard@laterre.ca</t>
         </is>
       </c>
       <c r="D18" s="36" t="inlineStr">
         <is>
-          <t>2021-07-22</t>
+          <t>2021-01-26</t>
         </is>
       </c>
       <c r="E18" s="37" t="inlineStr">
         <is>
-          <t>Entrevue Radio-Canada</t>
+          <t>Entrevue La Terre</t>
         </is>
       </c>
       <c r="F18" s="36" t="inlineStr">
@@ -2295,17 +2296,17 @@
       </c>
       <c r="M18" s="25" t="inlineStr">
         <is>
-          <t>Bonjour Alex,</t>
+          <t>Bonjour Martin,</t>
         </is>
       </c>
       <c r="N18" s="46" t="inlineStr">
         <is>
-          <t>Bonjour M. Perreault,
-On s'était parlé en juillet 2021. Merci de l'intérêt que vous nous aviez porté à l'époque : on partait de zéro.
+          <t>Bonjour M. Ménard,
+On s'était parlé à La Terre en janvier 2021. Cinq ans plus tard, on achète encore de l'asclépiade québécoise et on la transforme nous-mêmes à Québec. Merci d'avoir porté le sujet auprès des producteurs : c'est le lectorat qui compte le plus pour nous, sans champs il n'y a pas de fibre.
 On se concentre sur nos 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part : je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer une suite à votre dernier article.
 Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
@@ -2320,27 +2321,27 @@
     <row r="19" ht="240" customHeight="1" s="26">
       <c r="A19" s="36" t="inlineStr">
         <is>
-          <t>Fanny Samson</t>
+          <t>Anne-Sophie Roy</t>
         </is>
       </c>
       <c r="B19" s="36" t="inlineStr">
         <is>
-          <t>Radio-Canada</t>
+          <t>Québecor Média</t>
         </is>
       </c>
       <c r="C19" s="36" t="inlineStr">
         <is>
-          <t>fanny.samson@radio-canada.ca</t>
+          <t>anne-sophie.roy@quebecormedia.com</t>
         </is>
       </c>
       <c r="D19" s="36" t="inlineStr">
         <is>
-          <t>2021-03-13</t>
+          <t>2020-12-13</t>
         </is>
       </c>
       <c r="E19" s="37" t="inlineStr">
         <is>
-          <t>Reportage</t>
+          <t>Série d'articles</t>
         </is>
       </c>
       <c r="F19" s="36" t="inlineStr">
@@ -2363,67 +2364,51 @@
       </c>
       <c r="L19" s="25" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M19" s="25" t="inlineStr">
         <is>
-          <t>Bonjour Fanny,</t>
+          <t>Bonjour Anne-Sophie,</t>
         </is>
       </c>
       <c r="N19" s="46" t="inlineStr">
         <is>
-          <t>Bonjour Mme Samson,
-En mars 2021, vous aviez signé « Les grandes promesses de l'asclépiade, la soie d'Amérique ». Cinq ans plus tard, je peux vous dire lesquelles ont été tenues : il y a des produits finis, l'isolant se transforme toujours au Québec, on achète encore de l'asclépiade québécoise, et un manteau Lasclay se vend au prix très abordable de 300 $.
-On se concentre sur nos 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
-Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
-Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer une suite à votre dernier article.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
-J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
-Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
+          <t>NE PAS ENVOYER — même journaliste que la ligne Radio-Canada, à une ancienne adresse. Écrire à anne-sophie.roy@radio-canada.ca. Garder cette adresse en réserve si l'autre rebondit.</t>
         </is>
       </c>
       <c r="O19" s="25" t="inlineStr">
         <is>
-          <t>vous</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="20" ht="240" customHeight="1" s="26">
       <c r="A20" s="36" t="inlineStr">
         <is>
-          <t>Martin Ménard</t>
+          <t>G. Roy</t>
         </is>
       </c>
       <c r="B20" s="36" t="inlineStr">
         <is>
-          <t>La Terre de chez nous</t>
+          <t>Le Quotidien</t>
         </is>
       </c>
       <c r="C20" s="36" t="inlineStr">
         <is>
-          <t>mmenard@laterre.ca</t>
-        </is>
-      </c>
-      <c r="D20" s="36" t="inlineStr">
-        <is>
-          <t>2021-01-26</t>
-        </is>
-      </c>
-      <c r="E20" s="37" t="inlineStr">
-        <is>
-          <t>Entrevue La Terre</t>
-        </is>
-      </c>
+          <t>groy@lequotidien.com</t>
+        </is>
+      </c>
+      <c r="D20" s="36" t="n"/>
+      <c r="E20" s="37" t="n"/>
       <c r="F20" s="36" t="inlineStr">
         <is>
-          <t>Missive — boîte LAS Media</t>
-        </is>
-      </c>
-      <c r="G20" s="36" t="inlineStr">
-        <is>
-          <t>Correspondance confirmée</t>
+          <t>Fournie par Gabriel</t>
+        </is>
+      </c>
+      <c r="G20" s="40" t="inlineStr">
+        <is>
+          <t>Non recoupée dans Missive</t>
         </is>
       </c>
       <c r="H20" s="38" t="n"/>
@@ -2441,13 +2426,13 @@
       </c>
       <c r="M20" s="25" t="inlineStr">
         <is>
-          <t>Bonjour Martin,</t>
+          <t>Bonjour,</t>
         </is>
       </c>
       <c r="N20" s="46" t="inlineStr">
         <is>
-          <t>Bonjour M. Ménard,
-On s'était parlé à La Terre en janvier 2021. Cinq ans plus tard, on achète encore de l'asclépiade québécoise et on la transforme nous-mêmes à Québec. Merci d'avoir porté le sujet auprès des producteurs : c'est le lectorat qui compte le plus pour nous, sans champs il n'y a pas de fibre.
+          <t>Bonjour M. Roy,
+En octobre 2020, vous avez écrit « La deuxième vie de l'asclépiade ». Vous avez été le tout premier journaliste à parler de nous. Et l'agriculteur du Lac-Saint-Jean qui vous avait donné envie du sujet est encore notre fournisseur aujourd'hui : six ans plus tard, l'asclépiade de chez vous se retrouve toujours dans nos produits. Merci, sincèrement : on n'oublie pas qui a écrit le premier article, et le vôtre nous a servi de carte de visite pendant des années.
 On se concentre sur nos 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -2466,37 +2451,29 @@
     <row r="21" ht="240" customHeight="1" s="26">
       <c r="A21" s="36" t="inlineStr">
         <is>
-          <t>Anne-Sophie Roy</t>
+          <t>Sophie Laforest</t>
         </is>
       </c>
       <c r="B21" s="36" t="inlineStr">
         <is>
-          <t>Québecor Média</t>
+          <t>Radio-Canada</t>
         </is>
       </c>
       <c r="C21" s="36" t="inlineStr">
         <is>
-          <t>anne-sophie.roy@quebecormedia.com</t>
-        </is>
-      </c>
-      <c r="D21" s="36" t="inlineStr">
-        <is>
-          <t>2020-12-13</t>
-        </is>
-      </c>
-      <c r="E21" s="37" t="inlineStr">
-        <is>
-          <t>Série d'articles</t>
-        </is>
-      </c>
+          <t>sophie.laforest@radio-canada.ca</t>
+        </is>
+      </c>
+      <c r="D21" s="36" t="n"/>
+      <c r="E21" s="37" t="n"/>
       <c r="F21" s="36" t="inlineStr">
         <is>
-          <t>Missive — boîte LAS Media</t>
-        </is>
-      </c>
-      <c r="G21" s="36" t="inlineStr">
-        <is>
-          <t>Correspondance confirmée</t>
+          <t>Fournie par Gabriel</t>
+        </is>
+      </c>
+      <c r="G21" s="40" t="inlineStr">
+        <is>
+          <t>Non recoupée dans Missive</t>
         </is>
       </c>
       <c r="H21" s="38" t="n"/>
@@ -2509,56 +2486,75 @@
       </c>
       <c r="L21" s="25" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="M21" s="25" t="inlineStr">
         <is>
-          <t>Bonjour Anne-Sophie,</t>
+          <t>Bonjour Sophie,</t>
         </is>
       </c>
       <c r="N21" s="46" t="inlineStr">
         <is>
-          <t>NE PAS ENVOYER — même journaliste que la ligne Radio-Canada, à une ancienne adresse. Écrire à anne-sophie.roy@radio-canada.ca. Garder cette adresse en réserve si l'autre rebondit.</t>
+          <t>Bonjour Mme Laforest,
+Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe : l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé, le papillon monarque.
+Depuis 5 ans, on travaille fort à la faire connaître et le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
+Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
+Aller parler de cette fibre québécoise unique à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part : je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
+Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
+Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
       </c>
       <c r="O21" s="25" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>vous</t>
         </is>
       </c>
     </row>
     <row r="22" ht="240" customHeight="1" s="26">
       <c r="A22" s="36" t="inlineStr">
         <is>
-          <t>G. Roy</t>
+          <t>Alain McKenna</t>
         </is>
       </c>
       <c r="B22" s="36" t="inlineStr">
         <is>
-          <t>Le Quotidien</t>
+          <t>Le Devoir</t>
         </is>
       </c>
       <c r="C22" s="36" t="inlineStr">
         <is>
-          <t>groy@lequotidien.com</t>
-        </is>
-      </c>
-      <c r="D22" s="36" t="n"/>
-      <c r="E22" s="37" t="n"/>
+          <t>amckenna@ledevoir.com</t>
+        </is>
+      </c>
+      <c r="D22" s="36" t="inlineStr">
+        <is>
+          <t>2021-12-24</t>
+        </is>
+      </c>
+      <c r="E22" s="37" t="inlineStr">
+        <is>
+          <t>Des écouteurs de Québec pour oublier les AirPods (Sounds Good)</t>
+        </is>
+      </c>
       <c r="F22" s="36" t="inlineStr">
         <is>
-          <t>Fournie par Gabriel</t>
+          <t>Lien fourni par Gabriel</t>
         </is>
       </c>
       <c r="G22" s="40" t="inlineStr">
         <is>
-          <t>Non recoupée dans Missive</t>
+          <t>Correspondance confirmée</t>
         </is>
       </c>
       <c r="H22" s="38" t="n"/>
       <c r="I22" s="38" t="n"/>
-      <c r="J22" s="39" t="n"/>
+      <c r="J22" s="39" t="inlineStr">
+        <is>
+          <t>A couvert Sounds Good, la première entreprise de Gabriel, à l'époque des trois associés. Gabriel a vendu ses parts en 2022 : le dire d'entrée, McKenna suit encore Sounds Good.</t>
+        </is>
+      </c>
       <c r="K22" s="25" t="inlineStr">
         <is>
           <t>A</t>
@@ -2571,13 +2567,13 @@
       </c>
       <c r="M22" s="25" t="inlineStr">
         <is>
-          <t>Bonjour,</t>
+          <t>Bonjour Alain,</t>
         </is>
       </c>
       <c r="N22" s="46" t="inlineStr">
         <is>
-          <t>Bonjour M. Roy,
-En octobre 2020, vous avez écrit « La deuxième vie de l'asclépiade ». Vous avez été le tout premier journaliste à parler de nous. Et l'agriculteur du Lac-Saint-Jean qui vous avait donné envie du sujet est encore notre fournisseur aujourd'hui : six ans plus tard, l'asclépiade de chez vous se retrouve toujours dans nos produits. Merci, sincèrement : on n'oublie pas qui a écrit le premier article, et le vôtre nous a servi de carte de visite pendant des années.
+          <t>Bonjour M. McKenna,
+En décembre 2021, vous aviez écrit « Des écouteurs de Québec pour oublier les AirPods », sur Sounds Good. J'étais un des trois. J'ai vendu mes parts en 2022 pour me consacrer entièrement à Lasclay, l'autre entreprise que j'avais démarrée entretemps, qui transforme la soie d'asclépiade en isolant textile. Merci encore pour ce texte : il a compté pour Sounds Good.
 On se concentre sur nos 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -2596,17 +2592,17 @@
     <row r="23" ht="240" customHeight="1" s="26">
       <c r="A23" s="36" t="inlineStr">
         <is>
-          <t>Sophie Laforest</t>
+          <t>Sylvie Lemieux</t>
         </is>
       </c>
       <c r="B23" s="36" t="inlineStr">
         <is>
-          <t>Radio-Canada</t>
+          <t>Pigiste</t>
         </is>
       </c>
       <c r="C23" s="36" t="inlineStr">
         <is>
-          <t>sophie.laforest@radio-canada.ca</t>
+          <t>sylvielemieux16@gmail.com</t>
         </is>
       </c>
       <c r="D23" s="36" t="n"/>
@@ -2636,151 +2632,10 @@
       </c>
       <c r="M23" s="25" t="inlineStr">
         <is>
-          <t>Bonjour Sophie,</t>
+          <t>Bonjour Sylvie,</t>
         </is>
       </c>
       <c r="N23" s="46" t="inlineStr">
-        <is>
-          <t>Bonjour Mme Laforest,
-Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe : l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé, le papillon monarque.
-Depuis 5 ans, on travaille fort à la faire connaître et le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
-Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller parler de cette fibre québécoise unique à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part : je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
-J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
-Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
-        </is>
-      </c>
-      <c r="O23" s="25" t="inlineStr">
-        <is>
-          <t>vous</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="240" customHeight="1" s="26">
-      <c r="A24" s="36" t="inlineStr">
-        <is>
-          <t>Alain McKenna</t>
-        </is>
-      </c>
-      <c r="B24" s="36" t="inlineStr">
-        <is>
-          <t>Le Devoir</t>
-        </is>
-      </c>
-      <c r="C24" s="36" t="inlineStr">
-        <is>
-          <t>amckenna@ledevoir.com</t>
-        </is>
-      </c>
-      <c r="D24" s="36" t="inlineStr">
-        <is>
-          <t>2021-12-24</t>
-        </is>
-      </c>
-      <c r="E24" s="37" t="inlineStr">
-        <is>
-          <t>Des écouteurs de Québec pour oublier les AirPods (Sounds Good)</t>
-        </is>
-      </c>
-      <c r="F24" s="36" t="inlineStr">
-        <is>
-          <t>Lien fourni par Gabriel</t>
-        </is>
-      </c>
-      <c r="G24" s="40" t="inlineStr">
-        <is>
-          <t>Correspondance confirmée</t>
-        </is>
-      </c>
-      <c r="H24" s="38" t="n"/>
-      <c r="I24" s="38" t="n"/>
-      <c r="J24" s="39" t="inlineStr">
-        <is>
-          <t>A couvert Sounds Good, la première entreprise de Gabriel, à l'époque des trois associés. Gabriel a vendu ses parts en 2022 : le dire d'entrée, McKenna suit encore Sounds Good.</t>
-        </is>
-      </c>
-      <c r="K24" s="25" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="L24" s="25" t="inlineStr">
-        <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
-        </is>
-      </c>
-      <c r="M24" s="25" t="inlineStr">
-        <is>
-          <t>Bonjour Alain,</t>
-        </is>
-      </c>
-      <c r="N24" s="46" t="inlineStr">
-        <is>
-          <t>Bonjour M. McKenna,
-En décembre 2021, vous aviez écrit « Des écouteurs de Québec pour oublier les AirPods », sur Sounds Good. J'étais un des trois. J'ai vendu mes parts en 2022 pour me consacrer entièrement à Lasclay, l'autre entreprise que j'avais démarrée entretemps, qui transforme la soie d'asclépiade en isolant textile. Merci encore pour ce texte : il a compté pour Sounds Good.
-On se concentre sur nos 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
-Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
-Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer une suite à votre dernier article.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
-J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
-Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
-        </is>
-      </c>
-      <c r="O24" s="25" t="inlineStr">
-        <is>
-          <t>vous</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="240" customHeight="1" s="26">
-      <c r="A25" s="36" t="inlineStr">
-        <is>
-          <t>Sylvie Lemieux</t>
-        </is>
-      </c>
-      <c r="B25" s="36" t="inlineStr">
-        <is>
-          <t>Pigiste</t>
-        </is>
-      </c>
-      <c r="C25" s="36" t="inlineStr">
-        <is>
-          <t>sylvielemieux16@gmail.com</t>
-        </is>
-      </c>
-      <c r="D25" s="36" t="n"/>
-      <c r="E25" s="37" t="n"/>
-      <c r="F25" s="36" t="inlineStr">
-        <is>
-          <t>Fournie par Gabriel</t>
-        </is>
-      </c>
-      <c r="G25" s="40" t="inlineStr">
-        <is>
-          <t>Non recoupée dans Missive</t>
-        </is>
-      </c>
-      <c r="H25" s="38" t="n"/>
-      <c r="I25" s="38" t="n"/>
-      <c r="J25" s="39" t="n"/>
-      <c r="K25" s="25" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="L25" s="25" t="inlineStr">
-        <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
-        </is>
-      </c>
-      <c r="M25" s="25" t="inlineStr">
-        <is>
-          <t>Bonjour Sylvie,</t>
-        </is>
-      </c>
-      <c r="N25" s="46" t="inlineStr">
         <is>
           <t>Bonjour Mme Lemieux,
 En décembre 2021, vous aviez écrit « Les deux mains dans l'écoresponsabilité » pour le Journal de Montréal. Notre modèle manufacturier a changé depuis, et j'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
@@ -2792,59 +2647,59 @@
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
       </c>
-      <c r="O25" s="25" t="inlineStr">
+      <c r="O23" s="25" t="inlineStr">
         <is>
           <t>vous</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="240" customHeight="1" s="26">
-      <c r="A26" s="36" t="inlineStr">
+    <row r="24" ht="240" customHeight="1" s="26">
+      <c r="A24" s="36" t="inlineStr">
         <is>
           <t>Sophie Grenier-Héroux</t>
         </is>
       </c>
-      <c r="B26" s="36" t="inlineStr">
+      <c r="B24" s="36" t="inlineStr">
         <is>
           <t>Pigiste</t>
         </is>
       </c>
-      <c r="C26" s="36" t="inlineStr">
+      <c r="C24" s="36" t="inlineStr">
         <is>
           <t>sophiegrenierheroux@hotmail.com</t>
         </is>
       </c>
-      <c r="D26" s="36" t="n"/>
-      <c r="E26" s="37" t="n"/>
-      <c r="F26" s="36" t="inlineStr">
+      <c r="D24" s="36" t="n"/>
+      <c r="E24" s="37" t="n"/>
+      <c r="F24" s="36" t="inlineStr">
         <is>
           <t>Fournie par Gabriel</t>
         </is>
       </c>
-      <c r="G26" s="40" t="inlineStr">
+      <c r="G24" s="40" t="inlineStr">
         <is>
           <t>Non recoupée dans Missive</t>
         </is>
       </c>
-      <c r="H26" s="38" t="n"/>
-      <c r="I26" s="38" t="n"/>
-      <c r="J26" s="39" t="n"/>
-      <c r="K26" s="25" t="inlineStr">
+      <c r="H24" s="38" t="n"/>
+      <c r="I24" s="38" t="n"/>
+      <c r="J24" s="39" t="n"/>
+      <c r="K24" s="25" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="L26" s="25" t="inlineStr">
+      <c r="L24" s="25" t="inlineStr">
         <is>
           <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
-      <c r="M26" s="25" t="inlineStr">
+      <c r="M24" s="25" t="inlineStr">
         <is>
           <t>Bonjour Sophie,</t>
         </is>
       </c>
-      <c r="N26" s="46" t="inlineStr">
+      <c r="N24" s="46" t="inlineStr">
         <is>
           <t>Bonjour Mme Grenier-Héroux,
 En janvier 2021, vous aviez écrit « La soie d'Amérique, le pari de deux ambitieux » dans Le Devoir. Le pari a six ans, et il tient : plus de 40 produits, environ 10 millions de graines distribuées, et un isolant toujours transformé à Limoilou. Merci encore pour cet article.
@@ -2857,59 +2712,59 @@
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
       </c>
-      <c r="O26" s="25" t="inlineStr">
+      <c r="O24" s="25" t="inlineStr">
         <is>
           <t>vous</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="240" customHeight="1" s="26">
-      <c r="A27" s="36" t="inlineStr">
+    <row r="25" ht="240" customHeight="1" s="26">
+      <c r="A25" s="36" t="inlineStr">
         <is>
           <t>Madeleine Goubau</t>
         </is>
       </c>
-      <c r="B27" s="36" t="inlineStr">
+      <c r="B25" s="36" t="inlineStr">
         <is>
           <t>Pigiste</t>
         </is>
       </c>
-      <c r="C27" s="36" t="inlineStr">
+      <c r="C25" s="36" t="inlineStr">
         <is>
           <t>madeleine.goubau@gmail.com</t>
         </is>
       </c>
-      <c r="D27" s="36" t="n"/>
-      <c r="E27" s="37" t="n"/>
-      <c r="F27" s="36" t="inlineStr">
+      <c r="D25" s="36" t="n"/>
+      <c r="E25" s="37" t="n"/>
+      <c r="F25" s="36" t="inlineStr">
         <is>
           <t>Fournie par Gabriel</t>
         </is>
       </c>
-      <c r="G27" s="40" t="inlineStr">
+      <c r="G25" s="40" t="inlineStr">
         <is>
           <t>Non recoupée dans Missive</t>
         </is>
       </c>
-      <c r="H27" s="38" t="n"/>
-      <c r="I27" s="38" t="n"/>
-      <c r="J27" s="39" t="n"/>
-      <c r="K27" s="25" t="inlineStr">
+      <c r="H25" s="38" t="n"/>
+      <c r="I25" s="38" t="n"/>
+      <c r="J25" s="39" t="n"/>
+      <c r="K25" s="25" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="L27" s="25" t="inlineStr">
+      <c r="L25" s="25" t="inlineStr">
         <is>
           <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
-      <c r="M27" s="25" t="inlineStr">
+      <c r="M25" s="25" t="inlineStr">
         <is>
           <t>Bonjour Madeleine,</t>
         </is>
       </c>
-      <c r="N27" s="46" t="inlineStr">
+      <c r="N25" s="46" t="inlineStr">
         <is>
           <t>Bonjour Mme Goubau,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe : l'asclépiade, que vous connaissez bien je pense.
@@ -2921,67 +2776,67 @@
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
       </c>
-      <c r="O27" s="25" t="inlineStr">
+      <c r="O25" s="25" t="inlineStr">
         <is>
           <t>vous</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="240" customHeight="1" s="26">
-      <c r="A28" s="46" t="inlineStr">
+    <row r="26" ht="240" customHeight="1" s="26">
+      <c r="A26" s="46" t="inlineStr">
         <is>
           <t>Jean-Michel Leprince</t>
         </is>
       </c>
-      <c r="B28" s="46" t="inlineStr">
+      <c r="B26" s="46" t="inlineStr">
         <is>
           <t>Radio-Canada</t>
         </is>
       </c>
-      <c r="C28" s="46" t="inlineStr">
+      <c r="C26" s="46" t="inlineStr">
         <is>
           <t>jean-michel_leprince@radio-canada.ca</t>
         </is>
       </c>
-      <c r="D28" s="46" t="inlineStr">
+      <c r="D26" s="46" t="inlineStr">
         <is>
           <t>2014-2019</t>
         </is>
       </c>
-      <c r="E28" s="46" t="inlineStr">
+      <c r="E26" s="46" t="inlineStr">
         <is>
           <t>Reportages sur l'asclépiade au Téléjournal</t>
         </is>
       </c>
-      <c r="F28" s="46" t="inlineStr">
+      <c r="F26" s="46" t="inlineStr">
         <is>
           <t>Recherche web</t>
         </is>
       </c>
-      <c r="G28" s="46" t="inlineStr">
+      <c r="G26" s="46" t="inlineStr">
         <is>
           <t>Adresse à confirmer</t>
         </is>
       </c>
-      <c r="H28" s="46" t="n"/>
-      <c r="I28" s="46" t="n"/>
-      <c r="J28" s="46" t="inlineStr">
+      <c r="H26" s="46" t="n"/>
+      <c r="I26" s="46" t="n"/>
+      <c r="J26" s="46" t="inlineStr">
         <is>
           <t>A suivi l'asclépiade plus longtemps que quiconque au Québec, sans jamais couvrir Lasclay. Promu de la liste froide sur demande de Gabriel.</t>
         </is>
       </c>
-      <c r="K28" s="46" t="inlineStr">
+      <c r="K26" s="46" t="inlineStr">
         <is>
           <t>J</t>
         </is>
       </c>
-      <c r="L28" s="46" t="inlineStr">
+      <c r="L26" s="46" t="inlineStr">
         <is>
           <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
-      <c r="M28" s="46" t="n"/>
-      <c r="N28" s="46" t="inlineStr">
+      <c r="M26" s="46" t="n"/>
+      <c r="N26" s="46" t="inlineStr">
         <is>
           <t>Bonjour M. Leprince,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
@@ -2995,12 +2850,14 @@
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
       </c>
-      <c r="O28" s="46" t="inlineStr">
+      <c r="O26" s="46" t="inlineStr">
         <is>
           <t>vous</t>
         </is>
       </c>
     </row>
+    <row r="27" ht="240" customHeight="1" s="26"/>
+    <row r="28" ht="240" customHeight="1" s="26"/>
     <row r="29" ht="240" customHeight="1" s="26"/>
     <row r="30" ht="240" customHeight="1" s="26"/>
     <row r="31" ht="240" customHeight="1" s="26"/>

</xml_diff>

<commit_message>
Retire Ariane Aubert Bonn de la liste chaude
23 brouillons chauds, 241 contacts.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015pjLsGPzf1MX1JC7QiKGGk
</commit_message>
<xml_diff>
--- a/communique-dragons/Lasclay_v2.xlsx
+++ b/communique-dragons/Lasclay_v2.xlsx
@@ -990,7 +990,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O26"/>
+  <dimension ref="A1:O25"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="26" customWidth="1" style="25" min="1" max="1"/>
@@ -1812,27 +1812,27 @@
     <row r="12" ht="240" customHeight="1" s="26">
       <c r="A12" s="36" t="inlineStr">
         <is>
-          <t>Ariane Aubert Bonn</t>
+          <t>Eugénie Émond</t>
         </is>
       </c>
       <c r="B12" s="36" t="inlineStr">
         <is>
-          <t>La Tribune</t>
+          <t>Radio-Canada</t>
         </is>
       </c>
       <c r="C12" s="36" t="inlineStr">
         <is>
-          <t>aabonn@latribune.qc.ca</t>
+          <t>eugenie.emond@radio-canada.ca</t>
         </is>
       </c>
       <c r="D12" s="36" t="inlineStr">
         <is>
-          <t>2022-11-30</t>
+          <t>2022-09-01</t>
         </is>
       </c>
       <c r="E12" s="37" t="inlineStr">
         <is>
-          <t>Nouveaux produits d'asclépiade</t>
+          <t>Entrevue — glacière d'asclépiade imprimée 3D</t>
         </is>
       </c>
       <c r="F12" s="36" t="inlineStr">
@@ -1860,17 +1860,17 @@
       </c>
       <c r="M12" s="25" t="inlineStr">
         <is>
-          <t>Bonjour Ariane,</t>
+          <t>Bonjour Eugénie,</t>
         </is>
       </c>
       <c r="N12" s="46" t="inlineStr">
         <is>
-          <t>Bonjour Mme Aubert Bonn,
-En novembre 2022, vous aviez couvert nos nouveaux produits d'asclépiade. Le catalogue compte maintenant plus de 40 produits, et La Tribune a repris en décembre dernier l'article de Chloé Pouliot sur notre changement de modèle manufacturier. Merci encore : l'Estrie nous suit depuis, et ça part de là.
-Parmi les raisons de ce changement, il y avait clairement que j'avais besoin de temps pour me recentrer sur mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+          <t>Bonjour Mme Émond,
+En septembre 2022, on s'était parlé de notre glacière d'asclépiade imprimée en 3D. On a continué à inventer nos propres procédés depuis, parce que personne d'autre ne les fait. Merci encore pour ce reportage.
+On se concentre sur nos 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer une suite à votre dernier article.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet.
 Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
@@ -1885,27 +1885,27 @@
     <row r="13" ht="240" customHeight="1" s="26">
       <c r="A13" s="36" t="inlineStr">
         <is>
-          <t>Eugénie Émond</t>
+          <t>Marc Tison</t>
         </is>
       </c>
       <c r="B13" s="36" t="inlineStr">
         <is>
-          <t>Radio-Canada</t>
+          <t>La Presse</t>
         </is>
       </c>
       <c r="C13" s="36" t="inlineStr">
         <is>
-          <t>eugenie.emond@radio-canada.ca</t>
+          <t>mtison1@lapresse.ca</t>
         </is>
       </c>
       <c r="D13" s="36" t="inlineStr">
         <is>
-          <t>2022-09-01</t>
+          <t>2021-09-20</t>
         </is>
       </c>
       <c r="E13" s="37" t="inlineStr">
         <is>
-          <t>Entrevue — glacière d'asclépiade imprimée 3D</t>
+          <t>Entrevue — section Affaires</t>
         </is>
       </c>
       <c r="F13" s="36" t="inlineStr">
@@ -1933,17 +1933,17 @@
       </c>
       <c r="M13" s="25" t="inlineStr">
         <is>
-          <t>Bonjour Eugénie,</t>
+          <t>Bonjour Marc,</t>
         </is>
       </c>
       <c r="N13" s="46" t="inlineStr">
         <is>
-          <t>Bonjour Mme Émond,
-En septembre 2022, on s'était parlé de notre glacière d'asclépiade imprimée en 3D. On a continué à inventer nos propres procédés depuis, parce que personne d'autre ne les fait. Merci encore pour ce reportage.
-On se concentre sur nos 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+          <t>Bonjour M. Tison,
+On s'était parlé pour la section Affaires en septembre 2021, à l'époque où on venait de rapatrier notre production faute de sous-traitant prêt à toucher à la fibre. Le modèle a changé depuis : la vidéo est ici, https://www.youtube.com/watch?v=GKyHh-Ok9JU, et Sylvain Larocque en a parlé en mai. Merci encore : le texte a beaucoup circulé chez nos clients.
+Parmi les raisons de ce changement, il y avait clairement que j'avais besoin de temps pour me recentrer sur mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer un sujet.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer une suite à votre dernier article.
 Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
@@ -1958,7 +1958,7 @@
     <row r="14" ht="240" customHeight="1" s="26">
       <c r="A14" s="36" t="inlineStr">
         <is>
-          <t>Marc Tison</t>
+          <t>Valérie Simard</t>
         </is>
       </c>
       <c r="B14" s="36" t="inlineStr">
@@ -1968,17 +1968,17 @@
       </c>
       <c r="C14" s="36" t="inlineStr">
         <is>
-          <t>mtison1@lapresse.ca</t>
+          <t>vsimard@lapresse.ca</t>
         </is>
       </c>
       <c r="D14" s="36" t="inlineStr">
         <is>
-          <t>2021-09-20</t>
+          <t>2021-09-17</t>
         </is>
       </c>
       <c r="E14" s="37" t="inlineStr">
         <is>
-          <t>Entrevue — section Affaires</t>
+          <t>Demande média</t>
         </is>
       </c>
       <c r="F14" s="36" t="inlineStr">
@@ -2006,16 +2006,14 @@
       </c>
       <c r="M14" s="25" t="inlineStr">
         <is>
-          <t>Bonjour Marc,</t>
+          <t>Bonjour Valérie,</t>
         </is>
       </c>
       <c r="N14" s="46" t="inlineStr">
         <is>
-          <t>Bonjour M. Tison,
-On s'était parlé pour la section Affaires en septembre 2021, à l'époque où on venait de rapatrier notre production faute de sous-traitant prêt à toucher à la fibre. Le modèle a changé depuis : la vidéo est ici, https://www.youtube.com/watch?v=GKyHh-Ok9JU, et Sylvain Larocque en a parlé en mai. Merci encore : le texte a beaucoup circulé chez nos clients.
-Parmi les raisons de ce changement, il y avait clairement que j'avais besoin de temps pour me recentrer sur mes 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
-Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
-Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
+          <t>Bonjour Mme Simard,
+Vous aviez présenté nos mitaines isolées à l'asclépiade le 17 septembre 2021. Merci pour ce coup de pouce de la première heure.
+Nous avons fait beaucoup de chemin depuis et le 17 septembre prochain, on va faire un autre énorme pas dans la bonne direction : Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
 Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer une suite à votre dernier article.
 Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
@@ -2031,27 +2029,27 @@
     <row r="15" ht="240" customHeight="1" s="26">
       <c r="A15" s="36" t="inlineStr">
         <is>
-          <t>Valérie Simard</t>
+          <t>Alex Perreault</t>
         </is>
       </c>
       <c r="B15" s="36" t="inlineStr">
         <is>
-          <t>La Presse</t>
+          <t>Radio-Canada</t>
         </is>
       </c>
       <c r="C15" s="36" t="inlineStr">
         <is>
-          <t>vsimard@lapresse.ca</t>
+          <t>alex.perreault@radio-canada.ca</t>
         </is>
       </c>
       <c r="D15" s="36" t="inlineStr">
         <is>
-          <t>2021-09-17</t>
+          <t>2021-07-22</t>
         </is>
       </c>
       <c r="E15" s="37" t="inlineStr">
         <is>
-          <t>Demande média</t>
+          <t>Entrevue Radio-Canada</t>
         </is>
       </c>
       <c r="F15" s="36" t="inlineStr">
@@ -2079,15 +2077,17 @@
       </c>
       <c r="M15" s="25" t="inlineStr">
         <is>
-          <t>Bonjour Valérie,</t>
+          <t>Bonjour Alex,</t>
         </is>
       </c>
       <c r="N15" s="46" t="inlineStr">
         <is>
-          <t>Bonjour Mme Simard,
-Vous aviez présenté nos mitaines isolées à l'asclépiade le 17 septembre 2021. Merci pour ce coup de pouce de la première heure.
-Nous avons fait beaucoup de chemin depuis et le 17 septembre prochain, on va faire un autre énorme pas dans la bonne direction : Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer une suite à votre dernier article.
+          <t>Bonjour M. Perreault,
+On s'était parlé en juillet 2021. Merci de l'intérêt que vous nous aviez porté à l'époque : on partait de zéro.
+On se concentre sur nos 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
+Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part : je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
 Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
@@ -2102,7 +2102,7 @@
     <row r="16" ht="240" customHeight="1" s="26">
       <c r="A16" s="36" t="inlineStr">
         <is>
-          <t>Alex Perreault</t>
+          <t>Fanny Samson</t>
         </is>
       </c>
       <c r="B16" s="36" t="inlineStr">
@@ -2112,17 +2112,17 @@
       </c>
       <c r="C16" s="36" t="inlineStr">
         <is>
-          <t>alex.perreault@radio-canada.ca</t>
+          <t>fanny.samson@radio-canada.ca</t>
         </is>
       </c>
       <c r="D16" s="36" t="inlineStr">
         <is>
-          <t>2021-07-22</t>
+          <t>2021-03-13</t>
         </is>
       </c>
       <c r="E16" s="37" t="inlineStr">
         <is>
-          <t>Entrevue Radio-Canada</t>
+          <t>Reportage</t>
         </is>
       </c>
       <c r="F16" s="36" t="inlineStr">
@@ -2150,17 +2150,17 @@
       </c>
       <c r="M16" s="25" t="inlineStr">
         <is>
-          <t>Bonjour Alex,</t>
+          <t>Bonjour Fanny,</t>
         </is>
       </c>
       <c r="N16" s="46" t="inlineStr">
         <is>
-          <t>Bonjour M. Perreault,
-On s'était parlé en juillet 2021. Merci de l'intérêt que vous nous aviez porté à l'époque : on partait de zéro.
+          <t>Bonjour Mme Samson,
+En mars 2021, vous aviez signé « Les grandes promesses de l'asclépiade, la soie d'Amérique ». Cinq ans plus tard, je peux vous dire lesquelles ont été tenues : il y a des produits finis, l'isolant se transforme toujours au Québec, on achète encore de l'asclépiade québécoise, et un manteau Lasclay se vend au prix très abordable de 300 $.
 On se concentre sur nos 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part : je suis disponible pour une entrevue la semaine du 14 septembre et le vendredi 18 au matin.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer une suite à votre dernier article.
 Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
 J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
@@ -2175,27 +2175,27 @@
     <row r="17" ht="240" customHeight="1" s="26">
       <c r="A17" s="36" t="inlineStr">
         <is>
-          <t>Fanny Samson</t>
+          <t>Martin Ménard</t>
         </is>
       </c>
       <c r="B17" s="36" t="inlineStr">
         <is>
-          <t>Radio-Canada</t>
+          <t>La Terre de chez nous</t>
         </is>
       </c>
       <c r="C17" s="36" t="inlineStr">
         <is>
-          <t>fanny.samson@radio-canada.ca</t>
+          <t>mmenard@laterre.ca</t>
         </is>
       </c>
       <c r="D17" s="36" t="inlineStr">
         <is>
-          <t>2021-03-13</t>
+          <t>2021-01-26</t>
         </is>
       </c>
       <c r="E17" s="37" t="inlineStr">
         <is>
-          <t>Reportage</t>
+          <t>Entrevue La Terre</t>
         </is>
       </c>
       <c r="F17" s="36" t="inlineStr">
@@ -2223,13 +2223,13 @@
       </c>
       <c r="M17" s="25" t="inlineStr">
         <is>
-          <t>Bonjour Fanny,</t>
+          <t>Bonjour Martin,</t>
         </is>
       </c>
       <c r="N17" s="46" t="inlineStr">
         <is>
-          <t>Bonjour Mme Samson,
-En mars 2021, vous aviez signé « Les grandes promesses de l'asclépiade, la soie d'Amérique ». Cinq ans plus tard, je peux vous dire lesquelles ont été tenues : il y a des produits finis, l'isolant se transforme toujours au Québec, on achète encore de l'asclépiade québécoise, et un manteau Lasclay se vend au prix très abordable de 300 $.
+          <t>Bonjour M. Ménard,
+On s'était parlé à La Terre en janvier 2021. Cinq ans plus tard, on achète encore de l'asclépiade québécoise et on la transforme nous-mêmes à Québec. Merci d'avoir porté le sujet auprès des producteurs : c'est le lectorat qui compte le plus pour nous, sans champs il n'y a pas de fibre.
 On se concentre sur nos 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
 Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
 Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
@@ -2248,27 +2248,27 @@
     <row r="18" ht="240" customHeight="1" s="26">
       <c r="A18" s="36" t="inlineStr">
         <is>
-          <t>Martin Ménard</t>
+          <t>Anne-Sophie Roy</t>
         </is>
       </c>
       <c r="B18" s="36" t="inlineStr">
         <is>
-          <t>La Terre de chez nous</t>
+          <t>Québecor Média</t>
         </is>
       </c>
       <c r="C18" s="36" t="inlineStr">
         <is>
-          <t>mmenard@laterre.ca</t>
+          <t>anne-sophie.roy@quebecormedia.com</t>
         </is>
       </c>
       <c r="D18" s="36" t="inlineStr">
         <is>
-          <t>2021-01-26</t>
+          <t>2020-12-13</t>
         </is>
       </c>
       <c r="E18" s="37" t="inlineStr">
         <is>
-          <t>Entrevue La Terre</t>
+          <t>Série d'articles</t>
         </is>
       </c>
       <c r="F18" s="36" t="inlineStr">
@@ -2291,67 +2291,51 @@
       </c>
       <c r="L18" s="25" t="inlineStr">
         <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M18" s="25" t="inlineStr">
         <is>
-          <t>Bonjour Martin,</t>
+          <t>Bonjour Anne-Sophie,</t>
         </is>
       </c>
       <c r="N18" s="46" t="inlineStr">
         <is>
-          <t>Bonjour M. Ménard,
-On s'était parlé à La Terre en janvier 2021. Cinq ans plus tard, on achète encore de l'asclépiade québécoise et on la transforme nous-mêmes à Québec. Merci d'avoir porté le sujet auprès des producteurs : c'est le lectorat qui compte le plus pour nous, sans champs il n'y a pas de fibre.
-On se concentre sur nos 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
-Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
-Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer une suite à votre dernier article.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
-J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
-Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
+          <t>NE PAS ENVOYER — même journaliste que la ligne Radio-Canada, à une ancienne adresse. Écrire à anne-sophie.roy@radio-canada.ca. Garder cette adresse en réserve si l'autre rebondit.</t>
         </is>
       </c>
       <c r="O18" s="25" t="inlineStr">
         <is>
-          <t>vous</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="19" ht="240" customHeight="1" s="26">
       <c r="A19" s="36" t="inlineStr">
         <is>
-          <t>Anne-Sophie Roy</t>
+          <t>G. Roy</t>
         </is>
       </c>
       <c r="B19" s="36" t="inlineStr">
         <is>
-          <t>Québecor Média</t>
+          <t>Le Quotidien</t>
         </is>
       </c>
       <c r="C19" s="36" t="inlineStr">
         <is>
-          <t>anne-sophie.roy@quebecormedia.com</t>
-        </is>
-      </c>
-      <c r="D19" s="36" t="inlineStr">
-        <is>
-          <t>2020-12-13</t>
-        </is>
-      </c>
-      <c r="E19" s="37" t="inlineStr">
-        <is>
-          <t>Série d'articles</t>
-        </is>
-      </c>
+          <t>groy@lequotidien.com</t>
+        </is>
+      </c>
+      <c r="D19" s="36" t="n"/>
+      <c r="E19" s="37" t="n"/>
       <c r="F19" s="36" t="inlineStr">
         <is>
-          <t>Missive — boîte LAS Media</t>
-        </is>
-      </c>
-      <c r="G19" s="36" t="inlineStr">
-        <is>
-          <t>Correspondance confirmée</t>
+          <t>Fournie par Gabriel</t>
+        </is>
+      </c>
+      <c r="G19" s="40" t="inlineStr">
+        <is>
+          <t>Non recoupée dans Missive</t>
         </is>
       </c>
       <c r="H19" s="38" t="n"/>
@@ -2364,39 +2348,47 @@
       </c>
       <c r="L19" s="25" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
       <c r="M19" s="25" t="inlineStr">
         <is>
-          <t>Bonjour Anne-Sophie,</t>
+          <t>Bonjour,</t>
         </is>
       </c>
       <c r="N19" s="46" t="inlineStr">
         <is>
-          <t>NE PAS ENVOYER — même journaliste que la ligne Radio-Canada, à une ancienne adresse. Écrire à anne-sophie.roy@radio-canada.ca. Garder cette adresse en réserve si l'autre rebondit.</t>
+          <t>Bonjour M. Roy,
+En octobre 2020, vous avez écrit « La deuxième vie de l'asclépiade ». Vous avez été le tout premier journaliste à parler de nous. Et l'agriculteur du Lac-Saint-Jean qui vous avait donné envie du sujet est encore notre fournisseur aujourd'hui : six ans plus tard, l'asclépiade de chez vous se retrouve toujours dans nos produits. Merci, sincèrement : on n'oublie pas qui a écrit le premier article, et le vôtre nous a servi de carte de visite pendant des années.
+On se concentre sur nos 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
+Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer une suite à votre dernier article.
+Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
+Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
       </c>
       <c r="O19" s="25" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>vous</t>
         </is>
       </c>
     </row>
     <row r="20" ht="240" customHeight="1" s="26">
       <c r="A20" s="36" t="inlineStr">
         <is>
-          <t>G. Roy</t>
+          <t>Sophie Laforest</t>
         </is>
       </c>
       <c r="B20" s="36" t="inlineStr">
         <is>
-          <t>Le Quotidien</t>
+          <t>Radio-Canada</t>
         </is>
       </c>
       <c r="C20" s="36" t="inlineStr">
         <is>
-          <t>groy@lequotidien.com</t>
+          <t>sophie.laforest@radio-canada.ca</t>
         </is>
       </c>
       <c r="D20" s="36" t="n"/>
@@ -2426,75 +2418,10 @@
       </c>
       <c r="M20" s="25" t="inlineStr">
         <is>
-          <t>Bonjour,</t>
+          <t>Bonjour Sophie,</t>
         </is>
       </c>
       <c r="N20" s="46" t="inlineStr">
-        <is>
-          <t>Bonjour M. Roy,
-En octobre 2020, vous avez écrit « La deuxième vie de l'asclépiade ». Vous avez été le tout premier journaliste à parler de nous. Et l'agriculteur du Lac-Saint-Jean qui vous avait donné envie du sujet est encore notre fournisseur aujourd'hui : six ans plus tard, l'asclépiade de chez vous se retrouve toujours dans nos produits. Merci, sincèrement : on n'oublie pas qui a écrit le premier article, et le vôtre nous a servi de carte de visite pendant des années.
-On se concentre sur nos 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
-Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
-Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer une suite à votre dernier article.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
-J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
-Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
-        </is>
-      </c>
-      <c r="O20" s="25" t="inlineStr">
-        <is>
-          <t>vous</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="240" customHeight="1" s="26">
-      <c r="A21" s="36" t="inlineStr">
-        <is>
-          <t>Sophie Laforest</t>
-        </is>
-      </c>
-      <c r="B21" s="36" t="inlineStr">
-        <is>
-          <t>Radio-Canada</t>
-        </is>
-      </c>
-      <c r="C21" s="36" t="inlineStr">
-        <is>
-          <t>sophie.laforest@radio-canada.ca</t>
-        </is>
-      </c>
-      <c r="D21" s="36" t="n"/>
-      <c r="E21" s="37" t="n"/>
-      <c r="F21" s="36" t="inlineStr">
-        <is>
-          <t>Fournie par Gabriel</t>
-        </is>
-      </c>
-      <c r="G21" s="40" t="inlineStr">
-        <is>
-          <t>Non recoupée dans Missive</t>
-        </is>
-      </c>
-      <c r="H21" s="38" t="n"/>
-      <c r="I21" s="38" t="n"/>
-      <c r="J21" s="39" t="n"/>
-      <c r="K21" s="25" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="L21" s="25" t="inlineStr">
-        <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
-        </is>
-      </c>
-      <c r="M21" s="25" t="inlineStr">
-        <is>
-          <t>Bonjour Sophie,</t>
-        </is>
-      </c>
-      <c r="N21" s="46" t="inlineStr">
         <is>
           <t>Bonjour Mme Laforest,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe : l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé, le papillon monarque.
@@ -2506,71 +2433,71 @@
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
       </c>
-      <c r="O21" s="25" t="inlineStr">
+      <c r="O20" s="25" t="inlineStr">
         <is>
           <t>vous</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="240" customHeight="1" s="26">
-      <c r="A22" s="36" t="inlineStr">
+    <row r="21" ht="240" customHeight="1" s="26">
+      <c r="A21" s="36" t="inlineStr">
         <is>
           <t>Alain McKenna</t>
         </is>
       </c>
-      <c r="B22" s="36" t="inlineStr">
+      <c r="B21" s="36" t="inlineStr">
         <is>
           <t>Le Devoir</t>
         </is>
       </c>
-      <c r="C22" s="36" t="inlineStr">
+      <c r="C21" s="36" t="inlineStr">
         <is>
           <t>amckenna@ledevoir.com</t>
         </is>
       </c>
-      <c r="D22" s="36" t="inlineStr">
+      <c r="D21" s="36" t="inlineStr">
         <is>
           <t>2021-12-24</t>
         </is>
       </c>
-      <c r="E22" s="37" t="inlineStr">
+      <c r="E21" s="37" t="inlineStr">
         <is>
           <t>Des écouteurs de Québec pour oublier les AirPods (Sounds Good)</t>
         </is>
       </c>
-      <c r="F22" s="36" t="inlineStr">
+      <c r="F21" s="36" t="inlineStr">
         <is>
           <t>Lien fourni par Gabriel</t>
         </is>
       </c>
-      <c r="G22" s="40" t="inlineStr">
+      <c r="G21" s="40" t="inlineStr">
         <is>
           <t>Correspondance confirmée</t>
         </is>
       </c>
-      <c r="H22" s="38" t="n"/>
-      <c r="I22" s="38" t="n"/>
-      <c r="J22" s="39" t="inlineStr">
+      <c r="H21" s="38" t="n"/>
+      <c r="I21" s="38" t="n"/>
+      <c r="J21" s="39" t="inlineStr">
         <is>
           <t>A couvert Sounds Good, la première entreprise de Gabriel, à l'époque des trois associés. Gabriel a vendu ses parts en 2022 : le dire d'entrée, McKenna suit encore Sounds Good.</t>
         </is>
       </c>
-      <c r="K22" s="25" t="inlineStr">
+      <c r="K21" s="25" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="L22" s="25" t="inlineStr">
+      <c r="L21" s="25" t="inlineStr">
         <is>
           <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
-      <c r="M22" s="25" t="inlineStr">
+      <c r="M21" s="25" t="inlineStr">
         <is>
           <t>Bonjour Alain,</t>
         </is>
       </c>
-      <c r="N22" s="46" t="inlineStr">
+      <c r="N21" s="46" t="inlineStr">
         <is>
           <t>Bonjour M. McKenna,
 En décembre 2021, vous aviez écrit « Des écouteurs de Québec pour oublier les AirPods », sur Sounds Good. J'étais un des trois. J'ai vendu mes parts en 2022 pour me consacrer entièrement à Lasclay, l'autre entreprise que j'avais démarrée entretemps, qui transforme la soie d'asclépiade en isolant textile. Merci encore pour ce texte : il a compté pour Sounds Good.
@@ -2583,59 +2510,59 @@
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
       </c>
-      <c r="O22" s="25" t="inlineStr">
+      <c r="O21" s="25" t="inlineStr">
         <is>
           <t>vous</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="240" customHeight="1" s="26">
-      <c r="A23" s="36" t="inlineStr">
+    <row r="22" ht="240" customHeight="1" s="26">
+      <c r="A22" s="36" t="inlineStr">
         <is>
           <t>Sylvie Lemieux</t>
         </is>
       </c>
-      <c r="B23" s="36" t="inlineStr">
+      <c r="B22" s="36" t="inlineStr">
         <is>
           <t>Pigiste</t>
         </is>
       </c>
-      <c r="C23" s="36" t="inlineStr">
+      <c r="C22" s="36" t="inlineStr">
         <is>
           <t>sylvielemieux16@gmail.com</t>
         </is>
       </c>
-      <c r="D23" s="36" t="n"/>
-      <c r="E23" s="37" t="n"/>
-      <c r="F23" s="36" t="inlineStr">
+      <c r="D22" s="36" t="n"/>
+      <c r="E22" s="37" t="n"/>
+      <c r="F22" s="36" t="inlineStr">
         <is>
           <t>Fournie par Gabriel</t>
         </is>
       </c>
-      <c r="G23" s="40" t="inlineStr">
+      <c r="G22" s="40" t="inlineStr">
         <is>
           <t>Non recoupée dans Missive</t>
         </is>
       </c>
-      <c r="H23" s="38" t="n"/>
-      <c r="I23" s="38" t="n"/>
-      <c r="J23" s="39" t="n"/>
-      <c r="K23" s="25" t="inlineStr">
+      <c r="H22" s="38" t="n"/>
+      <c r="I22" s="38" t="n"/>
+      <c r="J22" s="39" t="n"/>
+      <c r="K22" s="25" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="L23" s="25" t="inlineStr">
+      <c r="L22" s="25" t="inlineStr">
         <is>
           <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
-      <c r="M23" s="25" t="inlineStr">
+      <c r="M22" s="25" t="inlineStr">
         <is>
           <t>Bonjour Sylvie,</t>
         </is>
       </c>
-      <c r="N23" s="46" t="inlineStr">
+      <c r="N22" s="46" t="inlineStr">
         <is>
           <t>Bonjour Mme Lemieux,
 En décembre 2021, vous aviez écrit « Les deux mains dans l'écoresponsabilité » pour le Journal de Montréal. Notre modèle manufacturier a changé depuis, et j'en ai fait une vidéo ici : https://www.youtube.com/watch?v=GKyHh-Ok9JU.
@@ -2647,6 +2574,71 @@
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
       </c>
+      <c r="O22" s="25" t="inlineStr">
+        <is>
+          <t>vous</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="240" customHeight="1" s="26">
+      <c r="A23" s="36" t="inlineStr">
+        <is>
+          <t>Sophie Grenier-Héroux</t>
+        </is>
+      </c>
+      <c r="B23" s="36" t="inlineStr">
+        <is>
+          <t>Pigiste</t>
+        </is>
+      </c>
+      <c r="C23" s="36" t="inlineStr">
+        <is>
+          <t>sophiegrenierheroux@hotmail.com</t>
+        </is>
+      </c>
+      <c r="D23" s="36" t="n"/>
+      <c r="E23" s="37" t="n"/>
+      <c r="F23" s="36" t="inlineStr">
+        <is>
+          <t>Fournie par Gabriel</t>
+        </is>
+      </c>
+      <c r="G23" s="40" t="inlineStr">
+        <is>
+          <t>Non recoupée dans Missive</t>
+        </is>
+      </c>
+      <c r="H23" s="38" t="n"/>
+      <c r="I23" s="38" t="n"/>
+      <c r="J23" s="39" t="n"/>
+      <c r="K23" s="25" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="L23" s="25" t="inlineStr">
+        <is>
+          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
+        </is>
+      </c>
+      <c r="M23" s="25" t="inlineStr">
+        <is>
+          <t>Bonjour Sophie,</t>
+        </is>
+      </c>
+      <c r="N23" s="46" t="inlineStr">
+        <is>
+          <t>Bonjour Mme Grenier-Héroux,
+En janvier 2021, vous aviez écrit « La soie d'Amérique, le pari de deux ambitieux » dans Le Devoir. Le pari a six ans, et il tient : plus de 40 produits, environ 10 millions de graines distribuées, et un isolant toujours transformé à Limoilou. Merci encore pour cet article.
+On se concentre sur nos 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
+Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
+Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
+Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer une suite à votre dernier article.
+Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
+J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
+Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
+        </is>
+      </c>
       <c r="O23" s="25" t="inlineStr">
         <is>
           <t>vous</t>
@@ -2656,7 +2648,7 @@
     <row r="24" ht="240" customHeight="1" s="26">
       <c r="A24" s="36" t="inlineStr">
         <is>
-          <t>Sophie Grenier-Héroux</t>
+          <t>Madeleine Goubau</t>
         </is>
       </c>
       <c r="B24" s="36" t="inlineStr">
@@ -2666,7 +2658,7 @@
       </c>
       <c r="C24" s="36" t="inlineStr">
         <is>
-          <t>sophiegrenierheroux@hotmail.com</t>
+          <t>madeleine.goubau@gmail.com</t>
         </is>
       </c>
       <c r="D24" s="36" t="n"/>
@@ -2696,75 +2688,10 @@
       </c>
       <c r="M24" s="25" t="inlineStr">
         <is>
-          <t>Bonjour Sophie,</t>
+          <t>Bonjour Madeleine,</t>
         </is>
       </c>
       <c r="N24" s="46" t="inlineStr">
-        <is>
-          <t>Bonjour Mme Grenier-Héroux,
-En janvier 2021, vous aviez écrit « La soie d'Amérique, le pari de deux ambitieux » dans Le Devoir. Le pari a six ans, et il tient : plus de 40 produits, environ 10 millions de graines distribuées, et un isolant toujours transformé à Limoilou. Merci encore pour cet article.
-On se concentre sur nos 2 grandes missions : faire connaître l'asclépiade et sauvegarder les monarques par la culture de l'asclépiade.
-Eh bien, le 17 septembre prochain, on va faire un énorme pas dans la bonne direction :
-Je vais présenter Lasclay dans le premier épisode de la 21e saison de Dragons' Den, sur CBC et CBC Gem.
-Aller présenter notre entreprise et sa mission à la télévision nationale est une opportunité qui arrive bien rarement. Je voulais vous en faire part et qui sait, peut-être vous inspirer une suite à votre dernier article.
-Si ça vous intéresse de couvrir (ou un.e collègue?), notre média kit est ici, avec les images de notre passage à Dragons' Den et de l'entreprise : https://drive.google.com/drive/folders/1pyCUbfHYQhpXXl4FoCC2RCFXKRvGS5Zr
-J'espère vraiment un boom des ventes avec cette visibilité, ce qui, plus largement, sera extrêmement bénéfique pour les cultivateurs d'asclépiade du Québec chez qui on continue d'acheter, et pour les papillons monarques menacés qui continuent de se reproduire dans leurs plantations.
-Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
-        </is>
-      </c>
-      <c r="O24" s="25" t="inlineStr">
-        <is>
-          <t>vous</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="240" customHeight="1" s="26">
-      <c r="A25" s="36" t="inlineStr">
-        <is>
-          <t>Madeleine Goubau</t>
-        </is>
-      </c>
-      <c r="B25" s="36" t="inlineStr">
-        <is>
-          <t>Pigiste</t>
-        </is>
-      </c>
-      <c r="C25" s="36" t="inlineStr">
-        <is>
-          <t>madeleine.goubau@gmail.com</t>
-        </is>
-      </c>
-      <c r="D25" s="36" t="n"/>
-      <c r="E25" s="37" t="n"/>
-      <c r="F25" s="36" t="inlineStr">
-        <is>
-          <t>Fournie par Gabriel</t>
-        </is>
-      </c>
-      <c r="G25" s="40" t="inlineStr">
-        <is>
-          <t>Non recoupée dans Missive</t>
-        </is>
-      </c>
-      <c r="H25" s="38" t="n"/>
-      <c r="I25" s="38" t="n"/>
-      <c r="J25" s="39" t="n"/>
-      <c r="K25" s="25" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="L25" s="25" t="inlineStr">
-        <is>
-          <t>Nous serons diffusés à Dragons' Den le 17 septembre!</t>
-        </is>
-      </c>
-      <c r="M25" s="25" t="inlineStr">
-        <is>
-          <t>Bonjour Madeleine,</t>
-        </is>
-      </c>
-      <c r="N25" s="46" t="inlineStr">
         <is>
           <t>Bonjour Mme Goubau,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe : l'asclépiade, que vous connaissez bien je pense.
@@ -2776,67 +2703,67 @@
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
       </c>
-      <c r="O25" s="25" t="inlineStr">
+      <c r="O24" s="25" t="inlineStr">
         <is>
           <t>vous</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="240" customHeight="1" s="26">
-      <c r="A26" s="46" t="inlineStr">
+    <row r="25" ht="240" customHeight="1" s="26">
+      <c r="A25" s="46" t="inlineStr">
         <is>
           <t>Jean-Michel Leprince</t>
         </is>
       </c>
-      <c r="B26" s="46" t="inlineStr">
+      <c r="B25" s="46" t="inlineStr">
         <is>
           <t>Radio-Canada</t>
         </is>
       </c>
-      <c r="C26" s="46" t="inlineStr">
+      <c r="C25" s="46" t="inlineStr">
         <is>
           <t>jean-michel_leprince@radio-canada.ca</t>
         </is>
       </c>
-      <c r="D26" s="46" t="inlineStr">
+      <c r="D25" s="46" t="inlineStr">
         <is>
           <t>2014-2019</t>
         </is>
       </c>
-      <c r="E26" s="46" t="inlineStr">
+      <c r="E25" s="46" t="inlineStr">
         <is>
           <t>Reportages sur l'asclépiade au Téléjournal</t>
         </is>
       </c>
-      <c r="F26" s="46" t="inlineStr">
+      <c r="F25" s="46" t="inlineStr">
         <is>
           <t>Recherche web</t>
         </is>
       </c>
-      <c r="G26" s="46" t="inlineStr">
+      <c r="G25" s="46" t="inlineStr">
         <is>
           <t>Adresse à confirmer</t>
         </is>
       </c>
-      <c r="H26" s="46" t="n"/>
-      <c r="I26" s="46" t="n"/>
-      <c r="J26" s="46" t="inlineStr">
+      <c r="H25" s="46" t="n"/>
+      <c r="I25" s="46" t="n"/>
+      <c r="J25" s="46" t="inlineStr">
         <is>
           <t>A suivi l'asclépiade plus longtemps que quiconque au Québec, sans jamais couvrir Lasclay. Promu de la liste froide sur demande de Gabriel.</t>
         </is>
       </c>
-      <c r="K26" s="46" t="inlineStr">
+      <c r="K25" s="46" t="inlineStr">
         <is>
           <t>J</t>
         </is>
       </c>
-      <c r="L26" s="46" t="inlineStr">
+      <c r="L25" s="46" t="inlineStr">
         <is>
           <t>L'asclépiade s'en va à Dragons' Den le 17 septembre!</t>
         </is>
       </c>
-      <c r="M26" s="46" t="n"/>
-      <c r="N26" s="46" t="inlineStr">
+      <c r="M25" s="46" t="n"/>
+      <c r="N25" s="46" t="inlineStr">
         <is>
           <t>Bonjour M. Leprince,
 Je m'appelle Gabriel Gouveia, fondateur de Lasclay. On isole des vêtements d'hiver avec une mauvaise herbe, l'asclépiade, qu'on cultive pour sauvegarder un pollinisateur emblématique et menacé : le papillon monarque.
@@ -2850,12 +2777,13 @@
 Au plaisir et n'hésitez pas à me contacter si vous avez des questions.</t>
         </is>
       </c>
-      <c r="O26" s="46" t="inlineStr">
+      <c r="O25" s="46" t="inlineStr">
         <is>
           <t>vous</t>
         </is>
       </c>
     </row>
+    <row r="26" ht="240" customHeight="1" s="26"/>
     <row r="27" ht="240" customHeight="1" s="26"/>
     <row r="28" ht="240" customHeight="1" s="26"/>
     <row r="29" ht="240" customHeight="1" s="26"/>

</xml_diff>